<commit_message>
Bumper should-cost workbook: Methodology & Q&A sheet
New sheet after Summary: the 8-step calculation method (make/buy split,
material, process, labour, tooling amortisation, overhead & margin,
assembly, roll-up) each with a plain-language explanation and a LIVE
worked example pulled by formula from the fascia row; plus 15 likely
manager questions with prepared answers and live reference values
(mechanical-only subtotal, tooling investment, painted-fascia price).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142L4rKS2AV8rxQTDWMs7dy
</commit_message>
<xml_diff>
--- a/Altroz-Front-Bumper-Should-Cost-India.xlsx
+++ b/Altroz-Front-Bumper-Should-Cost-India.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parts Costing" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bought-Out" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assembly &amp; Packing" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tooling" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology &amp; Q&amp;A" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parts Costing" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bought-Out" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assembly &amp; Packing" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tooling" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +31,7 @@
     <numFmt numFmtId="169" formatCode="0.00 &quot;Cr&quot;"/>
     <numFmt numFmtId="170" formatCode="#,##0 &quot;veh/yr&quot;"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -129,8 +130,37 @@
       <color rgb="0064748B"/>
       <sz val="10.5"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="004F46E5"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0064748B"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00059669"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -155,6 +185,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECFDF5"/>
       </patternFill>
     </fill>
   </fills>
@@ -184,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -221,6 +256,50 @@
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -317,7 +396,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1065,6 +1143,598 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>How this should-cost was calculated — step by step</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Read top to bottom. The right-hand column shows LIVE numbers pulled by formula from the costing sheets (worked example: front bumper fascia).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>THE 8-STEP METHOD  (worked example on the right: Front Bumper Fascia — values are LIVE, they change if you edit inputs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>Break the assembly into parts and decide make vs buy</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>The 26-line part list from the drawing was split into: 18 MANUFACTURED items (we cost these bottom-up on the Parts Costing sheet) and 7 BOUGHT-OUT items (electronics &amp; standard hardware — no one should-costs a radar chip bottom-up; we use market reference prices + 3% handling on the Bought-Out sheet).</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>Manufactured line items</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="62" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>Material cost per part</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>Net part mass × (1 + scrap%) × material price ₹/kg, minus scrap credit for the recoverable portion.  Formula in words: you buy slightly more plastic/steel than ends up in the part (runners, offal), and sell back what you can.  Excel: =Mass×(1+Scrap)×Price − Mass×Scrap×Credit  →  Fascia: 4.20 kg TPO at ₹142/kg with 4% runner scrap.</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>Fascia material ₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="D6" s="25">
+        <f>'Parts Costing'!J4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="62" customHeight="1">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Process (machine) cost</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>Cycle time ÷ 3600 × machine hour rate ÷ cavities.  The machine rate (Assumptions sheet) is a full build-up: depreciation + energy @ ₹8.5/kWh + maintenance + floor space + supervision.  A 1500-tonne press at ₹2,100/hr running a 58 s cycle costs ₹33.83 of machine time per shot — big-ticket machines, small per-part cost, because the hour is shared across every part made in it.</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>Fascia process ₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="D8" s="25">
+        <f>'Parts Costing'!O4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>Direct labour</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>Cycle time × manning × labour rate ÷ 3600 ÷ cavities.  Manning below 1.0 means one operator tends several machines (standard moulding practice — 0.5 = one operator per two presses).  Labour rates are FULLY LOADED: wages + statutory contributions + benefits + supervision share.</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>Fascia labour ₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="D10" s="25">
+        <f>'Parts Costing'!R4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="55" customHeight="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>Tooling amortisation</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Tool cost ÷ (annual volume × amortisation years × parts per vehicle).  The ₹2.2 Cr fascia mould spread over 72,000 vehicles × 5 years = a per-part charge.  This is the number most sensitive to VOLUME — halve the volume and this line doubles.  If the OEM pays for tooling separately, set column S to zero on Parts Costing.</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>Fascia tooling ₹/pc</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="D12" s="25">
+        <f>'Parts Costing'!T4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="55" customHeight="1">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>Overheads and margin</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Factory overhead (40%) is applied on CONVERSION cost only (process + labour), never on material — a supplier does not "manage" resin price, so it earns no overhead on it.  Then SG&amp;A 8% on manufacturing cost, and 10% profit on top of that.  The result is the ex-works unit price we should expect a competitive tier-1 to quote.</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>Fascia unit price ₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="D14" s="25">
+        <f>'Parts Costing'!Y4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>Assembly &amp; packing</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>Six stations, each = manned seconds × operators × labour rate.  Add fixture and end-of-line equipment amortisation, 45% assembly overhead on the labour, consumables, and the returnable-dunnage trip cost.  Bumper assembly is clip-and-screw work — it is deliberately cheap (~1% of total).</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>Assembly &amp; packing ₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="D16" s="25">
+        <f>'Assembly &amp; Packing'!$F$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="55" customHeight="1">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>Roll up the total</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>Total = Σ(manufactured unit price × qty) + Σ(bought-out landed × qty) + assembly &amp; packing.  The Summary sheet also shows the MECHANICAL-ONLY subtotal (excluding radar/camera/sensors/harness) because that is the number to compare against a bumper supplier's quote — the electronics are usually priced separately.</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL should cost ₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="D18" s="25">
+        <f>Summary!D8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>MANAGER Q&amp;A — the questions you will get, and the answers (live numbers in the right column)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="66" customHeight="1">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>“Why should I trust these numbers?”</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t>Because nothing is a black box. Every figure is built bottom-up from physics and visible inputs: mass × material price, cycle × machine rate, tool ÷ volume. Every input sits in a yellow cell you can challenge and change — and the whole workbook recalculates. A supplier quote can be compared against this line by line.</t>
+        </is>
+      </c>
+      <c r="D21" s="29" t="n"/>
+    </row>
+    <row r="22" ht="66" customHeight="1">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B22" s="31" t="inlineStr">
+        <is>
+          <t>“Where do the rates come from?”</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="inlineStr">
+        <is>
+          <t>India tier-1 benchmarks, July 2026: delivered polymer/steel contract prices, machine-hour build-ups at Indian energy (₹8.5/kWh) and wage levels, fully-loaded labour. They are on the Assumptions sheet with a note per line. If purchasing has better contract rates, type them in — that makes the model MORE accurate, not broken.</t>
+        </is>
+      </c>
+      <c r="D22" s="33" t="n"/>
+    </row>
+    <row r="23" ht="66" customHeight="1">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>“₹13,000 for a bumper? The aftermarket part is ₹5,000!”</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="inlineStr">
+        <is>
+          <t>Two different things. The ₹13.2k includes the ADAS electronics — radar, camera, 4 parking sensors, harness — which are ~79% of the total and are usually on separate commodity contracts. The mechanical bumper module (what a bumper supplier actually quotes) is the number on the right. Aftermarket MRP is also a retail price with distribution margins — not comparable to an OEM ex-works piece price.</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>Mechanical module ₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="D24" s="25">
+        <f>Summary!D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="66" customHeight="1">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>“What happens if the volume assumption is wrong?”</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="inlineStr">
+        <is>
+          <t>One cell: Assumptions B4. Volume only touches amortisation (tooling, fixtures, equipment) — material, process and labour are per-piece and unaffected. At 72k/yr the fascia carries ₹61 of tooling; at 36k/yr it would carry ₹122. Test any scenario in seconds by editing the cell.</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="inlineStr">
+        <is>
+          <t>Current volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" s="34">
+        <f>Assumptions!$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="66" customHeight="1">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>“Why is tooling inside the piece price?”</t>
+        </is>
+      </c>
+      <c r="C27" s="28" t="inlineStr">
+        <is>
+          <t>Convention for should-cost comparisons — most Indian RFQs quote amortised piece price. If our programme pays tooling as a separate one-time invoice, zero out column S on Parts Costing; the piece prices drop and the Tooling sheet still shows the ₹ Cr investment to negotiate separately.</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>Tooling investment ₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" s="25">
+        <f>Tooling!B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="66" customHeight="1">
+      <c r="A29" s="26" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>“Are the part weights real?”</t>
+        </is>
+      </c>
+      <c r="C29" s="28" t="inlineStr">
+        <is>
+          <t>They are engineering estimates from typical B-segment bumper benchmarks (fascia 4.2 kg, beam 4.8 kg…). They sit in yellow cells on Parts Costing — replace them with CAD or weighed actuals and the model tightens immediately. Until then treat the result as a ±15–20% class estimate.</t>
+        </is>
+      </c>
+      <c r="D29" s="29" t="n"/>
+    </row>
+    <row r="30" ht="66" customHeight="1">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="inlineStr">
+        <is>
+          <t>“The part list says ABS for the grilles but you costed PP?”</t>
+        </is>
+      </c>
+      <c r="C30" s="32" t="inlineStr">
+        <is>
+          <t>The exploded drawing says PP, the part list says ABS — a genuine document conflict, flagged rather than hidden. PP (textured black) is typical for this segment, so PP was used. To switch: change the material price reference on the two grille rows to the ABS cell — roughly +₹50/kg on ~1.2 kg of parts.</t>
+        </is>
+      </c>
+      <c r="D30" s="33" t="n"/>
+    </row>
+    <row r="31" ht="66" customHeight="1">
+      <c r="A31" s="26" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B31" s="27" t="inlineStr">
+        <is>
+          <t>“What is included and what is not?”</t>
+        </is>
+      </c>
+      <c r="C31" s="28" t="inlineStr">
+        <is>
+          <t>Included: material, process, labour, tooling amortisation, factory overhead, SG&amp;A, profit, assembly, returnable packaging — ex-works supplier. Excluded (by should-cost convention): freight to OEM plant, GST/duties, warranty provisions, ED&amp;D. Add a logistics line if you need landed cost.</t>
+        </is>
+      </c>
+      <c r="D31" s="29" t="n"/>
+    </row>
+    <row r="32" ht="66" customHeight="1">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B32" s="31" t="inlineStr">
+        <is>
+          <t>“Isn't 40% overhead too high (or too low)?”</t>
+        </is>
+      </c>
+      <c r="C32" s="32" t="inlineStr">
+        <is>
+          <t>It is applied on conversion only (process + labour), NOT on material — so it is a much smaller ₹ than it sounds. 35–50% on conversion is the normal band for Indian tier-1 plastics/stamping plants. It is one editable cell (Assumptions B38) if our benchmark differs.</t>
+        </is>
+      </c>
+      <c r="D32" s="33" t="n"/>
+    </row>
+    <row r="33" ht="66" customHeight="1">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>“How much margin did we allow the supplier?”</t>
+        </is>
+      </c>
+      <c r="C33" s="28" t="inlineStr">
+        <is>
+          <t>SG&amp;A 8% + profit 10%, both visible and editable. Together they are the negotiation band: a quote at our number ±5% is honest; a quote 25% above it needs a line-by-line conversation — and this workbook is exactly the agenda for that conversation.</t>
+        </is>
+      </c>
+      <c r="D33" s="29" t="n"/>
+    </row>
+    <row r="34" ht="66" customHeight="1">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="inlineStr">
+        <is>
+          <t>“Which parts carry the most cost?”</t>
+        </is>
+      </c>
+      <c r="C34" s="32" t="inlineStr">
+        <is>
+          <t>Painted fascia (~₹1,276 = moulding + body-colour paint), then the steel reinforcement beam (~₹495), then the grilles. Everything else is small brackets and covers below ₹120. In bought-out: the radar alone is more than the entire painted fascia.</t>
+        </is>
+      </c>
+      <c r="D34" s="35" t="inlineStr">
+        <is>
+          <t>Painted fascia ₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="D35" s="25">
+        <f>'Parts Costing'!Y4+'Parts Costing'!Y5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="66" customHeight="1">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B36" s="31" t="inlineStr">
+        <is>
+          <t>“Can we use this in a supplier negotiation?”</t>
+        </is>
+      </c>
+      <c r="C36" s="32" t="inlineStr">
+        <is>
+          <t>Yes — that is its purpose. Hand the supplier the same structure and ask them to fill THEIR numbers: where their material price, cycle time or overhead differs from ours, that specific cell becomes the discussion. Suppliers concede far more against a bottom-up model than against “please give 5% discount”.</t>
+        </is>
+      </c>
+      <c r="D36" s="33" t="n"/>
+    </row>
+    <row r="37" ht="66" customHeight="1">
+      <c r="A37" s="26" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B37" s="27" t="inlineStr">
+        <is>
+          <t>“Why does paint cost ₹416 when the paint material is only ₹185?”</t>
+        </is>
+      </c>
+      <c r="C37" s="28" t="inlineStr">
+        <is>
+          <t>Body-colour painting is a process cost, not a material cost: a robotic paint line at ₹2,800/hr with booth energy and ventilation, ~130 s per bumper, plus overhead and margin on that conversion. If the fascia is supplied moulded-in-colour, delete the paint row — the model drops it cleanly.</t>
+        </is>
+      </c>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>Paint line item ₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="D38" s="25">
+        <f>'Parts Costing'!Y5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="66" customHeight="1">
+      <c r="A39" s="26" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B39" s="27" t="inlineStr">
+        <is>
+          <t>“4 parking sensors or 8?”</t>
+        </is>
+      </c>
+      <c r="C39" s="28" t="inlineStr">
+        <is>
+          <t>Base trim = 4 (assumed), top trim = 8. One cell — Assumptions B44 — drives the sensor count, the holder count and the bought-out total together.</t>
+        </is>
+      </c>
+      <c r="D39" s="29" t="n"/>
+    </row>
+    <row r="40" ht="66" customHeight="1">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B40" s="31" t="inlineStr">
+        <is>
+          <t>“How would we make this part cheaper?”</t>
+        </is>
+      </c>
+      <c r="C40" s="32" t="inlineStr">
+        <is>
+          <t>The levers, in order of size: (1) delete/reduce paint (moulded-in-colour saves ~₹400), (2) resin contract price — every ₹10/kg on TPO is ~₹44 on the fascia, (3) volume pooling to spread tooling, (4) runner regrind reuse instead of selling scrap, (5) beam gauge/grade optimisation. The workbook quantifies each in seconds.</t>
+        </is>
+      </c>
+      <c r="D40" s="33" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1089,689 +1759,689 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="36" t="inlineStr">
         <is>
           <t>PROGRAMME</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="37" t="inlineStr">
         <is>
           <t>Annual vehicle volume</t>
         </is>
       </c>
-      <c r="B4" s="22" t="n">
+      <c r="B4" s="38" t="n">
         <v>72000</v>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C4" s="39" t="inlineStr">
         <is>
           <t>veh/yr</t>
         </is>
       </c>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D4" s="39" t="inlineStr">
         <is>
           <t>Altroz-class volume assumption — EDIT to your programme volume; all amortisation recalculates.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="37" t="inlineStr">
         <is>
           <t>Tooling amortisation period</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="40" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C5" s="39" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="39" t="inlineStr">
         <is>
           <t>Tooling amortised into piece price over volume × years (standard should-cost practice).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="40" t="inlineStr">
         <is>
           <t>INR</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr"/>
-      <c r="D6" s="23" t="inlineStr">
+      <c r="C6" s="39" t="inlineStr"/>
+      <c r="D6" s="39" t="inlineStr">
         <is>
           <t>All values in Indian Rupees, ex-works supplier (logistics to OEM excluded).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t>FX reference</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="38" t="n">
         <v>106</v>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="39" t="inlineStr">
         <is>
           <t>INR/GBP</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="39" t="inlineStr">
         <is>
           <t>Reference only — no conversion applied in this workbook.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t>MATERIAL PRICES  (₹/kg, delivered India plant)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>PP (black, textured grade)</t>
         </is>
       </c>
-      <c r="B10" s="25" t="n">
+      <c r="B10" s="41" t="n">
         <v>98</v>
       </c>
-      <c r="C10" s="23" t="inlineStr">
+      <c r="C10" s="39" t="inlineStr">
         <is>
           <t>₹/kg</t>
         </is>
       </c>
-      <c r="D10" s="23" t="inlineStr">
+      <c r="D10" s="39" t="inlineStr">
         <is>
           <t>Polypropylene copolymer, bulk OEM contract.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t>PP+EPDM (TPO bumper grade)</t>
         </is>
       </c>
-      <c r="B11" s="25" t="n">
+      <c r="B11" s="41" t="n">
         <v>142</v>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C11" s="39" t="inlineStr">
         <is>
           <t>₹/kg</t>
         </is>
       </c>
-      <c r="D11" s="23" t="inlineStr">
+      <c r="D11" s="39" t="inlineStr">
         <is>
           <t>Impact-modified bumper compound, paintable grade.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="37" t="inlineStr">
         <is>
           <t>ABS (plating/paint grade)</t>
         </is>
       </c>
-      <c r="B12" s="25" t="n">
+      <c r="B12" s="41" t="n">
         <v>148</v>
       </c>
-      <c r="C12" s="23" t="inlineStr">
+      <c r="C12" s="39" t="inlineStr">
         <is>
           <t>₹/kg</t>
         </is>
       </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="D12" s="39" t="inlineStr">
         <is>
           <t>For fog-lamp bezels / DRL housings.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="37" t="inlineStr">
         <is>
           <t>EPP beads (45 g/l)</t>
         </is>
       </c>
-      <c r="B13" s="25" t="n">
+      <c r="B13" s="41" t="n">
         <v>330</v>
       </c>
-      <c r="C13" s="23" t="inlineStr">
+      <c r="C13" s="39" t="inlineStr">
         <is>
           <t>₹/kg</t>
         </is>
       </c>
-      <c r="D13" s="23" t="inlineStr">
+      <c r="D13" s="39" t="inlineStr">
         <is>
           <t>Expanded polypropylene for energy absorber.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="37" t="inlineStr">
         <is>
           <t>POM (clips)</t>
         </is>
       </c>
-      <c r="B14" s="25" t="n">
+      <c r="B14" s="41" t="n">
         <v>210</v>
       </c>
-      <c r="C14" s="23" t="inlineStr">
+      <c r="C14" s="39" t="inlineStr">
         <is>
           <t>₹/kg</t>
         </is>
       </c>
-      <c r="D14" s="23" t="inlineStr">
+      <c r="D14" s="39" t="inlineStr">
         <is>
           <t>Reference for clip costing (bought-out set used instead).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="37" t="inlineStr">
         <is>
           <t>High-strength steel sheet (HR, 590+)</t>
         </is>
       </c>
-      <c r="B15" s="25" t="n">
+      <c r="B15" s="41" t="n">
         <v>68</v>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="C15" s="39" t="inlineStr">
         <is>
           <t>₹/kg</t>
         </is>
       </c>
-      <c r="D15" s="23" t="inlineStr">
+      <c r="D15" s="39" t="inlineStr">
         <is>
           <t>For reinforcement beam &amp; steel brackets.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="37" t="inlineStr">
         <is>
           <t>Steel scrap credit</t>
         </is>
       </c>
-      <c r="B16" s="25" t="n">
+      <c r="B16" s="41" t="n">
         <v>32</v>
       </c>
-      <c r="C16" s="23" t="inlineStr">
+      <c r="C16" s="39" t="inlineStr">
         <is>
           <t>₹/kg</t>
         </is>
       </c>
-      <c r="D16" s="23" t="inlineStr">
+      <c r="D16" s="39" t="inlineStr">
         <is>
           <t>Offal / engineered scrap sold back.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="37" t="inlineStr">
         <is>
           <t>Plastic regrind credit</t>
         </is>
       </c>
-      <c r="B17" s="25" t="n">
+      <c r="B17" s="41" t="n">
         <v>40</v>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C17" s="39" t="inlineStr">
         <is>
           <t>₹/kg</t>
         </is>
       </c>
-      <c r="D17" s="23" t="inlineStr">
+      <c r="D17" s="39" t="inlineStr">
         <is>
           <t>Runner/sprue regrind value (where not reused).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="37" t="inlineStr">
         <is>
           <t>Paint material per bumper (primer+base+clear)</t>
         </is>
       </c>
-      <c r="B18" s="25" t="n">
+      <c r="B18" s="41" t="n">
         <v>185</v>
       </c>
-      <c r="C18" s="23" t="inlineStr">
+      <c r="C18" s="39" t="inlineStr">
         <is>
           <t>₹/unit</t>
         </is>
       </c>
-      <c r="D18" s="23" t="inlineStr">
+      <c r="D18" s="39" t="inlineStr">
         <is>
           <t>Body-colour robotic paint, material only.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="A20" s="36" t="inlineStr">
         <is>
           <t>MACHINE RATES  (₹/hr — includes depreciation, energy @ ₹8.5/kWh, maintenance, floor space, supervision)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="37" t="inlineStr">
         <is>
           <t>Injection moulding 1500T</t>
         </is>
       </c>
-      <c r="B21" s="26" t="n">
+      <c r="B21" s="42" t="n">
         <v>2100</v>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C21" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D21" s="23" t="inlineStr">
+      <c r="D21" s="39" t="inlineStr">
         <is>
           <t>For bumper fascia.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="37" t="inlineStr">
         <is>
           <t>Injection moulding 800T</t>
         </is>
       </c>
-      <c r="B22" s="26" t="n">
+      <c r="B22" s="42" t="n">
         <v>1150</v>
       </c>
-      <c r="C22" s="23" t="inlineStr">
+      <c r="C22" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D22" s="23" t="inlineStr">
+      <c r="D22" s="39" t="inlineStr">
         <is>
           <t>Spare class (unused by default).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="37" t="inlineStr">
         <is>
           <t>Injection moulding 450T</t>
         </is>
       </c>
-      <c r="B23" s="26" t="n">
+      <c r="B23" s="42" t="n">
         <v>700</v>
       </c>
-      <c r="C23" s="23" t="inlineStr">
+      <c r="C23" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D23" s="23" t="inlineStr">
+      <c r="D23" s="39" t="inlineStr">
         <is>
           <t>Grilles, air deflector.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="37" t="inlineStr">
         <is>
           <t>Injection moulding 250T</t>
         </is>
       </c>
-      <c r="B24" s="26" t="n">
+      <c r="B24" s="42" t="n">
         <v>520</v>
       </c>
-      <c r="C24" s="23" t="inlineStr">
+      <c r="C24" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D24" s="23" t="inlineStr">
+      <c r="D24" s="39" t="inlineStr">
         <is>
           <t>Bezels, wheel-arch retainers.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="inlineStr">
+      <c r="A25" s="37" t="inlineStr">
         <is>
           <t>Injection moulding 150T</t>
         </is>
       </c>
-      <c r="B25" s="26" t="n">
+      <c r="B25" s="42" t="n">
         <v>400</v>
       </c>
-      <c r="C25" s="23" t="inlineStr">
+      <c r="C25" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D25" s="23" t="inlineStr">
+      <c r="D25" s="39" t="inlineStr">
         <is>
           <t>Small brackets, holders, covers.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="37" t="inlineStr">
         <is>
           <t>EPP shape-moulding machine</t>
         </is>
       </c>
-      <c r="B26" s="26" t="n">
+      <c r="B26" s="42" t="n">
         <v>650</v>
       </c>
-      <c r="C26" s="23" t="inlineStr">
+      <c r="C26" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D26" s="23" t="inlineStr">
+      <c r="D26" s="39" t="inlineStr">
         <is>
           <t>Steam-chest moulding for energy absorber.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="21" t="inlineStr">
+      <c r="A27" s="37" t="inlineStr">
         <is>
           <t>Progressive press 250T (with feeder)</t>
         </is>
       </c>
-      <c r="B27" s="26" t="n">
+      <c r="B27" s="42" t="n">
         <v>900</v>
       </c>
-      <c r="C27" s="23" t="inlineStr">
+      <c r="C27" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D27" s="23" t="inlineStr">
+      <c r="D27" s="39" t="inlineStr">
         <is>
           <t>Steel beam brackets.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="37" t="inlineStr">
         <is>
           <t>Rollform + pierce + sweep line</t>
         </is>
       </c>
-      <c r="B28" s="26" t="n">
+      <c r="B28" s="42" t="n">
         <v>1600</v>
       </c>
-      <c r="C28" s="23" t="inlineStr">
+      <c r="C28" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D28" s="23" t="inlineStr">
+      <c r="D28" s="39" t="inlineStr">
         <is>
           <t>Reinforcement beam forming.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="37" t="inlineStr">
         <is>
           <t>MIG/spot weld cell</t>
         </is>
       </c>
-      <c r="B29" s="26" t="n">
+      <c r="B29" s="42" t="n">
         <v>800</v>
       </c>
-      <c r="C29" s="23" t="inlineStr">
+      <c r="C29" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D29" s="23" t="inlineStr">
+      <c r="D29" s="39" t="inlineStr">
         <is>
           <t>Beam bracket welding.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="inlineStr">
+      <c r="A30" s="37" t="inlineStr">
         <is>
           <t>Robotic paint line (bumper)</t>
         </is>
       </c>
-      <c r="B30" s="26" t="n">
+      <c r="B30" s="42" t="n">
         <v>2800</v>
       </c>
-      <c r="C30" s="23" t="inlineStr">
+      <c r="C30" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D30" s="23" t="inlineStr">
+      <c r="D30" s="39" t="inlineStr">
         <is>
           <t>Conveyorised, incl. booth energy &amp; ventilation.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="20" t="inlineStr">
+      <c r="A32" s="36" t="inlineStr">
         <is>
           <t>LABOUR RATES  (₹/hr, fully loaded — wages + statutory + benefits + supervision share)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="21" t="inlineStr">
+      <c r="A33" s="37" t="inlineStr">
         <is>
           <t>Operator (semi-skilled)</t>
         </is>
       </c>
-      <c r="B33" s="26" t="n">
+      <c r="B33" s="42" t="n">
         <v>190</v>
       </c>
-      <c r="C33" s="23" t="inlineStr">
+      <c r="C33" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D33" s="23" t="inlineStr">
+      <c r="D33" s="39" t="inlineStr">
         <is>
           <t>Press/moulding/assembly operator.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="21" t="inlineStr">
+      <c r="A34" s="37" t="inlineStr">
         <is>
           <t>Skilled (setter / welder / painter)</t>
         </is>
       </c>
-      <c r="B34" s="26" t="n">
+      <c r="B34" s="42" t="n">
         <v>260</v>
       </c>
-      <c r="C34" s="23" t="inlineStr">
+      <c r="C34" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D34" s="23" t="inlineStr"/>
+      <c r="D34" s="39" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="21" t="inlineStr">
+      <c r="A35" s="37" t="inlineStr">
         <is>
           <t>Quality inspector</t>
         </is>
       </c>
-      <c r="B35" s="26" t="n">
+      <c r="B35" s="42" t="n">
         <v>230</v>
       </c>
-      <c r="C35" s="23" t="inlineStr">
+      <c r="C35" s="39" t="inlineStr">
         <is>
           <t>₹/hr</t>
         </is>
       </c>
-      <c r="D35" s="23" t="inlineStr">
+      <c r="D35" s="39" t="inlineStr">
         <is>
           <t>End-of-line checks.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="20" t="inlineStr">
+      <c r="A37" s="36" t="inlineStr">
         <is>
           <t>COMMERCIAL FACTORS</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="21" t="inlineStr">
+      <c r="A38" s="37" t="inlineStr">
         <is>
           <t>Factory overhead (on conversion cost)</t>
         </is>
       </c>
-      <c r="B38" s="27" t="n">
+      <c r="B38" s="43" t="n">
         <v>0.4</v>
       </c>
-      <c r="C38" s="23" t="inlineStr">
+      <c r="C38" s="39" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D38" s="23" t="inlineStr">
+      <c r="D38" s="39" t="inlineStr">
         <is>
           <t>Indirect staff, utilities, quality system, maintenance overheads.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+      <c r="A39" s="37" t="inlineStr">
         <is>
           <t>SG&amp;A</t>
         </is>
       </c>
-      <c r="B39" s="27" t="n">
+      <c r="B39" s="43" t="n">
         <v>0.08</v>
       </c>
-      <c r="C39" s="23" t="inlineStr">
+      <c r="C39" s="39" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D39" s="23" t="inlineStr">
+      <c r="D39" s="39" t="inlineStr">
         <is>
           <t>Sales, general &amp; administrative on manufacturing cost.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="21" t="inlineStr">
+      <c r="A40" s="37" t="inlineStr">
         <is>
           <t>Profit</t>
         </is>
       </c>
-      <c r="B40" s="27" t="n">
+      <c r="B40" s="43" t="n">
         <v>0.1</v>
       </c>
-      <c r="C40" s="23" t="inlineStr">
+      <c r="C40" s="39" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D40" s="23" t="inlineStr">
+      <c r="D40" s="39" t="inlineStr">
         <is>
           <t>Supplier margin on manufacturing cost + SG&amp;A.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="21" t="inlineStr">
+      <c r="A41" s="37" t="inlineStr">
         <is>
           <t>Bought-out handling &amp; inbound</t>
         </is>
       </c>
-      <c r="B41" s="27" t="n">
+      <c r="B41" s="43" t="n">
         <v>0.03</v>
       </c>
-      <c r="C41" s="23" t="inlineStr">
+      <c r="C41" s="39" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D41" s="23" t="inlineStr">
+      <c r="D41" s="39" t="inlineStr">
         <is>
           <t>Applied to bought-out (pass-through) items.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="21" t="inlineStr">
+      <c r="A42" s="37" t="inlineStr">
         <is>
           <t>Assembly overhead (on assembly conversion)</t>
         </is>
       </c>
-      <c r="B42" s="27" t="n">
+      <c r="B42" s="43" t="n">
         <v>0.45</v>
       </c>
-      <c r="C42" s="23" t="inlineStr">
+      <c r="C42" s="39" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D42" s="23" t="inlineStr">
+      <c r="D42" s="39" t="inlineStr">
         <is>
           <t>Line management, MHE, utilities at assembly plant.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="21" t="inlineStr">
+      <c r="A43" s="37" t="inlineStr">
         <is>
           <t>Packaging per finished assembly</t>
         </is>
       </c>
-      <c r="B43" s="25" t="n">
+      <c r="B43" s="41" t="n">
         <v>55</v>
       </c>
-      <c r="C43" s="23" t="inlineStr">
+      <c r="C43" s="39" t="inlineStr">
         <is>
           <t>₹/unit</t>
         </is>
       </c>
-      <c r="D43" s="23" t="inlineStr">
+      <c r="D43" s="39" t="inlineStr">
         <is>
           <t>Returnable dunnage trip cost, amortised.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="21" t="inlineStr">
+      <c r="A44" s="37" t="inlineStr">
         <is>
           <t>Parking sensors fitted</t>
         </is>
       </c>
-      <c r="B44" s="28" t="n">
+      <c r="B44" s="44" t="n">
         <v>4</v>
       </c>
-      <c r="C44" s="23" t="inlineStr">
+      <c r="C44" s="39" t="inlineStr">
         <is>
           <t>pcs</t>
         </is>
       </c>
-      <c r="D44" s="23" t="inlineStr">
+      <c r="D44" s="39" t="inlineStr">
         <is>
           <t>Part list says 4–8 — set 4 (base) to 8 (top trim); sensors, holders &amp; BOM recalc.</t>
         </is>
@@ -1791,7 +2461,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1975,1855 +2645,1855 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="29" t="n">
+      <c r="A4" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="30" t="inlineStr">
+      <c r="B4" s="46" t="inlineStr">
         <is>
           <t>Front bumper fascia</t>
         </is>
       </c>
-      <c r="C4" s="31" t="inlineStr">
+      <c r="C4" s="47" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D4" s="31" t="inlineStr">
+      <c r="D4" s="47" t="inlineStr">
         <is>
           <t>PP+EPDM (TPO)</t>
         </is>
       </c>
-      <c r="E4" s="29" t="n">
+      <c r="E4" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="32" t="n">
+      <c r="F4" s="48" t="n">
         <v>4.2</v>
       </c>
-      <c r="G4" s="33" t="n">
+      <c r="G4" s="49" t="n">
         <v>0.04</v>
       </c>
-      <c r="H4" s="34">
+      <c r="H4" s="50">
         <f>Assumptions!$B$11</f>
         <v/>
       </c>
-      <c r="I4" s="34">
+      <c r="I4" s="50">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J4" s="34">
+      <c r="J4" s="50">
         <f>F4*(1+G4)*H4-F4*G4*I4</f>
         <v/>
       </c>
-      <c r="K4" s="31" t="inlineStr">
+      <c r="K4" s="47" t="inlineStr">
         <is>
           <t>IMM 1500T</t>
         </is>
       </c>
-      <c r="L4" s="35">
+      <c r="L4" s="51">
         <f>Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="M4" s="36" t="n">
+      <c r="M4" s="52" t="n">
         <v>58</v>
       </c>
-      <c r="N4" s="37" t="n">
+      <c r="N4" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="O4" s="34">
+      <c r="O4" s="50">
         <f>M4*L4/3600/N4</f>
         <v/>
       </c>
-      <c r="P4" s="37" t="n">
+      <c r="P4" s="53" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q4" s="35">
+      <c r="Q4" s="51">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R4" s="34">
+      <c r="R4" s="50">
         <f>M4*P4*Q4/3600/N4</f>
         <v/>
       </c>
-      <c r="S4" s="38" t="n">
+      <c r="S4" s="54" t="n">
         <v>22000000</v>
       </c>
-      <c r="T4" s="34">
+      <c r="T4" s="50">
         <f>S4/(Assumptions!$B$4*Assumptions!$B$5*E4)</f>
         <v/>
       </c>
-      <c r="U4" s="34">
+      <c r="U4" s="50">
         <f>(O4+R4)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V4" s="34">
+      <c r="V4" s="50">
         <f>J4+O4+R4+T4+U4</f>
         <v/>
       </c>
-      <c r="W4" s="34">
+      <c r="W4" s="50">
         <f>V4*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X4" s="34">
+      <c r="X4" s="50">
         <f>(V4+W4)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y4" s="39">
+      <c r="Y4" s="55">
         <f>V4+W4+X4</f>
         <v/>
       </c>
-      <c r="Z4" s="39">
+      <c r="Z4" s="55">
         <f>Y4*E4</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="40" t="n">
+      <c r="A5" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="41" t="inlineStr">
+      <c r="B5" s="57" t="inlineStr">
         <is>
           <t>Painting — fascia, body colour</t>
         </is>
       </c>
-      <c r="C5" s="42" t="inlineStr">
+      <c r="C5" s="58" t="inlineStr">
         <is>
           <t>Robotic paint (P+B+C)</t>
         </is>
       </c>
-      <c r="D5" s="42" t="inlineStr">
+      <c r="D5" s="58" t="inlineStr">
         <is>
           <t>Paint system</t>
         </is>
       </c>
-      <c r="E5" s="40" t="n">
+      <c r="E5" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="40" t="n"/>
-      <c r="G5" s="40" t="n"/>
-      <c r="H5" s="40" t="n"/>
-      <c r="I5" s="40" t="n"/>
-      <c r="J5" s="43">
+      <c r="F5" s="56" t="n"/>
+      <c r="G5" s="56" t="n"/>
+      <c r="H5" s="56" t="n"/>
+      <c r="I5" s="56" t="n"/>
+      <c r="J5" s="59">
         <f>Assumptions!$B$18</f>
         <v/>
       </c>
-      <c r="K5" s="42" t="inlineStr">
+      <c r="K5" s="58" t="inlineStr">
         <is>
           <t>Paint line</t>
         </is>
       </c>
-      <c r="L5" s="44">
+      <c r="L5" s="60">
         <f>Assumptions!$B$30</f>
         <v/>
       </c>
-      <c r="M5" s="36" t="n">
+      <c r="M5" s="52" t="n">
         <v>130</v>
       </c>
-      <c r="N5" s="37" t="n">
+      <c r="N5" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="O5" s="43">
+      <c r="O5" s="59">
         <f>M5*L5/3600/N5</f>
         <v/>
       </c>
-      <c r="P5" s="37" t="n">
+      <c r="P5" s="53" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q5" s="44">
+      <c r="Q5" s="60">
         <f>Assumptions!$B$34</f>
         <v/>
       </c>
-      <c r="R5" s="43">
+      <c r="R5" s="59">
         <f>M5*P5*Q5/3600/N5</f>
         <v/>
       </c>
-      <c r="S5" s="38" t="n">
+      <c r="S5" s="54" t="n">
         <v>6000000</v>
       </c>
-      <c r="T5" s="43">
+      <c r="T5" s="59">
         <f>S5/(Assumptions!$B$4*Assumptions!$B$5*E5)</f>
         <v/>
       </c>
-      <c r="U5" s="43">
+      <c r="U5" s="59">
         <f>(O5+R5)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V5" s="43">
+      <c r="V5" s="59">
         <f>J5+O5+R5+T5+U5</f>
         <v/>
       </c>
-      <c r="W5" s="43">
+      <c r="W5" s="59">
         <f>V5*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X5" s="43">
+      <c r="X5" s="59">
         <f>(V5+W5)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y5" s="45">
+      <c r="Y5" s="61">
         <f>V5+W5+X5</f>
         <v/>
       </c>
-      <c r="Z5" s="45">
+      <c r="Z5" s="61">
         <f>Y5*E5</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="29" t="n">
+      <c r="A6" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="46" t="inlineStr">
         <is>
           <t>Upper grille</t>
         </is>
       </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C6" s="47" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D6" s="31" t="inlineStr">
+      <c r="D6" s="47" t="inlineStr">
         <is>
           <t>PP (textured)</t>
         </is>
       </c>
-      <c r="E6" s="29" t="n">
+      <c r="E6" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="32" t="n">
+      <c r="F6" s="48" t="n">
         <v>0.55</v>
       </c>
-      <c r="G6" s="33" t="n">
+      <c r="G6" s="49" t="n">
         <v>0.05</v>
       </c>
-      <c r="H6" s="34">
+      <c r="H6" s="50">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="I6" s="34">
+      <c r="I6" s="50">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J6" s="34">
+      <c r="J6" s="50">
         <f>F6*(1+G6)*H6-F6*G6*I6</f>
         <v/>
       </c>
-      <c r="K6" s="31" t="inlineStr">
+      <c r="K6" s="47" t="inlineStr">
         <is>
           <t>IMM 450T</t>
         </is>
       </c>
-      <c r="L6" s="35">
+      <c r="L6" s="51">
         <f>Assumptions!$B$23</f>
         <v/>
       </c>
-      <c r="M6" s="36" t="n">
+      <c r="M6" s="52" t="n">
         <v>34</v>
       </c>
-      <c r="N6" s="37" t="n">
+      <c r="N6" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="O6" s="34">
+      <c r="O6" s="50">
         <f>M6*L6/3600/N6</f>
         <v/>
       </c>
-      <c r="P6" s="37" t="n">
+      <c r="P6" s="53" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q6" s="35">
+      <c r="Q6" s="51">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R6" s="34">
+      <c r="R6" s="50">
         <f>M6*P6*Q6/3600/N6</f>
         <v/>
       </c>
-      <c r="S6" s="38" t="n">
+      <c r="S6" s="54" t="n">
         <v>5500000</v>
       </c>
-      <c r="T6" s="34">
+      <c r="T6" s="50">
         <f>S6/(Assumptions!$B$4*Assumptions!$B$5*E6)</f>
         <v/>
       </c>
-      <c r="U6" s="34">
+      <c r="U6" s="50">
         <f>(O6+R6)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V6" s="34">
+      <c r="V6" s="50">
         <f>J6+O6+R6+T6+U6</f>
         <v/>
       </c>
-      <c r="W6" s="34">
+      <c r="W6" s="50">
         <f>V6*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X6" s="34">
+      <c r="X6" s="50">
         <f>(V6+W6)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y6" s="39">
+      <c r="Y6" s="55">
         <f>V6+W6+X6</f>
         <v/>
       </c>
-      <c r="Z6" s="39">
+      <c r="Z6" s="55">
         <f>Y6*E6</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="40" t="n">
+      <c r="A7" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="41" t="inlineStr">
+      <c r="B7" s="57" t="inlineStr">
         <is>
           <t>Lower grille</t>
         </is>
       </c>
-      <c r="C7" s="42" t="inlineStr">
+      <c r="C7" s="58" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D7" s="42" t="inlineStr">
+      <c r="D7" s="58" t="inlineStr">
         <is>
           <t>PP (textured)</t>
         </is>
       </c>
-      <c r="E7" s="40" t="n">
+      <c r="E7" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="32" t="n">
+      <c r="F7" s="48" t="n">
         <v>0.65</v>
       </c>
-      <c r="G7" s="33" t="n">
+      <c r="G7" s="49" t="n">
         <v>0.05</v>
       </c>
-      <c r="H7" s="43">
+      <c r="H7" s="59">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="I7" s="43">
+      <c r="I7" s="59">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J7" s="43">
+      <c r="J7" s="59">
         <f>F7*(1+G7)*H7-F7*G7*I7</f>
         <v/>
       </c>
-      <c r="K7" s="42" t="inlineStr">
+      <c r="K7" s="58" t="inlineStr">
         <is>
           <t>IMM 450T</t>
         </is>
       </c>
-      <c r="L7" s="44">
+      <c r="L7" s="60">
         <f>Assumptions!$B$23</f>
         <v/>
       </c>
-      <c r="M7" s="36" t="n">
+      <c r="M7" s="52" t="n">
         <v>40</v>
       </c>
-      <c r="N7" s="37" t="n">
+      <c r="N7" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="O7" s="43">
+      <c r="O7" s="59">
         <f>M7*L7/3600/N7</f>
         <v/>
       </c>
-      <c r="P7" s="37" t="n">
+      <c r="P7" s="53" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q7" s="44">
+      <c r="Q7" s="60">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R7" s="43">
+      <c r="R7" s="59">
         <f>M7*P7*Q7/3600/N7</f>
         <v/>
       </c>
-      <c r="S7" s="38" t="n">
+      <c r="S7" s="54" t="n">
         <v>5500000</v>
       </c>
-      <c r="T7" s="43">
+      <c r="T7" s="59">
         <f>S7/(Assumptions!$B$4*Assumptions!$B$5*E7)</f>
         <v/>
       </c>
-      <c r="U7" s="43">
+      <c r="U7" s="59">
         <f>(O7+R7)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V7" s="43">
+      <c r="V7" s="59">
         <f>J7+O7+R7+T7+U7</f>
         <v/>
       </c>
-      <c r="W7" s="43">
+      <c r="W7" s="59">
         <f>V7*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X7" s="43">
+      <c r="X7" s="59">
         <f>(V7+W7)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y7" s="45">
+      <c r="Y7" s="61">
         <f>V7+W7+X7</f>
         <v/>
       </c>
-      <c r="Z7" s="45">
+      <c r="Z7" s="61">
         <f>Y7*E7</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="29" t="n">
+      <c r="A8" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="30" t="inlineStr">
+      <c r="B8" s="46" t="inlineStr">
         <is>
           <t>Side bracket LH+RH (fascia)</t>
         </is>
       </c>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D8" s="31" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>PP</t>
         </is>
       </c>
-      <c r="E8" s="29" t="n">
+      <c r="E8" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="32" t="n">
+      <c r="F8" s="48" t="n">
         <v>0.12</v>
       </c>
-      <c r="G8" s="33" t="n">
+      <c r="G8" s="49" t="n">
         <v>0.04</v>
       </c>
-      <c r="H8" s="34">
+      <c r="H8" s="50">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="I8" s="34">
+      <c r="I8" s="50">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J8" s="34">
+      <c r="J8" s="50">
         <f>F8*(1+G8)*H8-F8*G8*I8</f>
         <v/>
       </c>
-      <c r="K8" s="31" t="inlineStr">
+      <c r="K8" s="47" t="inlineStr">
         <is>
           <t>IMM 150T</t>
         </is>
       </c>
-      <c r="L8" s="35">
+      <c r="L8" s="51">
         <f>Assumptions!$B$25</f>
         <v/>
       </c>
-      <c r="M8" s="36" t="n">
+      <c r="M8" s="52" t="n">
         <v>26</v>
       </c>
-      <c r="N8" s="37" t="n">
+      <c r="N8" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="O8" s="34">
+      <c r="O8" s="50">
         <f>M8*L8/3600/N8</f>
         <v/>
       </c>
-      <c r="P8" s="37" t="n">
+      <c r="P8" s="53" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q8" s="35">
+      <c r="Q8" s="51">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R8" s="34">
+      <c r="R8" s="50">
         <f>M8*P8*Q8/3600/N8</f>
         <v/>
       </c>
-      <c r="S8" s="38" t="n">
+      <c r="S8" s="54" t="n">
         <v>1800000</v>
       </c>
-      <c r="T8" s="34">
+      <c r="T8" s="50">
         <f>S8/(Assumptions!$B$4*Assumptions!$B$5*E8)</f>
         <v/>
       </c>
-      <c r="U8" s="34">
+      <c r="U8" s="50">
         <f>(O8+R8)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V8" s="34">
+      <c r="V8" s="50">
         <f>J8+O8+R8+T8+U8</f>
         <v/>
       </c>
-      <c r="W8" s="34">
+      <c r="W8" s="50">
         <f>V8*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X8" s="34">
+      <c r="X8" s="50">
         <f>(V8+W8)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y8" s="39">
+      <c r="Y8" s="55">
         <f>V8+W8+X8</f>
         <v/>
       </c>
-      <c r="Z8" s="39">
+      <c r="Z8" s="55">
         <f>Y8*E8</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="40" t="n">
+      <c r="A9" s="56" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="41" t="inlineStr">
+      <c r="B9" s="57" t="inlineStr">
         <is>
           <t>Number / licence plate bracket</t>
         </is>
       </c>
-      <c r="C9" s="42" t="inlineStr">
+      <c r="C9" s="58" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
+      <c r="D9" s="58" t="inlineStr">
         <is>
           <t>PP</t>
         </is>
       </c>
-      <c r="E9" s="40" t="n">
+      <c r="E9" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="32" t="n">
+      <c r="F9" s="48" t="n">
         <v>0.18</v>
       </c>
-      <c r="G9" s="33" t="n">
+      <c r="G9" s="49" t="n">
         <v>0.04</v>
       </c>
-      <c r="H9" s="43">
+      <c r="H9" s="59">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="I9" s="43">
+      <c r="I9" s="59">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J9" s="43">
+      <c r="J9" s="59">
         <f>F9*(1+G9)*H9-F9*G9*I9</f>
         <v/>
       </c>
-      <c r="K9" s="42" t="inlineStr">
+      <c r="K9" s="58" t="inlineStr">
         <is>
           <t>IMM 150T</t>
         </is>
       </c>
-      <c r="L9" s="44">
+      <c r="L9" s="60">
         <f>Assumptions!$B$25</f>
         <v/>
       </c>
-      <c r="M9" s="36" t="n">
+      <c r="M9" s="52" t="n">
         <v>28</v>
       </c>
-      <c r="N9" s="37" t="n">
+      <c r="N9" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="O9" s="43">
+      <c r="O9" s="59">
         <f>M9*L9/3600/N9</f>
         <v/>
       </c>
-      <c r="P9" s="37" t="n">
+      <c r="P9" s="53" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q9" s="44">
+      <c r="Q9" s="60">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R9" s="43">
+      <c r="R9" s="59">
         <f>M9*P9*Q9/3600/N9</f>
         <v/>
       </c>
-      <c r="S9" s="38" t="n">
+      <c r="S9" s="54" t="n">
         <v>1200000</v>
       </c>
-      <c r="T9" s="43">
+      <c r="T9" s="59">
         <f>S9/(Assumptions!$B$4*Assumptions!$B$5*E9)</f>
         <v/>
       </c>
-      <c r="U9" s="43">
+      <c r="U9" s="59">
         <f>(O9+R9)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V9" s="43">
+      <c r="V9" s="59">
         <f>J9+O9+R9+T9+U9</f>
         <v/>
       </c>
-      <c r="W9" s="43">
+      <c r="W9" s="59">
         <f>V9*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X9" s="43">
+      <c r="X9" s="59">
         <f>(V9+W9)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y9" s="45">
+      <c r="Y9" s="61">
         <f>V9+W9+X9</f>
         <v/>
       </c>
-      <c r="Z9" s="45">
+      <c r="Z9" s="61">
         <f>Y9*E9</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="29" t="n">
+      <c r="A10" s="45" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="30" t="inlineStr">
+      <c r="B10" s="46" t="inlineStr">
         <is>
           <t>Fog lamp bezel / DRL housing LH+RH</t>
         </is>
       </c>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C10" s="47" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D10" s="31" t="inlineStr">
+      <c r="D10" s="47" t="inlineStr">
         <is>
           <t>ABS</t>
         </is>
       </c>
-      <c r="E10" s="29" t="n">
+      <c r="E10" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="32" t="n">
+      <c r="F10" s="48" t="n">
         <v>0.15</v>
       </c>
-      <c r="G10" s="33" t="n">
+      <c r="G10" s="49" t="n">
         <v>0.05</v>
       </c>
-      <c r="H10" s="34">
+      <c r="H10" s="50">
         <f>Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="I10" s="34">
+      <c r="I10" s="50">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J10" s="34">
+      <c r="J10" s="50">
         <f>F10*(1+G10)*H10-F10*G10*I10</f>
         <v/>
       </c>
-      <c r="K10" s="31" t="inlineStr">
+      <c r="K10" s="47" t="inlineStr">
         <is>
           <t>IMM 250T</t>
         </is>
       </c>
-      <c r="L10" s="35">
+      <c r="L10" s="51">
         <f>Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="M10" s="36" t="n">
+      <c r="M10" s="52" t="n">
         <v>34</v>
       </c>
-      <c r="N10" s="37" t="n">
+      <c r="N10" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="O10" s="34">
+      <c r="O10" s="50">
         <f>M10*L10/3600/N10</f>
         <v/>
       </c>
-      <c r="P10" s="37" t="n">
+      <c r="P10" s="53" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q10" s="35">
+      <c r="Q10" s="51">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R10" s="34">
+      <c r="R10" s="50">
         <f>M10*P10*Q10/3600/N10</f>
         <v/>
       </c>
-      <c r="S10" s="38" t="n">
+      <c r="S10" s="54" t="n">
         <v>2800000</v>
       </c>
-      <c r="T10" s="34">
+      <c r="T10" s="50">
         <f>S10/(Assumptions!$B$4*Assumptions!$B$5*E10)</f>
         <v/>
       </c>
-      <c r="U10" s="34">
+      <c r="U10" s="50">
         <f>(O10+R10)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V10" s="34">
+      <c r="V10" s="50">
         <f>J10+O10+R10+T10+U10</f>
         <v/>
       </c>
-      <c r="W10" s="34">
+      <c r="W10" s="50">
         <f>V10*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X10" s="34">
+      <c r="X10" s="50">
         <f>(V10+W10)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y10" s="39">
+      <c r="Y10" s="55">
         <f>V10+W10+X10</f>
         <v/>
       </c>
-      <c r="Z10" s="39">
+      <c r="Z10" s="55">
         <f>Y10*E10</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="40" t="n">
+      <c r="A11" s="56" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="41" t="inlineStr">
+      <c r="B11" s="57" t="inlineStr">
         <is>
           <t>Energy absorber</t>
         </is>
       </c>
-      <c r="C11" s="42" t="inlineStr">
+      <c r="C11" s="58" t="inlineStr">
         <is>
           <t>EPP shape moulding</t>
         </is>
       </c>
-      <c r="D11" s="42" t="inlineStr">
+      <c r="D11" s="58" t="inlineStr">
         <is>
           <t>EPP foam 45 g/l</t>
         </is>
       </c>
-      <c r="E11" s="40" t="n">
+      <c r="E11" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="32" t="n">
+      <c r="F11" s="48" t="n">
         <v>0.3</v>
       </c>
-      <c r="G11" s="33" t="n">
+      <c r="G11" s="49" t="n">
         <v>0.02</v>
       </c>
-      <c r="H11" s="43">
+      <c r="H11" s="59">
         <f>Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="I11" s="43">
+      <c r="I11" s="59">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J11" s="43">
+      <c r="J11" s="59">
         <f>F11*(1+G11)*H11-F11*G11*I11</f>
         <v/>
       </c>
-      <c r="K11" s="42" t="inlineStr">
+      <c r="K11" s="58" t="inlineStr">
         <is>
           <t>EPP moulder</t>
         </is>
       </c>
-      <c r="L11" s="44">
+      <c r="L11" s="60">
         <f>Assumptions!$B$26</f>
         <v/>
       </c>
-      <c r="M11" s="36" t="n">
+      <c r="M11" s="52" t="n">
         <v>95</v>
       </c>
-      <c r="N11" s="37" t="n">
+      <c r="N11" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="O11" s="43">
+      <c r="O11" s="59">
         <f>M11*L11/3600/N11</f>
         <v/>
       </c>
-      <c r="P11" s="37" t="n">
+      <c r="P11" s="53" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q11" s="44">
+      <c r="Q11" s="60">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R11" s="43">
+      <c r="R11" s="59">
         <f>M11*P11*Q11/3600/N11</f>
         <v/>
       </c>
-      <c r="S11" s="38" t="n">
+      <c r="S11" s="54" t="n">
         <v>3500000</v>
       </c>
-      <c r="T11" s="43">
+      <c r="T11" s="59">
         <f>S11/(Assumptions!$B$4*Assumptions!$B$5*E11)</f>
         <v/>
       </c>
-      <c r="U11" s="43">
+      <c r="U11" s="59">
         <f>(O11+R11)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V11" s="43">
+      <c r="V11" s="59">
         <f>J11+O11+R11+T11+U11</f>
         <v/>
       </c>
-      <c r="W11" s="43">
+      <c r="W11" s="59">
         <f>V11*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X11" s="43">
+      <c r="X11" s="59">
         <f>(V11+W11)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y11" s="45">
+      <c r="Y11" s="61">
         <f>V11+W11+X11</f>
         <v/>
       </c>
-      <c r="Z11" s="45">
+      <c r="Z11" s="61">
         <f>Y11*E11</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="29" t="n">
+      <c r="A12" s="45" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="30" t="inlineStr">
+      <c r="B12" s="46" t="inlineStr">
         <is>
           <t>Reinforcement beam — form &amp; pierce</t>
         </is>
       </c>
-      <c r="C12" s="31" t="inlineStr">
+      <c r="C12" s="47" t="inlineStr">
         <is>
           <t>Rollform + sweep</t>
         </is>
       </c>
-      <c r="D12" s="31" t="inlineStr">
+      <c r="D12" s="47" t="inlineStr">
         <is>
           <t>HSS 590 sheet</t>
         </is>
       </c>
-      <c r="E12" s="29" t="n">
+      <c r="E12" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="32" t="n">
+      <c r="F12" s="48" t="n">
         <v>4.8</v>
       </c>
-      <c r="G12" s="33" t="n">
+      <c r="G12" s="49" t="n">
         <v>0.08</v>
       </c>
-      <c r="H12" s="34">
+      <c r="H12" s="50">
         <f>Assumptions!$B$15</f>
         <v/>
       </c>
-      <c r="I12" s="34">
+      <c r="I12" s="50">
         <f>Assumptions!$B$16</f>
         <v/>
       </c>
-      <c r="J12" s="34">
+      <c r="J12" s="50">
         <f>F12*(1+G12)*H12-F12*G12*I12</f>
         <v/>
       </c>
-      <c r="K12" s="31" t="inlineStr">
+      <c r="K12" s="47" t="inlineStr">
         <is>
           <t>Rollform line</t>
         </is>
       </c>
-      <c r="L12" s="35">
+      <c r="L12" s="51">
         <f>Assumptions!$B$28</f>
         <v/>
       </c>
-      <c r="M12" s="36" t="n">
+      <c r="M12" s="52" t="n">
         <v>45</v>
       </c>
-      <c r="N12" s="37" t="n">
+      <c r="N12" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="O12" s="34">
+      <c r="O12" s="50">
         <f>M12*L12/3600/N12</f>
         <v/>
       </c>
-      <c r="P12" s="37" t="n">
+      <c r="P12" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="Q12" s="35">
+      <c r="Q12" s="51">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R12" s="34">
+      <c r="R12" s="50">
         <f>M12*P12*Q12/3600/N12</f>
         <v/>
       </c>
-      <c r="S12" s="38" t="n">
+      <c r="S12" s="54" t="n">
         <v>6000000</v>
       </c>
-      <c r="T12" s="34">
+      <c r="T12" s="50">
         <f>S12/(Assumptions!$B$4*Assumptions!$B$5*E12)</f>
         <v/>
       </c>
-      <c r="U12" s="34">
+      <c r="U12" s="50">
         <f>(O12+R12)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V12" s="34">
+      <c r="V12" s="50">
         <f>J12+O12+R12+T12+U12</f>
         <v/>
       </c>
-      <c r="W12" s="34">
+      <c r="W12" s="50">
         <f>V12*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X12" s="34">
+      <c r="X12" s="50">
         <f>(V12+W12)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y12" s="39">
+      <c r="Y12" s="55">
         <f>V12+W12+X12</f>
         <v/>
       </c>
-      <c r="Z12" s="39">
+      <c r="Z12" s="55">
         <f>Y12*E12</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="40" t="n">
+      <c r="A13" s="56" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="41" t="inlineStr">
+      <c r="B13" s="57" t="inlineStr">
         <is>
           <t>Reinforcement beam — bracket welding</t>
         </is>
       </c>
-      <c r="C13" s="42" t="inlineStr">
+      <c r="C13" s="58" t="inlineStr">
         <is>
           <t>MIG weld op</t>
         </is>
       </c>
-      <c r="D13" s="42" t="inlineStr">
+      <c r="D13" s="58" t="inlineStr">
         <is>
           <t>(consumables in rate)</t>
         </is>
       </c>
-      <c r="E13" s="40" t="n">
+      <c r="E13" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="40" t="n"/>
-      <c r="G13" s="40" t="n"/>
-      <c r="H13" s="40" t="n"/>
-      <c r="I13" s="40" t="n"/>
-      <c r="J13" s="43" t="n">
+      <c r="F13" s="56" t="n"/>
+      <c r="G13" s="56" t="n"/>
+      <c r="H13" s="56" t="n"/>
+      <c r="I13" s="56" t="n"/>
+      <c r="J13" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="42" t="inlineStr">
+      <c r="K13" s="58" t="inlineStr">
         <is>
           <t>Weld cell</t>
         </is>
       </c>
-      <c r="L13" s="44">
+      <c r="L13" s="60">
         <f>Assumptions!$B$29</f>
         <v/>
       </c>
-      <c r="M13" s="36" t="n">
+      <c r="M13" s="52" t="n">
         <v>60</v>
       </c>
-      <c r="N13" s="37" t="n">
+      <c r="N13" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="O13" s="43">
+      <c r="O13" s="59">
         <f>M13*L13/3600/N13</f>
         <v/>
       </c>
-      <c r="P13" s="37" t="n">
+      <c r="P13" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="Q13" s="44">
+      <c r="Q13" s="60">
         <f>Assumptions!$B$34</f>
         <v/>
       </c>
-      <c r="R13" s="43">
+      <c r="R13" s="59">
         <f>M13*P13*Q13/3600/N13</f>
         <v/>
       </c>
-      <c r="S13" s="38" t="n">
+      <c r="S13" s="54" t="n">
         <v>1500000</v>
       </c>
-      <c r="T13" s="43">
+      <c r="T13" s="59">
         <f>S13/(Assumptions!$B$4*Assumptions!$B$5*E13)</f>
         <v/>
       </c>
-      <c r="U13" s="43">
+      <c r="U13" s="59">
         <f>(O13+R13)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V13" s="43">
+      <c r="V13" s="59">
         <f>J13+O13+R13+T13+U13</f>
         <v/>
       </c>
-      <c r="W13" s="43">
+      <c r="W13" s="59">
         <f>V13*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X13" s="43">
+      <c r="X13" s="59">
         <f>(V13+W13)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y13" s="45">
+      <c r="Y13" s="61">
         <f>V13+W13+X13</f>
         <v/>
       </c>
-      <c r="Z13" s="45">
+      <c r="Z13" s="61">
         <f>Y13*E13</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="29" t="n">
+      <c r="A14" s="45" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="46" t="inlineStr">
         <is>
           <t>Side beam bracket LH+RH (crash-box)</t>
         </is>
       </c>
-      <c r="C14" s="31" t="inlineStr">
+      <c r="C14" s="47" t="inlineStr">
         <is>
           <t>Progressive stamping</t>
         </is>
       </c>
-      <c r="D14" s="31" t="inlineStr">
+      <c r="D14" s="47" t="inlineStr">
         <is>
           <t>HSS 590 sheet</t>
         </is>
       </c>
-      <c r="E14" s="29" t="n">
+      <c r="E14" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="32" t="n">
+      <c r="F14" s="48" t="n">
         <v>0.35</v>
       </c>
-      <c r="G14" s="33" t="n">
+      <c r="G14" s="49" t="n">
         <v>0.12</v>
       </c>
-      <c r="H14" s="34">
+      <c r="H14" s="50">
         <f>Assumptions!$B$15</f>
         <v/>
       </c>
-      <c r="I14" s="34">
+      <c r="I14" s="50">
         <f>Assumptions!$B$16</f>
         <v/>
       </c>
-      <c r="J14" s="34">
+      <c r="J14" s="50">
         <f>F14*(1+G14)*H14-F14*G14*I14</f>
         <v/>
       </c>
-      <c r="K14" s="31" t="inlineStr">
+      <c r="K14" s="47" t="inlineStr">
         <is>
           <t>Press 250T prog</t>
         </is>
       </c>
-      <c r="L14" s="35">
+      <c r="L14" s="51">
         <f>Assumptions!$B$27</f>
         <v/>
       </c>
-      <c r="M14" s="36" t="n">
+      <c r="M14" s="52" t="n">
         <v>12</v>
       </c>
-      <c r="N14" s="37" t="n">
+      <c r="N14" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="O14" s="34">
+      <c r="O14" s="50">
         <f>M14*L14/3600/N14</f>
         <v/>
       </c>
-      <c r="P14" s="37" t="n">
+      <c r="P14" s="53" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q14" s="35">
+      <c r="Q14" s="51">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R14" s="34">
+      <c r="R14" s="50">
         <f>M14*P14*Q14/3600/N14</f>
         <v/>
       </c>
-      <c r="S14" s="38" t="n">
+      <c r="S14" s="54" t="n">
         <v>2500000</v>
       </c>
-      <c r="T14" s="34">
+      <c r="T14" s="50">
         <f>S14/(Assumptions!$B$4*Assumptions!$B$5*E14)</f>
         <v/>
       </c>
-      <c r="U14" s="34">
+      <c r="U14" s="50">
         <f>(O14+R14)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V14" s="34">
+      <c r="V14" s="50">
         <f>J14+O14+R14+T14+U14</f>
         <v/>
       </c>
-      <c r="W14" s="34">
+      <c r="W14" s="50">
         <f>V14*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X14" s="34">
+      <c r="X14" s="50">
         <f>(V14+W14)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y14" s="39">
+      <c r="Y14" s="55">
         <f>V14+W14+X14</f>
         <v/>
       </c>
-      <c r="Z14" s="39">
+      <c r="Z14" s="55">
         <f>Y14*E14</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="40" t="n">
+      <c r="A15" s="56" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="41" t="inlineStr">
+      <c r="B15" s="57" t="inlineStr">
         <is>
           <t>Tow hook cover</t>
         </is>
       </c>
-      <c r="C15" s="42" t="inlineStr">
+      <c r="C15" s="58" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D15" s="42" t="inlineStr">
+      <c r="D15" s="58" t="inlineStr">
         <is>
           <t>PP</t>
         </is>
       </c>
-      <c r="E15" s="40" t="n">
+      <c r="E15" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="32" t="n">
+      <c r="F15" s="48" t="n">
         <v>0.05</v>
       </c>
-      <c r="G15" s="33" t="n">
+      <c r="G15" s="49" t="n">
         <v>0.04</v>
       </c>
-      <c r="H15" s="43">
+      <c r="H15" s="59">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="I15" s="43">
+      <c r="I15" s="59">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J15" s="43">
+      <c r="J15" s="59">
         <f>F15*(1+G15)*H15-F15*G15*I15</f>
         <v/>
       </c>
-      <c r="K15" s="42" t="inlineStr">
+      <c r="K15" s="58" t="inlineStr">
         <is>
           <t>IMM 150T</t>
         </is>
       </c>
-      <c r="L15" s="44">
+      <c r="L15" s="60">
         <f>Assumptions!$B$25</f>
         <v/>
       </c>
-      <c r="M15" s="36" t="n">
+      <c r="M15" s="52" t="n">
         <v>22</v>
       </c>
-      <c r="N15" s="37" t="n">
+      <c r="N15" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="O15" s="43">
+      <c r="O15" s="59">
         <f>M15*L15/3600/N15</f>
         <v/>
       </c>
-      <c r="P15" s="37" t="n">
+      <c r="P15" s="53" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q15" s="44">
+      <c r="Q15" s="60">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R15" s="43">
+      <c r="R15" s="59">
         <f>M15*P15*Q15/3600/N15</f>
         <v/>
       </c>
-      <c r="S15" s="38" t="n">
+      <c r="S15" s="54" t="n">
         <v>900000</v>
       </c>
-      <c r="T15" s="43">
+      <c r="T15" s="59">
         <f>S15/(Assumptions!$B$4*Assumptions!$B$5*E15)</f>
         <v/>
       </c>
-      <c r="U15" s="43">
+      <c r="U15" s="59">
         <f>(O15+R15)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V15" s="43">
+      <c r="V15" s="59">
         <f>J15+O15+R15+T15+U15</f>
         <v/>
       </c>
-      <c r="W15" s="43">
+      <c r="W15" s="59">
         <f>V15*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X15" s="43">
+      <c r="X15" s="59">
         <f>(V15+W15)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y15" s="45">
+      <c r="Y15" s="61">
         <f>V15+W15+X15</f>
         <v/>
       </c>
-      <c r="Z15" s="45">
+      <c r="Z15" s="61">
         <f>Y15*E15</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="29" t="n">
+      <c r="A16" s="45" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="30" t="inlineStr">
+      <c r="B16" s="46" t="inlineStr">
         <is>
           <t>Parking sensor holder</t>
         </is>
       </c>
-      <c r="C16" s="31" t="inlineStr">
+      <c r="C16" s="47" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D16" s="31" t="inlineStr">
+      <c r="D16" s="47" t="inlineStr">
         <is>
           <t>PP</t>
         </is>
       </c>
-      <c r="E16" s="29">
+      <c r="E16" s="45">
         <f>Assumptions!$B$44</f>
         <v/>
       </c>
-      <c r="F16" s="32" t="n">
+      <c r="F16" s="48" t="n">
         <v>0.02</v>
       </c>
-      <c r="G16" s="33" t="n">
+      <c r="G16" s="49" t="n">
         <v>0.04</v>
       </c>
-      <c r="H16" s="34">
+      <c r="H16" s="50">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="I16" s="34">
+      <c r="I16" s="50">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J16" s="34">
+      <c r="J16" s="50">
         <f>F16*(1+G16)*H16-F16*G16*I16</f>
         <v/>
       </c>
-      <c r="K16" s="31" t="inlineStr">
+      <c r="K16" s="47" t="inlineStr">
         <is>
           <t>IMM 150T</t>
         </is>
       </c>
-      <c r="L16" s="35">
+      <c r="L16" s="51">
         <f>Assumptions!$B$25</f>
         <v/>
       </c>
-      <c r="M16" s="36" t="n">
+      <c r="M16" s="52" t="n">
         <v>20</v>
       </c>
-      <c r="N16" s="37" t="n">
+      <c r="N16" s="53" t="n">
         <v>4</v>
       </c>
-      <c r="O16" s="34">
+      <c r="O16" s="50">
         <f>M16*L16/3600/N16</f>
         <v/>
       </c>
-      <c r="P16" s="37" t="n">
+      <c r="P16" s="53" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q16" s="35">
+      <c r="Q16" s="51">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R16" s="34">
+      <c r="R16" s="50">
         <f>M16*P16*Q16/3600/N16</f>
         <v/>
       </c>
-      <c r="S16" s="38" t="n">
+      <c r="S16" s="54" t="n">
         <v>1400000</v>
       </c>
-      <c r="T16" s="34">
+      <c r="T16" s="50">
         <f>S16/(Assumptions!$B$4*Assumptions!$B$5*E16)</f>
         <v/>
       </c>
-      <c r="U16" s="34">
+      <c r="U16" s="50">
         <f>(O16+R16)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V16" s="34">
+      <c r="V16" s="50">
         <f>J16+O16+R16+T16+U16</f>
         <v/>
       </c>
-      <c r="W16" s="34">
+      <c r="W16" s="50">
         <f>V16*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X16" s="34">
+      <c r="X16" s="50">
         <f>(V16+W16)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y16" s="39">
+      <c r="Y16" s="55">
         <f>V16+W16+X16</f>
         <v/>
       </c>
-      <c r="Z16" s="39">
+      <c r="Z16" s="55">
         <f>Y16*E16</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="40" t="n">
+      <c r="A17" s="56" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="41" t="inlineStr">
+      <c r="B17" s="57" t="inlineStr">
         <is>
           <t>Radar sensor bracket</t>
         </is>
       </c>
-      <c r="C17" s="42" t="inlineStr">
+      <c r="C17" s="58" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D17" s="42" t="inlineStr">
+      <c r="D17" s="58" t="inlineStr">
         <is>
           <t>PP</t>
         </is>
       </c>
-      <c r="E17" s="40" t="n">
+      <c r="E17" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="32" t="n">
+      <c r="F17" s="48" t="n">
         <v>0.08</v>
       </c>
-      <c r="G17" s="33" t="n">
+      <c r="G17" s="49" t="n">
         <v>0.04</v>
       </c>
-      <c r="H17" s="43">
+      <c r="H17" s="59">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="I17" s="43">
+      <c r="I17" s="59">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J17" s="43">
+      <c r="J17" s="59">
         <f>F17*(1+G17)*H17-F17*G17*I17</f>
         <v/>
       </c>
-      <c r="K17" s="42" t="inlineStr">
+      <c r="K17" s="58" t="inlineStr">
         <is>
           <t>IMM 150T</t>
         </is>
       </c>
-      <c r="L17" s="44">
+      <c r="L17" s="60">
         <f>Assumptions!$B$25</f>
         <v/>
       </c>
-      <c r="M17" s="36" t="n">
+      <c r="M17" s="52" t="n">
         <v>25</v>
       </c>
-      <c r="N17" s="37" t="n">
+      <c r="N17" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="O17" s="43">
+      <c r="O17" s="59">
         <f>M17*L17/3600/N17</f>
         <v/>
       </c>
-      <c r="P17" s="37" t="n">
+      <c r="P17" s="53" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q17" s="44">
+      <c r="Q17" s="60">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R17" s="43">
+      <c r="R17" s="59">
         <f>M17*P17*Q17/3600/N17</f>
         <v/>
       </c>
-      <c r="S17" s="38" t="n">
+      <c r="S17" s="54" t="n">
         <v>1100000</v>
       </c>
-      <c r="T17" s="43">
+      <c r="T17" s="59">
         <f>S17/(Assumptions!$B$4*Assumptions!$B$5*E17)</f>
         <v/>
       </c>
-      <c r="U17" s="43">
+      <c r="U17" s="59">
         <f>(O17+R17)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V17" s="43">
+      <c r="V17" s="59">
         <f>J17+O17+R17+T17+U17</f>
         <v/>
       </c>
-      <c r="W17" s="43">
+      <c r="W17" s="59">
         <f>V17*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X17" s="43">
+      <c r="X17" s="59">
         <f>(V17+W17)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y17" s="45">
+      <c r="Y17" s="61">
         <f>V17+W17+X17</f>
         <v/>
       </c>
-      <c r="Z17" s="45">
+      <c r="Z17" s="61">
         <f>Y17*E17</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="29" t="n">
+      <c r="A18" s="45" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="30" t="inlineStr">
+      <c r="B18" s="46" t="inlineStr">
         <is>
           <t>Camera mount bracket</t>
         </is>
       </c>
-      <c r="C18" s="31" t="inlineStr">
+      <c r="C18" s="47" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D18" s="31" t="inlineStr">
+      <c r="D18" s="47" t="inlineStr">
         <is>
           <t>PP</t>
         </is>
       </c>
-      <c r="E18" s="29" t="n">
+      <c r="E18" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="F18" s="32" t="n">
+      <c r="F18" s="48" t="n">
         <v>0.05</v>
       </c>
-      <c r="G18" s="33" t="n">
+      <c r="G18" s="49" t="n">
         <v>0.04</v>
       </c>
-      <c r="H18" s="34">
+      <c r="H18" s="50">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="I18" s="34">
+      <c r="I18" s="50">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J18" s="34">
+      <c r="J18" s="50">
         <f>F18*(1+G18)*H18-F18*G18*I18</f>
         <v/>
       </c>
-      <c r="K18" s="31" t="inlineStr">
+      <c r="K18" s="47" t="inlineStr">
         <is>
           <t>IMM 150T</t>
         </is>
       </c>
-      <c r="L18" s="35">
+      <c r="L18" s="51">
         <f>Assumptions!$B$25</f>
         <v/>
       </c>
-      <c r="M18" s="36" t="n">
+      <c r="M18" s="52" t="n">
         <v>22</v>
       </c>
-      <c r="N18" s="37" t="n">
+      <c r="N18" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="O18" s="34">
+      <c r="O18" s="50">
         <f>M18*L18/3600/N18</f>
         <v/>
       </c>
-      <c r="P18" s="37" t="n">
+      <c r="P18" s="53" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q18" s="35">
+      <c r="Q18" s="51">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R18" s="34">
+      <c r="R18" s="50">
         <f>M18*P18*Q18/3600/N18</f>
         <v/>
       </c>
-      <c r="S18" s="38" t="n">
+      <c r="S18" s="54" t="n">
         <v>900000</v>
       </c>
-      <c r="T18" s="34">
+      <c r="T18" s="50">
         <f>S18/(Assumptions!$B$4*Assumptions!$B$5*E18)</f>
         <v/>
       </c>
-      <c r="U18" s="34">
+      <c r="U18" s="50">
         <f>(O18+R18)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V18" s="34">
+      <c r="V18" s="50">
         <f>J18+O18+R18+T18+U18</f>
         <v/>
       </c>
-      <c r="W18" s="34">
+      <c r="W18" s="50">
         <f>V18*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X18" s="34">
+      <c r="X18" s="50">
         <f>(V18+W18)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y18" s="39">
+      <c r="Y18" s="55">
         <f>V18+W18+X18</f>
         <v/>
       </c>
-      <c r="Z18" s="39">
+      <c r="Z18" s="55">
         <f>Y18*E18</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="40" t="n">
+      <c r="A19" s="56" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="41" t="inlineStr">
+      <c r="B19" s="57" t="inlineStr">
         <is>
           <t>Air deflector</t>
         </is>
       </c>
-      <c r="C19" s="42" t="inlineStr">
+      <c r="C19" s="58" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D19" s="42" t="inlineStr">
+      <c r="D19" s="58" t="inlineStr">
         <is>
           <t>PP</t>
         </is>
       </c>
-      <c r="E19" s="40" t="n">
+      <c r="E19" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="32" t="n">
+      <c r="F19" s="48" t="n">
         <v>0.45</v>
       </c>
-      <c r="G19" s="33" t="n">
+      <c r="G19" s="49" t="n">
         <v>0.05</v>
       </c>
-      <c r="H19" s="43">
+      <c r="H19" s="59">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="I19" s="43">
+      <c r="I19" s="59">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J19" s="43">
+      <c r="J19" s="59">
         <f>F19*(1+G19)*H19-F19*G19*I19</f>
         <v/>
       </c>
-      <c r="K19" s="42" t="inlineStr">
+      <c r="K19" s="58" t="inlineStr">
         <is>
           <t>IMM 450T</t>
         </is>
       </c>
-      <c r="L19" s="44">
+      <c r="L19" s="60">
         <f>Assumptions!$B$23</f>
         <v/>
       </c>
-      <c r="M19" s="36" t="n">
+      <c r="M19" s="52" t="n">
         <v>36</v>
       </c>
-      <c r="N19" s="37" t="n">
+      <c r="N19" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="O19" s="43">
+      <c r="O19" s="59">
         <f>M19*L19/3600/N19</f>
         <v/>
       </c>
-      <c r="P19" s="37" t="n">
+      <c r="P19" s="53" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q19" s="44">
+      <c r="Q19" s="60">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R19" s="43">
+      <c r="R19" s="59">
         <f>M19*P19*Q19/3600/N19</f>
         <v/>
       </c>
-      <c r="S19" s="38" t="n">
+      <c r="S19" s="54" t="n">
         <v>3200000</v>
       </c>
-      <c r="T19" s="43">
+      <c r="T19" s="59">
         <f>S19/(Assumptions!$B$4*Assumptions!$B$5*E19)</f>
         <v/>
       </c>
-      <c r="U19" s="43">
+      <c r="U19" s="59">
         <f>(O19+R19)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V19" s="43">
+      <c r="V19" s="59">
         <f>J19+O19+R19+T19+U19</f>
         <v/>
       </c>
-      <c r="W19" s="43">
+      <c r="W19" s="59">
         <f>V19*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X19" s="43">
+      <c r="X19" s="59">
         <f>(V19+W19)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y19" s="45">
+      <c r="Y19" s="61">
         <f>V19+W19+X19</f>
         <v/>
       </c>
-      <c r="Z19" s="45">
+      <c r="Z19" s="61">
         <f>Y19*E19</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="29" t="n">
+      <c r="A20" s="45" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="30" t="inlineStr">
+      <c r="B20" s="46" t="inlineStr">
         <is>
           <t>Wheel-arch retainer LH+RH</t>
         </is>
       </c>
-      <c r="C20" s="31" t="inlineStr">
+      <c r="C20" s="47" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D20" s="31" t="inlineStr">
+      <c r="D20" s="47" t="inlineStr">
         <is>
           <t>PP</t>
         </is>
       </c>
-      <c r="E20" s="29" t="n">
+      <c r="E20" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="F20" s="32" t="n">
+      <c r="F20" s="48" t="n">
         <v>0.15</v>
       </c>
-      <c r="G20" s="33" t="n">
+      <c r="G20" s="49" t="n">
         <v>0.04</v>
       </c>
-      <c r="H20" s="34">
+      <c r="H20" s="50">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="I20" s="34">
+      <c r="I20" s="50">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J20" s="34">
+      <c r="J20" s="50">
         <f>F20*(1+G20)*H20-F20*G20*I20</f>
         <v/>
       </c>
-      <c r="K20" s="31" t="inlineStr">
+      <c r="K20" s="47" t="inlineStr">
         <is>
           <t>IMM 250T</t>
         </is>
       </c>
-      <c r="L20" s="35">
+      <c r="L20" s="51">
         <f>Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="M20" s="36" t="n">
+      <c r="M20" s="52" t="n">
         <v>30</v>
       </c>
-      <c r="N20" s="37" t="n">
+      <c r="N20" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="O20" s="34">
+      <c r="O20" s="50">
         <f>M20*L20/3600/N20</f>
         <v/>
       </c>
-      <c r="P20" s="37" t="n">
+      <c r="P20" s="53" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q20" s="35">
+      <c r="Q20" s="51">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R20" s="34">
+      <c r="R20" s="50">
         <f>M20*P20*Q20/3600/N20</f>
         <v/>
       </c>
-      <c r="S20" s="38" t="n">
+      <c r="S20" s="54" t="n">
         <v>1600000</v>
       </c>
-      <c r="T20" s="34">
+      <c r="T20" s="50">
         <f>S20/(Assumptions!$B$4*Assumptions!$B$5*E20)</f>
         <v/>
       </c>
-      <c r="U20" s="34">
+      <c r="U20" s="50">
         <f>(O20+R20)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V20" s="34">
+      <c r="V20" s="50">
         <f>J20+O20+R20+T20+U20</f>
         <v/>
       </c>
-      <c r="W20" s="34">
+      <c r="W20" s="50">
         <f>V20*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X20" s="34">
+      <c r="X20" s="50">
         <f>(V20+W20)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y20" s="39">
+      <c r="Y20" s="55">
         <f>V20+W20+X20</f>
         <v/>
       </c>
-      <c r="Z20" s="39">
+      <c r="Z20" s="55">
         <f>Y20*E20</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="40" t="n">
+      <c r="A21" s="56" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="41" t="inlineStr">
+      <c r="B21" s="57" t="inlineStr">
         <is>
           <t>Side support bracket LH+RH</t>
         </is>
       </c>
-      <c r="C21" s="42" t="inlineStr">
+      <c r="C21" s="58" t="inlineStr">
         <is>
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D21" s="42" t="inlineStr">
+      <c r="D21" s="58" t="inlineStr">
         <is>
           <t>PP</t>
         </is>
       </c>
-      <c r="E21" s="40" t="n">
+      <c r="E21" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="32" t="n">
+      <c r="F21" s="48" t="n">
         <v>0.15</v>
       </c>
-      <c r="G21" s="33" t="n">
+      <c r="G21" s="49" t="n">
         <v>0.04</v>
       </c>
-      <c r="H21" s="43">
+      <c r="H21" s="59">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="I21" s="43">
+      <c r="I21" s="59">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="J21" s="43">
+      <c r="J21" s="59">
         <f>F21*(1+G21)*H21-F21*G21*I21</f>
         <v/>
       </c>
-      <c r="K21" s="42" t="inlineStr">
+      <c r="K21" s="58" t="inlineStr">
         <is>
           <t>IMM 250T</t>
         </is>
       </c>
-      <c r="L21" s="44">
+      <c r="L21" s="60">
         <f>Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="M21" s="36" t="n">
+      <c r="M21" s="52" t="n">
         <v>30</v>
       </c>
-      <c r="N21" s="37" t="n">
+      <c r="N21" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="O21" s="43">
+      <c r="O21" s="59">
         <f>M21*L21/3600/N21</f>
         <v/>
       </c>
-      <c r="P21" s="37" t="n">
+      <c r="P21" s="53" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q21" s="44">
+      <c r="Q21" s="60">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="R21" s="43">
+      <c r="R21" s="59">
         <f>M21*P21*Q21/3600/N21</f>
         <v/>
       </c>
-      <c r="S21" s="38" t="n">
+      <c r="S21" s="54" t="n">
         <v>1600000</v>
       </c>
-      <c r="T21" s="43">
+      <c r="T21" s="59">
         <f>S21/(Assumptions!$B$4*Assumptions!$B$5*E21)</f>
         <v/>
       </c>
-      <c r="U21" s="43">
+      <c r="U21" s="59">
         <f>(O21+R21)*Assumptions!$B$38</f>
         <v/>
       </c>
-      <c r="V21" s="43">
+      <c r="V21" s="59">
         <f>J21+O21+R21+T21+U21</f>
         <v/>
       </c>
-      <c r="W21" s="43">
+      <c r="W21" s="59">
         <f>V21*Assumptions!$B$39</f>
         <v/>
       </c>
-      <c r="X21" s="43">
+      <c r="X21" s="59">
         <f>(V21+W21)*Assumptions!$B$40</f>
         <v/>
       </c>
-      <c r="Y21" s="45">
+      <c r="Y21" s="61">
         <f>V21+W21+X21</f>
         <v/>
       </c>
-      <c r="Z21" s="45">
+      <c r="Z21" s="61">
         <f>Y21*E21</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="46" t="n"/>
-      <c r="B22" s="46" t="inlineStr">
+      <c r="A22" s="62" t="n"/>
+      <c r="B22" s="62" t="inlineStr">
         <is>
           <t>MANUFACTURED PARTS — TOTAL PER VEHICLE</t>
         </is>
       </c>
-      <c r="C22" s="46" t="n"/>
-      <c r="D22" s="46" t="n"/>
-      <c r="E22" s="46" t="n"/>
-      <c r="F22" s="46" t="n"/>
-      <c r="G22" s="46" t="n"/>
-      <c r="H22" s="46" t="n"/>
-      <c r="I22" s="46" t="n"/>
-      <c r="J22" s="46" t="n"/>
-      <c r="K22" s="46" t="n"/>
-      <c r="L22" s="46" t="n"/>
-      <c r="M22" s="46" t="n"/>
-      <c r="N22" s="46" t="n"/>
-      <c r="O22" s="46" t="n"/>
-      <c r="P22" s="46" t="n"/>
-      <c r="Q22" s="46" t="n"/>
-      <c r="R22" s="46" t="n"/>
-      <c r="S22" s="47">
+      <c r="C22" s="62" t="n"/>
+      <c r="D22" s="62" t="n"/>
+      <c r="E22" s="62" t="n"/>
+      <c r="F22" s="62" t="n"/>
+      <c r="G22" s="62" t="n"/>
+      <c r="H22" s="62" t="n"/>
+      <c r="I22" s="62" t="n"/>
+      <c r="J22" s="62" t="n"/>
+      <c r="K22" s="62" t="n"/>
+      <c r="L22" s="62" t="n"/>
+      <c r="M22" s="62" t="n"/>
+      <c r="N22" s="62" t="n"/>
+      <c r="O22" s="62" t="n"/>
+      <c r="P22" s="62" t="n"/>
+      <c r="Q22" s="62" t="n"/>
+      <c r="R22" s="62" t="n"/>
+      <c r="S22" s="63">
         <f>SUM(S4:S21)</f>
         <v/>
       </c>
-      <c r="T22" s="46" t="n"/>
-      <c r="U22" s="46" t="n"/>
-      <c r="V22" s="46" t="n"/>
-      <c r="W22" s="46" t="n"/>
-      <c r="X22" s="46" t="n"/>
-      <c r="Y22" s="46" t="n"/>
-      <c r="Z22" s="48">
+      <c r="T22" s="62" t="n"/>
+      <c r="U22" s="62" t="n"/>
+      <c r="V22" s="62" t="n"/>
+      <c r="W22" s="62" t="n"/>
+      <c r="X22" s="62" t="n"/>
+      <c r="Y22" s="62" t="n"/>
+      <c r="Z22" s="64">
         <f>SUM(Z4:Z21)</f>
         <v/>
       </c>
@@ -3837,7 +4507,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3907,232 +4577,232 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="49" t="n">
+      <c r="A4" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="50" t="inlineStr">
+      <c r="B4" s="66" t="inlineStr">
         <is>
           <t>Ultrasonic parking sensor</t>
         </is>
       </c>
-      <c r="C4" s="50" t="inlineStr">
+      <c r="C4" s="66" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="D4" s="49">
+      <c r="D4" s="65">
         <f>Assumptions!$B$44</f>
         <v/>
       </c>
-      <c r="E4" s="51" t="n">
+      <c r="E4" s="67" t="n">
         <v>380</v>
       </c>
-      <c r="F4" s="52">
+      <c r="F4" s="68">
         <f>E4*Assumptions!$B$41</f>
         <v/>
       </c>
-      <c r="G4" s="52">
+      <c r="G4" s="68">
         <f>(E4+F4)*D4</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="49" t="n">
+      <c r="A5" s="65" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="50" t="inlineStr">
+      <c r="B5" s="66" t="inlineStr">
         <is>
           <t>Front radar sensor (77 GHz)</t>
         </is>
       </c>
-      <c r="C5" s="50" t="inlineStr">
+      <c r="C5" s="66" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="D5" s="49" t="n">
+      <c r="D5" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="51" t="n">
+      <c r="E5" s="67" t="n">
         <v>5800</v>
       </c>
-      <c r="F5" s="52">
+      <c r="F5" s="68">
         <f>E5*Assumptions!$B$41</f>
         <v/>
       </c>
-      <c r="G5" s="52">
+      <c r="G5" s="68">
         <f>(E5+F5)*D5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="49" t="n">
+      <c r="A6" s="65" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="50" t="inlineStr">
+      <c r="B6" s="66" t="inlineStr">
         <is>
           <t>Front camera module</t>
         </is>
       </c>
-      <c r="C6" s="50" t="inlineStr">
+      <c r="C6" s="66" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="D6" s="49" t="n">
+      <c r="D6" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="51" t="n">
+      <c r="E6" s="67" t="n">
         <v>2200</v>
       </c>
-      <c r="F6" s="52">
+      <c r="F6" s="68">
         <f>E6*Assumptions!$B$41</f>
         <v/>
       </c>
-      <c r="G6" s="52">
+      <c r="G6" s="68">
         <f>(E6+F6)*D6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="49" t="n">
+      <c r="A7" s="65" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="50" t="inlineStr">
+      <c r="B7" s="66" t="inlineStr">
         <is>
           <t>Bumper wiring harness</t>
         </is>
       </c>
-      <c r="C7" s="50" t="inlineStr">
+      <c r="C7" s="66" t="inlineStr">
         <is>
           <t>Electrical</t>
         </is>
       </c>
-      <c r="D7" s="49" t="n">
+      <c r="D7" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="51" t="n">
+      <c r="E7" s="67" t="n">
         <v>520</v>
       </c>
-      <c r="F7" s="52">
+      <c r="F7" s="68">
         <f>E7*Assumptions!$B$41</f>
         <v/>
       </c>
-      <c r="G7" s="52">
+      <c r="G7" s="68">
         <f>(E7+F7)*D7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="49" t="n">
+      <c r="A8" s="65" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="50" t="inlineStr">
+      <c r="B8" s="66" t="inlineStr">
         <is>
           <t>Clips &amp; fasteners set (push clips, u-nuts, spring nuts)</t>
         </is>
       </c>
-      <c r="C8" s="50" t="inlineStr">
+      <c r="C8" s="66" t="inlineStr">
         <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="D8" s="49" t="n">
+      <c r="D8" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="51" t="n">
+      <c r="E8" s="67" t="n">
         <v>95</v>
       </c>
-      <c r="F8" s="52">
+      <c r="F8" s="68">
         <f>E8*Assumptions!$B$41</f>
         <v/>
       </c>
-      <c r="G8" s="52">
+      <c r="G8" s="68">
         <f>(E8+F8)*D8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="49" t="n">
+      <c r="A9" s="65" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="50" t="inlineStr">
+      <c r="B9" s="66" t="inlineStr">
         <is>
           <t>Bolts M8/M10 set</t>
         </is>
       </c>
-      <c r="C9" s="50" t="inlineStr">
+      <c r="C9" s="66" t="inlineStr">
         <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="D9" s="49" t="n">
+      <c r="D9" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="51" t="n">
+      <c r="E9" s="67" t="n">
         <v>28</v>
       </c>
-      <c r="F9" s="52">
+      <c r="F9" s="68">
         <f>E9*Assumptions!$B$41</f>
         <v/>
       </c>
-      <c r="G9" s="52">
+      <c r="G9" s="68">
         <f>(E9+F9)*D9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="49" t="n">
+      <c r="A10" s="65" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="50" t="inlineStr">
+      <c r="B10" s="66" t="inlineStr">
         <is>
           <t>Nuts &amp; washers set</t>
         </is>
       </c>
-      <c r="C10" s="50" t="inlineStr">
+      <c r="C10" s="66" t="inlineStr">
         <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="D10" s="49" t="n">
+      <c r="D10" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="51" t="n">
+      <c r="E10" s="67" t="n">
         <v>20</v>
       </c>
-      <c r="F10" s="52">
+      <c r="F10" s="68">
         <f>E10*Assumptions!$B$41</f>
         <v/>
       </c>
-      <c r="G10" s="52">
+      <c r="G10" s="68">
         <f>(E10+F10)*D10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="46" t="n"/>
-      <c r="B11" s="46" t="inlineStr">
+      <c r="A11" s="62" t="n"/>
+      <c r="B11" s="62" t="inlineStr">
         <is>
           <t>BOUGHT-OUT — TOTAL PER VEHICLE</t>
         </is>
       </c>
-      <c r="C11" s="46" t="n"/>
-      <c r="D11" s="46" t="n"/>
-      <c r="E11" s="46" t="n"/>
-      <c r="F11" s="46" t="n"/>
-      <c r="G11" s="48">
+      <c r="C11" s="62" t="n"/>
+      <c r="D11" s="62" t="n"/>
+      <c r="E11" s="62" t="n"/>
+      <c r="F11" s="62" t="n"/>
+      <c r="G11" s="64">
         <f>SUM(G4:G10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="53" t="inlineStr">
+      <c r="B12" s="69" t="inlineStr">
         <is>
           <t xml:space="preserve">   of which electronics (sensors + radar + camera + harness)</t>
         </is>
       </c>
-      <c r="G12" s="54">
+      <c r="G12" s="70">
         <f>SUM(G4:G7)</f>
         <v/>
       </c>
@@ -4146,7 +4816,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4216,286 +4886,286 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="55" t="n">
+      <c r="A4" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="56" t="inlineStr">
+      <c r="B4" s="72" t="inlineStr">
         <is>
           <t>Beam sub-assembly: energy absorber + crash brackets to beam</t>
         </is>
       </c>
-      <c r="C4" s="57" t="n">
+      <c r="C4" s="73" t="n">
         <v>60</v>
       </c>
-      <c r="D4" s="58" t="n">
+      <c r="D4" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="59">
+      <c r="E4" s="75">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="F4" s="60">
+      <c r="F4" s="76">
         <f>C4*D4*E4/3600</f>
         <v/>
       </c>
-      <c r="G4" s="56" t="inlineStr">
+      <c r="G4" s="72" t="inlineStr">
         <is>
           <t>Bolted, torque-monitored</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="55" t="n">
+      <c r="A5" s="71" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="56" t="inlineStr">
+      <c r="B5" s="72" t="inlineStr">
         <is>
           <t>Fascia dress: grilles, bezels, number-plate bracket, tow cover</t>
         </is>
       </c>
-      <c r="C5" s="57" t="n">
+      <c r="C5" s="73" t="n">
         <v>120</v>
       </c>
-      <c r="D5" s="58" t="n">
+      <c r="D5" s="74" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="59">
+      <c r="E5" s="75">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="F5" s="60">
+      <c r="F5" s="76">
         <f>C5*D5*E5/3600</f>
         <v/>
       </c>
-      <c r="G5" s="56" t="inlineStr">
+      <c r="G5" s="72" t="inlineStr">
         <is>
           <t>Clip-fit + screw stations</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="55" t="n">
+      <c r="A6" s="71" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="56" t="inlineStr">
+      <c r="B6" s="72" t="inlineStr">
         <is>
           <t>Harness routing, parking sensors, radar &amp; camera fit</t>
         </is>
       </c>
-      <c r="C6" s="57" t="n">
+      <c r="C6" s="73" t="n">
         <v>150</v>
       </c>
-      <c r="D6" s="58" t="n">
+      <c r="D6" s="74" t="n">
         <v>1.5</v>
       </c>
-      <c r="E6" s="59">
+      <c r="E6" s="75">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="F6" s="60">
+      <c r="F6" s="76">
         <f>C6*D6*E6/3600</f>
         <v/>
       </c>
-      <c r="G6" s="56" t="inlineStr">
+      <c r="G6" s="72" t="inlineStr">
         <is>
           <t>Connector click-checks</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="55" t="n">
+      <c r="A7" s="71" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="56" t="inlineStr">
+      <c r="B7" s="72" t="inlineStr">
         <is>
           <t>Air deflector, wheel-arch retainers, side supports</t>
         </is>
       </c>
-      <c r="C7" s="57" t="n">
+      <c r="C7" s="73" t="n">
         <v>75</v>
       </c>
-      <c r="D7" s="58" t="n">
+      <c r="D7" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="59">
+      <c r="E7" s="75">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="F7" s="60">
+      <c r="F7" s="76">
         <f>C7*D7*E7/3600</f>
         <v/>
       </c>
-      <c r="G7" s="56" t="inlineStr"/>
+      <c r="G7" s="72" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="55" t="n">
+      <c r="A8" s="71" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="56" t="inlineStr">
+      <c r="B8" s="72" t="inlineStr">
         <is>
           <t>End-of-line inspection &amp; torque verification</t>
         </is>
       </c>
-      <c r="C8" s="57" t="n">
+      <c r="C8" s="73" t="n">
         <v>60</v>
       </c>
-      <c r="D8" s="58" t="n">
+      <c r="D8" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="59">
+      <c r="E8" s="75">
         <f>Assumptions!$B$35</f>
         <v/>
       </c>
-      <c r="F8" s="60">
+      <c r="F8" s="76">
         <f>C8*D8*E8/3600</f>
         <v/>
       </c>
-      <c r="G8" s="56" t="inlineStr">
+      <c r="G8" s="72" t="inlineStr">
         <is>
           <t>Poka-yoke checklist</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="55" t="n">
+      <c r="A9" s="71" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="56" t="inlineStr">
+      <c r="B9" s="72" t="inlineStr">
         <is>
           <t>Pack into returnable dunnage</t>
         </is>
       </c>
-      <c r="C9" s="57" t="n">
+      <c r="C9" s="73" t="n">
         <v>45</v>
       </c>
-      <c r="D9" s="58" t="n">
+      <c r="D9" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="59">
+      <c r="E9" s="75">
         <f>Assumptions!$B$33</f>
         <v/>
       </c>
-      <c r="F9" s="60">
+      <c r="F9" s="76">
         <f>C9*D9*E9/3600</f>
         <v/>
       </c>
-      <c r="G9" s="56" t="inlineStr"/>
+      <c r="G9" s="72" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="B11" s="61" t="inlineStr">
+      <c r="B11" s="77" t="inlineStr">
         <is>
           <t>Assembly labour subtotal</t>
         </is>
       </c>
-      <c r="C11" s="62" t="n"/>
-      <c r="D11" s="62" t="n"/>
-      <c r="E11" s="62" t="n"/>
-      <c r="F11" s="63">
+      <c r="C11" s="29" t="n"/>
+      <c r="D11" s="29" t="n"/>
+      <c r="E11" s="29" t="n"/>
+      <c r="F11" s="78">
         <f>SUM(F4:F9)</f>
         <v/>
       </c>
-      <c r="G11" s="64" t="inlineStr"/>
+      <c r="G11" s="79" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="B12" s="61" t="inlineStr">
+      <c r="B12" s="77" t="inlineStr">
         <is>
           <t>Fixtures &amp; jigs amortisation (₹40 L over volume × years)</t>
         </is>
       </c>
-      <c r="C12" s="62" t="n"/>
-      <c r="D12" s="62" t="n"/>
-      <c r="E12" s="62" t="n"/>
-      <c r="F12" s="63">
+      <c r="C12" s="29" t="n"/>
+      <c r="D12" s="29" t="n"/>
+      <c r="E12" s="29" t="n"/>
+      <c r="F12" s="78">
         <f>4000000/(Assumptions!$B$4*Assumptions!$B$5)</f>
         <v/>
       </c>
-      <c r="G12" s="64" t="inlineStr">
+      <c r="G12" s="79" t="inlineStr">
         <is>
           <t>Assembly fixtures, torque tools mounting</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="61" t="inlineStr">
+      <c r="B13" s="77" t="inlineStr">
         <is>
           <t>Equipment amortisation (EOL tester, torque tools — ₹60 L)</t>
         </is>
       </c>
-      <c r="C13" s="62" t="n"/>
-      <c r="D13" s="62" t="n"/>
-      <c r="E13" s="62" t="n"/>
-      <c r="F13" s="63">
+      <c r="C13" s="29" t="n"/>
+      <c r="D13" s="29" t="n"/>
+      <c r="E13" s="29" t="n"/>
+      <c r="F13" s="78">
         <f>6000000/(Assumptions!$B$4*Assumptions!$B$5)</f>
         <v/>
       </c>
-      <c r="G13" s="64" t="inlineStr"/>
+      <c r="G13" s="79" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="B14" s="61" t="inlineStr">
+      <c r="B14" s="77" t="inlineStr">
         <is>
           <t>Consumables per unit</t>
         </is>
       </c>
-      <c r="C14" s="62" t="n"/>
-      <c r="D14" s="62" t="n"/>
-      <c r="E14" s="62" t="n"/>
-      <c r="F14" s="65" t="n">
+      <c r="C14" s="29" t="n"/>
+      <c r="D14" s="29" t="n"/>
+      <c r="E14" s="29" t="n"/>
+      <c r="F14" s="80" t="n">
         <v>6</v>
       </c>
-      <c r="G14" s="64" t="inlineStr">
+      <c r="G14" s="79" t="inlineStr">
         <is>
           <t>Tapes, primers, gloves</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="61" t="inlineStr">
+      <c r="B15" s="77" t="inlineStr">
         <is>
           <t>Assembly overhead</t>
         </is>
       </c>
-      <c r="C15" s="62" t="n"/>
-      <c r="D15" s="62" t="n"/>
-      <c r="E15" s="62" t="n"/>
-      <c r="F15" s="63">
+      <c r="C15" s="29" t="n"/>
+      <c r="D15" s="29" t="n"/>
+      <c r="E15" s="29" t="n"/>
+      <c r="F15" s="78">
         <f>F11*Assumptions!$B$42</f>
         <v/>
       </c>
-      <c r="G15" s="64" t="inlineStr">
+      <c r="G15" s="79" t="inlineStr">
         <is>
           <t>On labour subtotal — rate from Assumptions</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="61" t="inlineStr">
+      <c r="B16" s="77" t="inlineStr">
         <is>
           <t>Packaging (returnable dunnage trip cost)</t>
         </is>
       </c>
-      <c r="C16" s="62" t="n"/>
-      <c r="D16" s="62" t="n"/>
-      <c r="E16" s="62" t="n"/>
-      <c r="F16" s="63">
+      <c r="C16" s="29" t="n"/>
+      <c r="D16" s="29" t="n"/>
+      <c r="E16" s="29" t="n"/>
+      <c r="F16" s="78">
         <f>Assumptions!$B$43</f>
         <v/>
       </c>
-      <c r="G16" s="64" t="inlineStr"/>
+      <c r="G16" s="79" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="B17" s="66" t="inlineStr">
+      <c r="B17" s="81" t="inlineStr">
         <is>
           <t>ASSEMBLY &amp; PACKING — TOTAL PER VEHICLE</t>
         </is>
       </c>
-      <c r="C17" s="66" t="n"/>
-      <c r="D17" s="66" t="n"/>
-      <c r="E17" s="66" t="n"/>
-      <c r="F17" s="67">
+      <c r="C17" s="81" t="n"/>
+      <c r="D17" s="81" t="n"/>
+      <c r="E17" s="81" t="n"/>
+      <c r="F17" s="82">
         <f>SUM(F11:F16)</f>
         <v/>
       </c>
-      <c r="G17" s="66" t="n"/>
+      <c r="G17" s="81" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4506,7 +5176,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4546,54 +5216,54 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="62" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Part tooling total (moulds, dies, fixtures)</t>
         </is>
       </c>
-      <c r="B4" s="68">
+      <c r="B4" s="83">
         <f>'Parts Costing'!S22</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="62" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>Assembly fixtures &amp; jigs</t>
         </is>
       </c>
-      <c r="B5" s="68" t="n">
+      <c r="B5" s="83" t="n">
         <v>4000000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="62" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Assembly equipment (EOL, torque)</t>
         </is>
       </c>
-      <c r="B6" s="68" t="n">
+      <c r="B6" s="83" t="n">
         <v>6000000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="69" t="inlineStr">
+      <c r="A7" s="84" t="inlineStr">
         <is>
           <t>TOTAL ONE-TIME INVESTMENT</t>
         </is>
       </c>
-      <c r="B7" s="70">
+      <c r="B7" s="85">
         <f>SUM(B4:B6)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="71" t="inlineStr">
+      <c r="A9" s="86" t="inlineStr">
         <is>
           <t>In ₹ Crore</t>
         </is>
       </c>
-      <c r="B9" s="72">
+      <c r="B9" s="87">
         <f>B7/10000000</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Bumper should-cost: refresh Methodology & Q&A to the re-audited model
Narrative text updated to current inputs (fascia 3.60 kg / 55 s / 1.8 Cr
tool, total 8.7k with electronics ~71%, painted fascia 1,078, beam 442,
paint 338 at 2,400/hr line, tooling 50->100 volume example, VA/VE levers
338/37) and the cheaper-part answer now cites the Summary savings table
with its live total pulled by formula. All worked-example cells verified
current after recalculation.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142L4rKS2AV8rxQTDWMs7dy
</commit_message>
<xml_diff>
--- a/Altroz-Front-Bumper-Should-Cost-India.xlsx
+++ b/Altroz-Front-Bumper-Should-Cost-India.xlsx
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="351">
   <si>
     <t xml:space="preserve">TATA ALTROZ — FRONT BUMPER ASSEMBLY  ·  SHOULD-COST SUMMARY (INDIA)</t>
   </si>
@@ -323,7 +323,7 @@
     <t xml:space="preserve">Material cost per part</t>
   </si>
   <si>
-    <t xml:space="preserve">Net part mass × (1 + scrap%) × material price ₹/kg, minus scrap credit for the recoverable portion.  Formula in words: you buy slightly more plastic/steel than ends up in the part (runners, offal), and sell back what you can.  Excel: =Mass×(1+Scrap)×Price − Mass×Scrap×Credit  →  Fascia: 4.20 kg TPO at ₹142/kg with 4% runner scrap.</t>
+    <t xml:space="preserve">Net part mass × (1 + scrap%) × material price ₹/kg, minus scrap credit for the recoverable portion.  Formula in words: you buy slightly more plastic/steel than ends up in the part (runners, offal), and sell back what you can.  Excel: =Mass×(1+Scrap)×Price − Mass×Scrap×Credit  →  Fascia: 3.60 kg TPO at ₹142/kg with 4% runner scrap.</t>
   </si>
   <si>
     <t xml:space="preserve">Fascia material ₹</t>
@@ -332,7 +332,7 @@
     <t xml:space="preserve">Process (machine) cost</t>
   </si>
   <si>
-    <t xml:space="preserve">Cycle time ÷ 3600 × machine hour rate ÷ cavities.  The machine rate (Assumptions sheet) is a full build-up: depreciation + energy @ ₹8.5/kWh + maintenance + floor space + supervision.  A 1500-tonne press at ₹2,100/hr running a 58 s cycle costs ₹33.83 of machine time per shot — big-ticket machines, small per-part cost, because the hour is shared across every part made in it.</t>
+    <t xml:space="preserve">Cycle time ÷ 3600 × machine hour rate ÷ cavities.  The machine rate (Assumptions sheet) is a full build-up: depreciation + energy @ ₹8.5/kWh + maintenance + floor space + supervision.  A 1500-tonne press at ₹2,100/hr running a 55 s cycle costs ₹32.08 of machine time per shot — big-ticket machines, small per-part cost, because the hour is shared across every part made in it.</t>
   </si>
   <si>
     <t xml:space="preserve">Fascia process ₹</t>
@@ -356,7 +356,7 @@
     <t xml:space="preserve">Tooling amortisation</t>
   </si>
   <si>
-    <t xml:space="preserve">Tool cost ÷ (annual volume × amortisation years × parts per vehicle).  The ₹2.2 Cr fascia mould spread over 72,000 vehicles × 5 years = a per-part charge.  This is the number most sensitive to VOLUME — halve the volume and this line doubles.  If the OEM pays for tooling separately, set column S to zero on Parts Costing.</t>
+    <t xml:space="preserve">Tool cost ÷ (annual volume × amortisation years × parts per vehicle).  The ₹1.8 Cr fascia mould spread over 72,000 vehicles × 5 years = a per-part charge (₹50/part).  This is the number most sensitive to VOLUME — halve the volume and this line doubles.  If the OEM pays for tooling separately, set column S to zero on Parts Costing.</t>
   </si>
   <si>
     <t xml:space="preserve">Fascia tooling ₹/pc</t>
@@ -416,7 +416,7 @@
     <t xml:space="preserve">“₹13,000 for a bumper? The aftermarket part is ₹5,000!”</t>
   </si>
   <si>
-    <t xml:space="preserve">Two different things. The ₹13.2k includes the ADAS electronics — radar, camera, 4 parking sensors, harness — which are ~79% of the total and are usually on separate commodity contracts. The mechanical bumper module (what a bumper supplier actually quotes) is the number on the right. Aftermarket MRP is also a retail price with distribution margins — not comparable to an OEM ex-works piece price.</t>
+    <t xml:space="preserve">Two different things. The ₹8.7k total includes the ADAS electronics — radar, camera, 4 parking sensors, harness — which are ~71% of the total and are usually on separate commodity contracts. The mechanical bumper module (what a bumper supplier actually quotes) is the number on the right. Aftermarket MRP is also a retail price with distribution margins — not comparable to an OEM ex-works piece price.</t>
   </si>
   <si>
     <t xml:space="preserve">Mechanical module ₹</t>
@@ -425,7 +425,7 @@
     <t xml:space="preserve">“What happens if the volume assumption is wrong?”</t>
   </si>
   <si>
-    <t xml:space="preserve">One cell: Assumptions B4. Volume only touches amortisation (tooling, fixtures, equipment) — material, process and labour are per-piece and unaffected. At 72k/yr the fascia carries ₹61 of tooling; at 36k/yr it would carry ₹122. Test any scenario in seconds by editing the cell.</t>
+    <t xml:space="preserve">One cell: Assumptions B4. Volume only touches amortisation (tooling, fixtures, equipment) — material, process and labour are per-piece and unaffected. At 72k/yr the fascia carries ₹50 of tooling; at 36k/yr it would carry ₹100. Test any scenario in seconds by editing the cell.</t>
   </si>
   <si>
     <t xml:space="preserve">Current volume</t>
@@ -473,7 +473,7 @@
     <t xml:space="preserve">“Which parts carry the most cost?”</t>
   </si>
   <si>
-    <t xml:space="preserve">Painted fascia (~₹1,276 = moulding + body-colour paint), then the steel reinforcement beam (~₹495), then the grilles. Everything else is small brackets and covers below ₹120. In bought-out: the radar alone is more than the entire painted fascia.</t>
+    <t xml:space="preserve">Painted fascia (~₹1,078 = moulding + body-colour paint), then the steel reinforcement beam (~₹442), then the grilles. Everything else is small brackets and covers below ₹120. In bought-out: the radar alone is more than the entire painted fascia.</t>
   </si>
   <si>
     <t xml:space="preserve">Painted fascia ₹</t>
@@ -485,10 +485,10 @@
     <t xml:space="preserve">Yes — that is its purpose. Hand the supplier the same structure and ask them to fill THEIR numbers: where their material price, cycle time or overhead differs from ours, that specific cell becomes the discussion. Suppliers concede far more against a bottom-up model than against “please give 5% discount”.</t>
   </si>
   <si>
-    <t xml:space="preserve">“Why does paint cost ₹416 when the paint material is only ₹185?”</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Body-colour painting is a process cost, not a material cost: a robotic paint line at ₹2,800/hr with booth energy and ventilation, ~130 s per bumper, plus overhead and margin on that conversion. If the fascia is supplied moulded-in-colour, delete the paint row — the model drops it cleanly.</t>
+    <t xml:space="preserve">“Why does paint cost ₹338 when the paint material is only ₹160?”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Body-colour painting is a process cost, not a material cost: a robotic paint line at ₹2,400/hr with booth energy and ventilation, ~110 s per bumper, plus overhead and margin on that conversion. If the fascia is supplied moulded-in-colour, delete the paint row — the model drops it cleanly.</t>
   </si>
   <si>
     <t xml:space="preserve">Paint line item ₹</t>
@@ -503,7 +503,10 @@
     <t xml:space="preserve">“How would we make this part cheaper?”</t>
   </si>
   <si>
-    <t xml:space="preserve">The levers, in order of size: (1) delete/reduce paint (moulded-in-colour saves ~₹400), (2) resin contract price — every ₹10/kg on TPO is ~₹44 on the fascia, (3) volume pooling to spread tooling, (4) runner regrind reuse instead of selling scrap, (5) beam gauge/grade optimisation. The workbook quantifies each in seconds.</t>
+    <t xml:space="preserve">The levers, in order of size: (1) delete/reduce paint (moulded-in-colour saves ~₹338), (2) resin contract price — every ₹10/kg on TPO is ~₹37 on the fascia, (3) volume pooling to spread tooling, (4) runner regrind reuse instead of selling scrap, (5) beam gauge/grade optimisation. All 15 ideas are quantified in the green COST-SAVING IDEAS table on the Summary sheet — the total indicative potential is shown live on the right.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Savings potential ₹/veh</t>
   </si>
   <si>
     <t xml:space="preserve">CostVision — Should-Cost Assumptions &amp; Rate Card (India, 2026)</t>
@@ -5574,7 +5577,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -5987,7 +5990,15 @@
       <c r="C40" s="50" t="s">
         <v>149</v>
       </c>
-      <c r="D40" s="51"/>
+      <c r="D40" s="53" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D41" s="44" t="n">
+        <f aca="false">Summary!D69</f>
+        <v>854.1639128</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -6022,7 +6033,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6030,7 +6041,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6038,7 +6049,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="54" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B3" s="54"/>
       <c r="C3" s="54"/>
@@ -6046,61 +6057,61 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="55" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B4" s="56" t="n">
         <v>72000</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="55" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B5" s="57" t="n">
         <v>5</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="55" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B6" s="57" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C6" s="23"/>
       <c r="D6" s="23" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="55" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B7" s="56" t="n">
         <v>106</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="54" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B9" s="54"/>
       <c r="C9" s="54"/>
@@ -6108,133 +6119,133 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="55" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B10" s="58" t="n">
         <v>98</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="55" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B11" s="58" t="n">
         <v>142</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="55" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B12" s="58" t="n">
         <v>148</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="55" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B13" s="58" t="n">
         <v>330</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="55" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B14" s="58" t="n">
         <v>210</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="55" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B15" s="58" t="n">
         <v>68</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="55" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B16" s="58" t="n">
         <v>32</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="55" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B17" s="58" t="n">
         <v>40</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="55" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B18" s="58" t="n">
         <v>160</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="54" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B20" s="54"/>
       <c r="C20" s="54"/>
@@ -6242,147 +6253,147 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="55" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B21" s="59" t="n">
         <v>2100</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="55" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B22" s="59" t="n">
         <v>1150</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="55" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B23" s="59" t="n">
         <v>700</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="55" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B24" s="59" t="n">
         <v>520</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="55" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B25" s="59" t="n">
         <v>400</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="55" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B26" s="59" t="n">
         <v>650</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="55" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B27" s="59" t="n">
         <v>900</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="55" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B28" s="59" t="n">
         <v>1600</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="55" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B29" s="59" t="n">
         <v>800</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="55" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B30" s="59" t="n">
         <v>2400</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="54" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B32" s="54"/>
       <c r="C32" s="54"/>
@@ -6390,47 +6401,47 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="55" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B33" s="59" t="n">
         <v>190</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="55" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B34" s="59" t="n">
         <v>260</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D34" s="23"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="55" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B35" s="59" t="n">
         <v>230</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="54" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B37" s="54"/>
       <c r="C37" s="54"/>
@@ -6438,16 +6449,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="55" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B38" s="60" t="n">
         <v>0.4</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6458,10 +6469,10 @@
         <v>0.08</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6472,66 +6483,66 @@
         <v>0.1</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="55" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B41" s="60" t="n">
         <v>0.03</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="55" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B42" s="60" t="n">
         <v>0.45</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="55" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B43" s="58" t="n">
         <v>55</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="55" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B44" s="61" t="n">
         <v>4</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -6588,7 +6599,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6618,7 +6629,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6648,10 +6659,10 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>53</v>
@@ -6660,73 +6671,73 @@
         <v>50</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="Z3" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AA3" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6734,13 +6745,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="63" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C4" s="64" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D4" s="64" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E4" s="62" t="n">
         <v>1</v>
@@ -6764,7 +6775,7 @@
         <v>525.888</v>
       </c>
       <c r="K4" s="64" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="L4" s="68" t="n">
         <f aca="false">Assumptions!$B$21</f>
@@ -6828,13 +6839,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="74" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C5" s="75" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D5" s="75" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E5" s="73" t="n">
         <v>1</v>
@@ -6848,7 +6859,7 @@
         <v>160</v>
       </c>
       <c r="K5" s="75" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="L5" s="77" t="n">
         <f aca="false">Assumptions!$B$30</f>
@@ -6912,13 +6923,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="63" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C6" s="64" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D6" s="64" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E6" s="62" t="n">
         <v>1</v>
@@ -6942,7 +6953,7 @@
         <v>45.405</v>
       </c>
       <c r="K6" s="64" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="L6" s="68" t="n">
         <f aca="false">Assumptions!$B$23</f>
@@ -7006,13 +7017,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="74" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C7" s="75" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D7" s="75" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E7" s="73" t="n">
         <v>1</v>
@@ -7036,7 +7047,7 @@
         <v>55.495</v>
       </c>
       <c r="K7" s="75" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="L7" s="77" t="n">
         <f aca="false">Assumptions!$B$23</f>
@@ -7100,13 +7111,13 @@
         <v>5</v>
       </c>
       <c r="B8" s="63" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C8" s="64" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D8" s="64" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E8" s="62" t="n">
         <v>2</v>
@@ -7130,7 +7141,7 @@
         <v>12.0384</v>
       </c>
       <c r="K8" s="64" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L8" s="68" t="n">
         <f aca="false">Assumptions!$B$25</f>
@@ -7194,13 +7205,13 @@
         <v>6</v>
       </c>
       <c r="B9" s="74" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C9" s="75" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D9" s="75" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E9" s="73" t="n">
         <v>1</v>
@@ -7224,7 +7235,7 @@
         <v>18.0576</v>
       </c>
       <c r="K9" s="75" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L9" s="77" t="n">
         <f aca="false">Assumptions!$B$25</f>
@@ -7288,13 +7299,13 @@
         <v>7</v>
       </c>
       <c r="B10" s="63" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C10" s="64" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D10" s="64" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E10" s="62" t="n">
         <v>2</v>
@@ -7318,7 +7329,7 @@
         <v>23.01</v>
       </c>
       <c r="K10" s="64" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L10" s="68" t="n">
         <f aca="false">Assumptions!$B$24</f>
@@ -7385,10 +7396,10 @@
         <v>58</v>
       </c>
       <c r="C11" s="75" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D11" s="75" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E11" s="73" t="n">
         <v>1</v>
@@ -7412,7 +7423,7 @@
         <v>83.95</v>
       </c>
       <c r="K11" s="75" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="L11" s="77" t="n">
         <f aca="false">Assumptions!$B$26</f>
@@ -7476,13 +7487,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="63" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C12" s="64" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D12" s="64" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E12" s="62" t="n">
         <v>1</v>
@@ -7506,7 +7517,7 @@
         <v>297.696</v>
       </c>
       <c r="K12" s="64" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L12" s="68" t="n">
         <f aca="false">Assumptions!$B$28</f>
@@ -7570,13 +7581,13 @@
         <v>10</v>
       </c>
       <c r="B13" s="74" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C13" s="75" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D13" s="75" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E13" s="73" t="n">
         <v>1</v>
@@ -7589,7 +7600,7 @@
         <v>0</v>
       </c>
       <c r="K13" s="75" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L13" s="77" t="n">
         <f aca="false">Assumptions!$B$29</f>
@@ -7653,13 +7664,13 @@
         <v>11</v>
       </c>
       <c r="B14" s="63" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C14" s="64" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D14" s="64" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E14" s="62" t="n">
         <v>2</v>
@@ -7683,7 +7694,7 @@
         <v>25.312</v>
       </c>
       <c r="K14" s="64" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="L14" s="68" t="n">
         <f aca="false">Assumptions!$B$27</f>
@@ -7747,13 +7758,13 @@
         <v>12</v>
       </c>
       <c r="B15" s="74" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C15" s="75" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D15" s="75" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E15" s="73" t="n">
         <v>1</v>
@@ -7777,7 +7788,7 @@
         <v>5.016</v>
       </c>
       <c r="K15" s="75" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L15" s="77" t="n">
         <f aca="false">Assumptions!$B$25</f>
@@ -7841,13 +7852,13 @@
         <v>13</v>
       </c>
       <c r="B16" s="63" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C16" s="64" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D16" s="64" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E16" s="79" t="n">
         <f aca="false">Assumptions!$B$44</f>
@@ -7872,7 +7883,7 @@
         <v>2.0064</v>
       </c>
       <c r="K16" s="64" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L16" s="68" t="n">
         <f aca="false">Assumptions!$B$25</f>
@@ -7936,13 +7947,13 @@
         <v>14</v>
       </c>
       <c r="B17" s="74" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C17" s="75" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D17" s="75" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E17" s="73" t="n">
         <v>1</v>
@@ -7966,7 +7977,7 @@
         <v>8.0256</v>
       </c>
       <c r="K17" s="75" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L17" s="77" t="n">
         <f aca="false">Assumptions!$B$25</f>
@@ -8030,13 +8041,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="63" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C18" s="64" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D18" s="64" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E18" s="62" t="n">
         <v>1</v>
@@ -8060,7 +8071,7 @@
         <v>5.016</v>
       </c>
       <c r="K18" s="64" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L18" s="68" t="n">
         <f aca="false">Assumptions!$B$25</f>
@@ -8124,13 +8135,13 @@
         <v>16</v>
       </c>
       <c r="B19" s="74" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C19" s="75" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D19" s="75" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E19" s="73" t="n">
         <v>1</v>
@@ -8154,7 +8165,7 @@
         <v>35.315</v>
       </c>
       <c r="K19" s="75" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="L19" s="77" t="n">
         <f aca="false">Assumptions!$B$23</f>
@@ -8218,13 +8229,13 @@
         <v>17</v>
       </c>
       <c r="B20" s="63" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C20" s="64" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D20" s="64" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E20" s="62" t="n">
         <v>2</v>
@@ -8248,7 +8259,7 @@
         <v>15.048</v>
       </c>
       <c r="K20" s="64" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L20" s="68" t="n">
         <f aca="false">Assumptions!$B$24</f>
@@ -8312,13 +8323,13 @@
         <v>18</v>
       </c>
       <c r="B21" s="74" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C21" s="75" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D21" s="75" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E21" s="73" t="n">
         <v>2</v>
@@ -8342,7 +8353,7 @@
         <v>15.048</v>
       </c>
       <c r="K21" s="75" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L21" s="77" t="n">
         <f aca="false">Assumptions!$B$24</f>
@@ -8404,7 +8415,7 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="36"/>
       <c r="B22" s="36" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C22" s="36"/>
       <c r="D22" s="36"/>
@@ -8472,7 +8483,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8483,7 +8494,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -8494,25 +8505,25 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8520,7 +8531,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="83" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C4" s="83" t="s">
         <v>68</v>
@@ -8546,7 +8557,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="83" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C5" s="83" t="s">
         <v>68</v>
@@ -8571,7 +8582,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="83" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C6" s="83" t="s">
         <v>68</v>
@@ -8596,10 +8607,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="83" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C7" s="83" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D7" s="82" t="n">
         <v>1</v>
@@ -8621,10 +8632,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="83" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C8" s="83" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D8" s="82" t="n">
         <v>1</v>
@@ -8646,10 +8657,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="83" t="s">
+        <v>311</v>
+      </c>
+      <c r="C9" s="83" t="s">
         <v>310</v>
-      </c>
-      <c r="C9" s="83" t="s">
-        <v>309</v>
       </c>
       <c r="D9" s="82" t="n">
         <v>1</v>
@@ -8671,10 +8682,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="83" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C10" s="83" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D10" s="82" t="n">
         <v>1</v>
@@ -8694,7 +8705,7 @@
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="36"/>
       <c r="B11" s="36" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C11" s="36"/>
       <c r="D11" s="36"/>
@@ -8707,7 +8718,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="87" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G12" s="18" t="n">
         <f aca="false">SUM(G4:G7)</f>
@@ -8747,7 +8758,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8758,7 +8769,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -8769,25 +8780,25 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8795,7 +8806,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="88" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C4" s="89" t="n">
         <v>60</v>
@@ -8812,7 +8823,7 @@
         <v>3.16666666666667</v>
       </c>
       <c r="G4" s="88" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8820,7 +8831,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="88" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C5" s="89" t="n">
         <v>120</v>
@@ -8837,7 +8848,7 @@
         <v>12.6666666666667</v>
       </c>
       <c r="G5" s="88" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8845,7 +8856,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="88" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C6" s="89" t="n">
         <v>150</v>
@@ -8862,7 +8873,7 @@
         <v>11.875</v>
       </c>
       <c r="G6" s="88" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8870,7 +8881,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="88" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C7" s="89" t="n">
         <v>75</v>
@@ -8893,7 +8904,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="88" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C8" s="89" t="n">
         <v>60</v>
@@ -8910,7 +8921,7 @@
         <v>3.83333333333333</v>
       </c>
       <c r="G8" s="88" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8918,7 +8929,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="88" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C9" s="89" t="n">
         <v>45</v>
@@ -8938,7 +8949,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="92" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C11" s="31"/>
       <c r="D11" s="31"/>
@@ -8951,7 +8962,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="92" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C12" s="31"/>
       <c r="D12" s="31"/>
@@ -8961,12 +8972,12 @@
         <v>11.1111111111111</v>
       </c>
       <c r="G12" s="94" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="92" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C13" s="31"/>
       <c r="D13" s="31"/>
@@ -8979,7 +8990,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="92" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C14" s="31"/>
       <c r="D14" s="31"/>
@@ -8988,12 +8999,12 @@
         <v>6</v>
       </c>
       <c r="G14" s="94" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="92" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C15" s="31"/>
       <c r="D15" s="31"/>
@@ -9003,12 +9014,12 @@
         <v>17.04375</v>
       </c>
       <c r="G15" s="94" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="92" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C16" s="31"/>
       <c r="D16" s="31"/>
@@ -9021,7 +9032,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="96" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C17" s="96"/>
       <c r="D17" s="96"/>
@@ -9061,7 +9072,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9069,7 +9080,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -9077,15 +9088,15 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B4" s="98" t="n">
         <f aca="false">'Parts Costing'!S22</f>
@@ -9094,7 +9105,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B5" s="98" t="n">
         <v>4000000</v>
@@ -9102,7 +9113,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="31" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B6" s="98" t="n">
         <v>6000000</v>
@@ -9110,7 +9121,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="99" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B7" s="100" t="n">
         <f aca="false">SUM(B4:B6)</f>
@@ -9119,7 +9130,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="101" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B9" s="102" t="n">
         <f aca="false">B7/10000000</f>

</xml_diff>

<commit_message>
Bumper should-cost: material prices verified against Jul-2026 India market
Deep-dive on all raw-material rates: EPP corrected 330->700/kg (330 was
FOB China bead price; delivered India automotive grade incl duty/freight,
per procurement input); PP 98->112 (OfBusiness spot 110-120); TPO 142->155
(PP + compounding premium); ABS 148->158 (coloured auto grade 155-170).
Steel/POM/credits confirmed in range. Totals: 8,747 -> 8,966; mechanical
module 2,567 -> 2,786; absorber 142 -> 254. Methodology narrative and
cost-driver comment synced.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142L4rKS2AV8rxQTDWMs7dy
</commit_message>
<xml_diff>
--- a/Altroz-Front-Bumper-Should-Cost-India.xlsx
+++ b/Altroz-Front-Bumper-Should-Cost-India.xlsx
@@ -40,12 +40,12 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">Major cost drivers:
-1. Front radar — largest single item (~38% of total)
+1. Front radar — largest single item (~37% of total)
 2. Painted fascia — largest manufactured part (~12%)
 3. Front camera (~18%)
 4. Parking sensors set (~10%)
 5. Steel reinforcement beam (~5%)
-Together the top 5 are ~83% of the should-cost — focus negotiation there.</t>
+Together the top 5 are ~82% of the should-cost — focus negotiation there.</t>
         </r>
       </text>
     </comment>
@@ -323,7 +323,7 @@
     <t xml:space="preserve">Material cost per part</t>
   </si>
   <si>
-    <t xml:space="preserve">Net part mass × (1 + scrap%) × material price ₹/kg, minus scrap credit for the recoverable portion.  Formula in words: you buy slightly more plastic/steel than ends up in the part (runners, offal), and sell back what you can.  Excel: =Mass×(1+Scrap)×Price − Mass×Scrap×Credit  →  Fascia: 3.60 kg TPO at ₹142/kg with 4% runner scrap.</t>
+    <t xml:space="preserve">Net part mass × (1 + scrap%) × material price ₹/kg, minus scrap credit for the recoverable portion.  Formula in words: you buy slightly more plastic/steel than ends up in the part (runners, offal), and sell back what you can.  Excel: =Mass×(1+Scrap)×Price − Mass×Scrap×Credit  →  Fascia: 3.60 kg TPO at ₹155/kg with 4% runner scrap.</t>
   </si>
   <si>
     <t xml:space="preserve">Fascia material ₹</t>
@@ -416,7 +416,7 @@
     <t xml:space="preserve">“₹13,000 for a bumper? The aftermarket part is ₹5,000!”</t>
   </si>
   <si>
-    <t xml:space="preserve">Two different things. The ₹8.7k total includes the ADAS electronics — radar, camera, 4 parking sensors, harness — which are ~71% of the total and are usually on separate commodity contracts. The mechanical bumper module (what a bumper supplier actually quotes) is the number on the right. Aftermarket MRP is also a retail price with distribution margins — not comparable to an OEM ex-works piece price.</t>
+    <t xml:space="preserve">Two different things. The ₹9.0k total includes the ADAS electronics — radar, camera, 4 parking sensors, harness — which are ~69% of the total and are usually on separate commodity contracts. The mechanical bumper module (what a bumper supplier actually quotes) is the number on the right. Aftermarket MRP is also a retail price with distribution margins — not comparable to an OEM ex-works piece price.</t>
   </si>
   <si>
     <t xml:space="preserve">Mechanical module ₹</t>
@@ -473,7 +473,7 @@
     <t xml:space="preserve">“Which parts carry the most cost?”</t>
   </si>
   <si>
-    <t xml:space="preserve">Painted fascia (~₹1,078 = moulding + body-colour paint), then the steel reinforcement beam (~₹442), then the grilles. Everything else is small brackets and covers below ₹120. In bought-out: the radar alone is more than the entire painted fascia.</t>
+    <t xml:space="preserve">Painted fascia (~₹1,136 = moulding + body-colour paint), then the steel reinforcement beam (~₹442), then the energy absorber (EPP is a premium imported material). Everything else is small brackets and covers below ₹120. In bought-out: the radar alone is more than the entire painted fascia.</t>
   </si>
   <si>
     <t xml:space="preserve">Painted fascia ₹</t>
@@ -563,25 +563,25 @@
     <t xml:space="preserve">₹/kg</t>
   </si>
   <si>
-    <t xml:space="preserve">Polypropylene copolymer, bulk OEM contract.</t>
+    <t xml:space="preserve">PP copolymer ₹110–120/kg India spot (OfBusiness, Jul 2026); OEM contract mid-range.</t>
   </si>
   <si>
     <t xml:space="preserve">PP+EPDM (TPO bumper grade)</t>
   </si>
   <si>
-    <t xml:space="preserve">Impact-modified bumper compound, paintable grade.</t>
+    <t xml:space="preserve">PP copolymer + EPDM/talc compounding premium ~₹35–45/kg; paintable bumper grade.</t>
   </si>
   <si>
     <t xml:space="preserve">ABS (plating/paint grade)</t>
   </si>
   <si>
-    <t xml:space="preserve">For fog-lamp bezels / DRL housings.</t>
+    <t xml:space="preserve">ABS coloured/auto grade ₹155–170/kg India (OfBusiness, Jul 2026).</t>
   </si>
   <si>
     <t xml:space="preserve">EPP beads (45 g/l)</t>
   </si>
   <si>
-    <t xml:space="preserve">Expanded polypropylene for energy absorber.</t>
+    <t xml:space="preserve">Delivered India automotive grade (imported beads + duty + freight); FOB China ~₹330 — corrected per procurement input.</t>
   </si>
   <si>
     <t xml:space="preserve">POM (clips)</t>
@@ -2126,7 +2126,7 @@
                 <c:formatCode>"₹ "#,##0.00</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>2567.11541687778</c:v>
+                  <c:v>2786.48413127778</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>6180</c:v>
@@ -2652,7 +2652,7 @@
                 <c:formatCode>"₹ "#,##0.00</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>1428.8026</c:v>
+                  <c:v>1613.4564</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>223.347402777778</c:v>
@@ -2664,10 +2664,10 @@
                   <c:v>89.3389611111111</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>153.274672666667</c:v>
+                  <c:v>168.046976666667</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>206.9208081</c:v>
+                  <c:v>226.8634185</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>6143</c:v>
@@ -3829,28 +3829,28 @@
                 <c:formatCode>"₹ "#,##0.00</c:formatCode>
                 <c:ptCount val="25"/>
                 <c:pt idx="0">
-                  <c:v>739.929894</c:v>
+                  <c:v>797.75223</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>338.4546</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>81.7168968</c:v>
+                  <c:v>89.5755168</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>95.8180212</c:v>
+                  <c:v>105.4230012</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>39.9186084</c:v>
+                  <c:v>44.0699556</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>31.2012888</c:v>
+                  <c:v>34.3147992</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>73.0648116</c:v>
+                  <c:v>76.8070116</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>142.2597</c:v>
+                  <c:v>254.3475</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>407.376948</c:v>
@@ -3862,25 +3862,25 @@
                   <c:v>73.907592</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>11.203203</c:v>
+                  <c:v>12.068067</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>18.2893128</c:v>
+                  <c:v>19.6730952</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>15.7487253</c:v>
+                  <c:v>17.1325077</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>11.203203</c:v>
+                  <c:v>12.068067</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>63.4823442</c:v>
+                  <c:v>69.5946042</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>49.11027</c:v>
+                  <c:v>54.299454</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>49.11027</c:v>
+                  <c:v>54.299454</c:v>
                 </c:pt>
                 <c:pt idx="18">
                   <c:v>906.4</c:v>
@@ -4718,11 +4718,11 @@
       </c>
       <c r="D5" s="7" t="n">
         <f aca="false">'Parts Costing'!$Z$22</f>
-        <v>2276.1288891</v>
+        <v>2495.4976035</v>
       </c>
       <c r="E5" s="8" t="n">
         <f aca="false">D5/$D$8</f>
-        <v>0.26021480003661</v>
+        <v>0.278313948584926</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4741,7 +4741,7 @@
       </c>
       <c r="E6" s="8" t="n">
         <f aca="false">D6/$D$8</f>
-        <v>0.723357323923191</v>
+        <v>0.705660090104718</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="E7" s="8" t="n">
         <f aca="false">D7/$D$8</f>
-        <v>0.0164278760401985</v>
+        <v>0.0160259613103559</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4771,7 +4771,7 @@
       <c r="C8" s="9"/>
       <c r="D8" s="11" t="n">
         <f aca="false">SUM(D5:D7)</f>
-        <v>8747.11541687778</v>
+        <v>8966.48413127778</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>1</v>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="D10" s="14" t="n">
         <f aca="false">D8-'Bought-Out'!$G$12</f>
-        <v>2567.11541687778</v>
+        <v>2786.48413127778</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4810,7 +4810,7 @@
       </c>
       <c r="D13" s="18" t="n">
         <f aca="false">'Parts Costing'!Y4+'Parts Costing'!Y5</f>
-        <v>1078.384494</v>
+        <v>1136.20683</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4853,7 +4853,7 @@
       </c>
       <c r="D36" s="22" t="n">
         <f aca="false">'Parts Costing'!Z4+'Parts Costing'!Z5</f>
-        <v>1078.384494</v>
+        <v>1136.20683</v>
       </c>
       <c r="E36" s="23" t="s">
         <v>26</v>
@@ -5069,7 +5069,7 @@
       </c>
       <c r="D60" s="30" t="n">
         <f aca="false">0.04*Assumptions!$B$13*1.35</f>
-        <v>17.82</v>
+        <v>37.8</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5084,7 +5084,7 @@
       </c>
       <c r="D61" s="34" t="n">
         <f aca="false">'Parts Costing'!Z16</f>
-        <v>18.2893128</v>
+        <v>19.6730952</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5196,7 +5196,7 @@
       <c r="C69" s="35"/>
       <c r="D69" s="37" t="n">
         <f aca="false">SUM(D54:D68)</f>
-        <v>854.1639128</v>
+        <v>875.5276952</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5210,7 +5210,7 @@
       </c>
       <c r="B100" s="18" t="n">
         <f aca="false">D8-'Bought-Out'!$G$12</f>
-        <v>2567.11541687778</v>
+        <v>2786.48413127778</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5228,7 +5228,7 @@
       </c>
       <c r="B103" s="18" t="n">
         <f aca="false">SUMPRODUCT('Parts Costing'!$J$4:$J$21,'Parts Costing'!$E$4:$E$21)</f>
-        <v>1428.8026</v>
+        <v>1613.4564</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="B107" s="18" t="n">
         <f aca="false">SUMPRODUCT('Parts Costing'!$W$4:$W$21,'Parts Costing'!$E$4:$E$21)</f>
-        <v>153.274672666667</v>
+        <v>168.046976666667</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="B108" s="18" t="n">
         <f aca="false">SUMPRODUCT('Parts Costing'!$X$4:$X$21,'Parts Costing'!$E$4:$E$21)</f>
-        <v>206.9208081</v>
+        <v>226.8634185</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5310,7 +5310,7 @@
       </c>
       <c r="B115" s="18" t="n">
         <f aca="false">'Parts Costing'!Z4</f>
-        <v>739.929894</v>
+        <v>797.75223</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="B117" s="18" t="n">
         <f aca="false">'Parts Costing'!Z6</f>
-        <v>81.7168968</v>
+        <v>89.5755168</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5340,7 +5340,7 @@
       </c>
       <c r="B118" s="18" t="n">
         <f aca="false">'Parts Costing'!Z7</f>
-        <v>95.8180212</v>
+        <v>105.4230012</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5350,7 +5350,7 @@
       </c>
       <c r="B119" s="18" t="n">
         <f aca="false">'Parts Costing'!Z8</f>
-        <v>39.9186084</v>
+        <v>44.0699556</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5360,7 +5360,7 @@
       </c>
       <c r="B120" s="18" t="n">
         <f aca="false">'Parts Costing'!Z9</f>
-        <v>31.2012888</v>
+        <v>34.3147992</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5370,7 +5370,7 @@
       </c>
       <c r="B121" s="18" t="n">
         <f aca="false">'Parts Costing'!Z10</f>
-        <v>73.0648116</v>
+        <v>76.8070116</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="B122" s="18" t="n">
         <f aca="false">'Parts Costing'!Z11</f>
-        <v>142.2597</v>
+        <v>254.3475</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="B126" s="18" t="n">
         <f aca="false">'Parts Costing'!Z15</f>
-        <v>11.203203</v>
+        <v>12.068067</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="B127" s="18" t="n">
         <f aca="false">'Parts Costing'!Z16</f>
-        <v>18.2893128</v>
+        <v>19.6730952</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5440,7 +5440,7 @@
       </c>
       <c r="B128" s="18" t="n">
         <f aca="false">'Parts Costing'!Z17</f>
-        <v>15.7487253</v>
+        <v>17.1325077</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="B129" s="18" t="n">
         <f aca="false">'Parts Costing'!Z18</f>
-        <v>11.203203</v>
+        <v>12.068067</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5460,7 +5460,7 @@
       </c>
       <c r="B130" s="18" t="n">
         <f aca="false">'Parts Costing'!Z19</f>
-        <v>63.4823442</v>
+        <v>69.5946042</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5470,7 +5470,7 @@
       </c>
       <c r="B131" s="18" t="n">
         <f aca="false">'Parts Costing'!Z20</f>
-        <v>49.11027</v>
+        <v>54.299454</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="B132" s="18" t="n">
         <f aca="false">'Parts Costing'!Z21</f>
-        <v>49.11027</v>
+        <v>54.299454</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5641,7 +5641,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D6" s="44" t="n">
         <f aca="false">'Parts Costing'!J4</f>
-        <v>525.888</v>
+        <v>574.56</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5721,7 +5721,7 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D14" s="44" t="n">
         <f aca="false">'Parts Costing'!Y4</f>
-        <v>739.929894</v>
+        <v>797.75223</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5761,7 +5761,7 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D18" s="44" t="n">
         <f aca="false">Summary!D8</f>
-        <v>8747.11541687778</v>
+        <v>8966.48413127778</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5813,7 +5813,7 @@
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D24" s="44" t="n">
         <f aca="false">Summary!D10</f>
-        <v>2567.11541687778</v>
+        <v>2786.48413127778</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5933,7 +5933,7 @@
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D35" s="44" t="n">
         <f aca="false">'Parts Costing'!Y4+'Parts Costing'!Y5</f>
-        <v>1078.384494</v>
+        <v>1136.20683</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5997,7 +5997,7 @@
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D41" s="44" t="n">
         <f aca="false">Summary!D69</f>
-        <v>854.1639128</v>
+        <v>875.5276952</v>
       </c>
     </row>
   </sheetData>
@@ -6122,7 +6122,7 @@
         <v>167</v>
       </c>
       <c r="B10" s="58" t="n">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="C10" s="23" t="s">
         <v>168</v>
@@ -6136,7 +6136,7 @@
         <v>170</v>
       </c>
       <c r="B11" s="58" t="n">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="C11" s="23" t="s">
         <v>168</v>
@@ -6150,7 +6150,7 @@
         <v>172</v>
       </c>
       <c r="B12" s="58" t="n">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="C12" s="23" t="s">
         <v>168</v>
@@ -6164,7 +6164,7 @@
         <v>174</v>
       </c>
       <c r="B13" s="58" t="n">
-        <v>330</v>
+        <v>700</v>
       </c>
       <c r="C13" s="23" t="s">
         <v>168</v>
@@ -6764,7 +6764,7 @@
       </c>
       <c r="H4" s="67" t="n">
         <f aca="false">Assumptions!$B$11</f>
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="I4" s="67" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="J4" s="67" t="n">
         <f aca="false">F4*(1+G4)*H4-F4*G4*I4</f>
-        <v>525.888</v>
+        <v>574.56</v>
       </c>
       <c r="K4" s="64" t="s">
         <v>260</v>
@@ -6815,23 +6815,23 @@
       </c>
       <c r="V4" s="67" t="n">
         <f aca="false">J4+O4+R4+T4+U4</f>
-        <v>622.836611111111</v>
+        <v>671.508611111111</v>
       </c>
       <c r="W4" s="67" t="n">
         <f aca="false">V4*Assumptions!$B$39</f>
-        <v>49.8269288888889</v>
+        <v>53.7206888888889</v>
       </c>
       <c r="X4" s="67" t="n">
         <f aca="false">(V4+W4)*Assumptions!$B$40</f>
-        <v>67.266354</v>
+        <v>72.52293</v>
       </c>
       <c r="Y4" s="72" t="n">
         <f aca="false">V4+W4+X4</f>
-        <v>739.929894</v>
+        <v>797.75223</v>
       </c>
       <c r="Z4" s="72" t="n">
         <f aca="false">Y4*E4</f>
-        <v>739.929894</v>
+        <v>797.75223</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6942,7 +6942,7 @@
       </c>
       <c r="H6" s="67" t="n">
         <f aca="false">Assumptions!$B$10</f>
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I6" s="67" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -6950,7 +6950,7 @@
       </c>
       <c r="J6" s="67" t="n">
         <f aca="false">F6*(1+G6)*H6-F6*G6*I6</f>
-        <v>45.405</v>
+        <v>52.02</v>
       </c>
       <c r="K6" s="64" t="s">
         <v>267</v>
@@ -6993,23 +6993,23 @@
       </c>
       <c r="V6" s="67" t="n">
         <f aca="false">J6+O6+R6+T6+U6</f>
-        <v>68.7852666666667</v>
+        <v>75.4002666666667</v>
       </c>
       <c r="W6" s="67" t="n">
         <f aca="false">V6*Assumptions!$B$39</f>
-        <v>5.50282133333333</v>
+        <v>6.03202133333333</v>
       </c>
       <c r="X6" s="67" t="n">
         <f aca="false">(V6+W6)*Assumptions!$B$40</f>
-        <v>7.4288088</v>
+        <v>8.1432288</v>
       </c>
       <c r="Y6" s="72" t="n">
         <f aca="false">V6+W6+X6</f>
-        <v>81.7168968</v>
+        <v>89.5755168</v>
       </c>
       <c r="Z6" s="72" t="n">
         <f aca="false">Y6*E6</f>
-        <v>81.7168968</v>
+        <v>89.5755168</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7036,7 +7036,7 @@
       </c>
       <c r="H7" s="76" t="n">
         <f aca="false">Assumptions!$B$10</f>
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I7" s="76" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="J7" s="76" t="n">
         <f aca="false">F7*(1+G7)*H7-F7*G7*I7</f>
-        <v>55.495</v>
+        <v>63.58</v>
       </c>
       <c r="K7" s="75" t="s">
         <v>267</v>
@@ -7087,23 +7087,23 @@
       </c>
       <c r="V7" s="76" t="n">
         <f aca="false">J7+O7+R7+T7+U7</f>
-        <v>80.6549</v>
+        <v>88.7399</v>
       </c>
       <c r="W7" s="76" t="n">
         <f aca="false">V7*Assumptions!$B$39</f>
-        <v>6.452392</v>
+        <v>7.099192</v>
       </c>
       <c r="X7" s="76" t="n">
         <f aca="false">(V7+W7)*Assumptions!$B$40</f>
-        <v>8.7107292</v>
+        <v>9.5839092</v>
       </c>
       <c r="Y7" s="78" t="n">
         <f aca="false">V7+W7+X7</f>
-        <v>95.8180212</v>
+        <v>105.4230012</v>
       </c>
       <c r="Z7" s="78" t="n">
         <f aca="false">Y7*E7</f>
-        <v>95.8180212</v>
+        <v>105.4230012</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7130,7 +7130,7 @@
       </c>
       <c r="H8" s="67" t="n">
         <f aca="false">Assumptions!$B$10</f>
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I8" s="67" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -7138,7 +7138,7 @@
       </c>
       <c r="J8" s="67" t="n">
         <f aca="false">F8*(1+G8)*H8-F8*G8*I8</f>
-        <v>12.0384</v>
+        <v>13.7856</v>
       </c>
       <c r="K8" s="64" t="s">
         <v>271</v>
@@ -7181,23 +7181,23 @@
       </c>
       <c r="V8" s="67" t="n">
         <f aca="false">J8+O8+R8+T8+U8</f>
-        <v>16.8007611111111</v>
+        <v>18.5479611111111</v>
       </c>
       <c r="W8" s="67" t="n">
         <f aca="false">V8*Assumptions!$B$39</f>
-        <v>1.34406088888889</v>
+        <v>1.48383688888889</v>
       </c>
       <c r="X8" s="67" t="n">
         <f aca="false">(V8+W8)*Assumptions!$B$40</f>
-        <v>1.8144822</v>
+        <v>2.0031798</v>
       </c>
       <c r="Y8" s="72" t="n">
         <f aca="false">V8+W8+X8</f>
-        <v>19.9593042</v>
+        <v>22.0349778</v>
       </c>
       <c r="Z8" s="72" t="n">
         <f aca="false">Y8*E8</f>
-        <v>39.9186084</v>
+        <v>44.0699556</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="H9" s="76" t="n">
         <f aca="false">Assumptions!$B$10</f>
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I9" s="76" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -7232,7 +7232,7 @@
       </c>
       <c r="J9" s="76" t="n">
         <f aca="false">F9*(1+G9)*H9-F9*G9*I9</f>
-        <v>18.0576</v>
+        <v>20.6784</v>
       </c>
       <c r="K9" s="75" t="s">
         <v>271</v>
@@ -7275,23 +7275,23 @@
       </c>
       <c r="V9" s="76" t="n">
         <f aca="false">J9+O9+R9+T9+U9</f>
-        <v>26.2637111111111</v>
+        <v>28.8845111111111</v>
       </c>
       <c r="W9" s="76" t="n">
         <f aca="false">V9*Assumptions!$B$39</f>
-        <v>2.10109688888889</v>
+        <v>2.31076088888889</v>
       </c>
       <c r="X9" s="76" t="n">
         <f aca="false">(V9+W9)*Assumptions!$B$40</f>
-        <v>2.8364808</v>
+        <v>3.1195272</v>
       </c>
       <c r="Y9" s="78" t="n">
         <f aca="false">V9+W9+X9</f>
-        <v>31.2012888</v>
+        <v>34.3147992</v>
       </c>
       <c r="Z9" s="78" t="n">
         <f aca="false">Y9*E9</f>
-        <v>31.2012888</v>
+        <v>34.3147992</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7318,7 +7318,7 @@
       </c>
       <c r="H10" s="67" t="n">
         <f aca="false">Assumptions!$B$12</f>
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="I10" s="67" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -7326,7 +7326,7 @@
       </c>
       <c r="J10" s="67" t="n">
         <f aca="false">F10*(1+G10)*H10-F10*G10*I10</f>
-        <v>23.01</v>
+        <v>24.585</v>
       </c>
       <c r="K10" s="64" t="s">
         <v>275</v>
@@ -7369,23 +7369,23 @@
       </c>
       <c r="V10" s="67" t="n">
         <f aca="false">J10+O10+R10+T10+U10</f>
-        <v>30.7511833333333</v>
+        <v>32.3261833333333</v>
       </c>
       <c r="W10" s="67" t="n">
         <f aca="false">V10*Assumptions!$B$39</f>
-        <v>2.46009466666667</v>
+        <v>2.58609466666667</v>
       </c>
       <c r="X10" s="67" t="n">
         <f aca="false">(V10+W10)*Assumptions!$B$40</f>
-        <v>3.3211278</v>
+        <v>3.4912278</v>
       </c>
       <c r="Y10" s="72" t="n">
         <f aca="false">V10+W10+X10</f>
-        <v>36.5324058</v>
+        <v>38.4035058</v>
       </c>
       <c r="Z10" s="72" t="n">
         <f aca="false">Y10*E10</f>
-        <v>73.0648116</v>
+        <v>76.8070116</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7412,7 +7412,7 @@
       </c>
       <c r="H11" s="76" t="n">
         <f aca="false">Assumptions!$B$13</f>
-        <v>330</v>
+        <v>700</v>
       </c>
       <c r="I11" s="76" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="J11" s="76" t="n">
         <f aca="false">F11*(1+G11)*H11-F11*G11*I11</f>
-        <v>83.95</v>
+        <v>178.3</v>
       </c>
       <c r="K11" s="75" t="s">
         <v>278</v>
@@ -7463,23 +7463,23 @@
       </c>
       <c r="V11" s="76" t="n">
         <f aca="false">J11+O11+R11+T11+U11</f>
-        <v>119.747222222222</v>
+        <v>214.097222222222</v>
       </c>
       <c r="W11" s="76" t="n">
         <f aca="false">V11*Assumptions!$B$39</f>
-        <v>9.57977777777778</v>
+        <v>17.1277777777778</v>
       </c>
       <c r="X11" s="76" t="n">
         <f aca="false">(V11+W11)*Assumptions!$B$40</f>
-        <v>12.9327</v>
+        <v>23.1225</v>
       </c>
       <c r="Y11" s="78" t="n">
         <f aca="false">V11+W11+X11</f>
-        <v>142.2597</v>
+        <v>254.3475</v>
       </c>
       <c r="Z11" s="78" t="n">
         <f aca="false">Y11*E11</f>
-        <v>142.2597</v>
+        <v>254.3475</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7777,7 +7777,7 @@
       </c>
       <c r="H15" s="76" t="n">
         <f aca="false">Assumptions!$B$10</f>
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I15" s="76" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -7785,7 +7785,7 @@
       </c>
       <c r="J15" s="76" t="n">
         <f aca="false">F15*(1+G15)*H15-F15*G15*I15</f>
-        <v>5.016</v>
+        <v>5.744</v>
       </c>
       <c r="K15" s="75" t="s">
         <v>271</v>
@@ -7828,23 +7828,23 @@
       </c>
       <c r="V15" s="76" t="n">
         <f aca="false">J15+O15+R15+T15+U15</f>
-        <v>9.43030555555555</v>
+        <v>10.1583055555556</v>
       </c>
       <c r="W15" s="76" t="n">
         <f aca="false">V15*Assumptions!$B$39</f>
-        <v>0.754424444444444</v>
+        <v>0.812664444444445</v>
       </c>
       <c r="X15" s="76" t="n">
         <f aca="false">(V15+W15)*Assumptions!$B$40</f>
-        <v>1.018473</v>
+        <v>1.097097</v>
       </c>
       <c r="Y15" s="78" t="n">
         <f aca="false">V15+W15+X15</f>
-        <v>11.203203</v>
+        <v>12.068067</v>
       </c>
       <c r="Z15" s="78" t="n">
         <f aca="false">Y15*E15</f>
-        <v>11.203203</v>
+        <v>12.068067</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7872,7 +7872,7 @@
       </c>
       <c r="H16" s="67" t="n">
         <f aca="false">Assumptions!$B$10</f>
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I16" s="67" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -7880,7 +7880,7 @@
       </c>
       <c r="J16" s="67" t="n">
         <f aca="false">F16*(1+G16)*H16-F16*G16*I16</f>
-        <v>2.0064</v>
+        <v>2.2976</v>
       </c>
       <c r="K16" s="64" t="s">
         <v>271</v>
@@ -7923,23 +7923,23 @@
       </c>
       <c r="V16" s="67" t="n">
         <f aca="false">J16+O16+R16+T16+U16</f>
-        <v>3.84876111111111</v>
+        <v>4.13996111111111</v>
       </c>
       <c r="W16" s="67" t="n">
         <f aca="false">V16*Assumptions!$B$39</f>
-        <v>0.307900888888889</v>
+        <v>0.331196888888889</v>
       </c>
       <c r="X16" s="67" t="n">
         <f aca="false">(V16+W16)*Assumptions!$B$40</f>
-        <v>0.4156662</v>
+        <v>0.4471158</v>
       </c>
       <c r="Y16" s="72" t="n">
         <f aca="false">V16+W16+X16</f>
-        <v>4.5723282</v>
+        <v>4.9182738</v>
       </c>
       <c r="Z16" s="72" t="n">
         <f aca="false">Y16*E16</f>
-        <v>18.2893128</v>
+        <v>19.6730952</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7966,7 +7966,7 @@
       </c>
       <c r="H17" s="76" t="n">
         <f aca="false">Assumptions!$B$10</f>
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I17" s="76" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -7974,7 +7974,7 @@
       </c>
       <c r="J17" s="76" t="n">
         <f aca="false">F17*(1+G17)*H17-F17*G17*I17</f>
-        <v>8.0256</v>
+        <v>9.1904</v>
       </c>
       <c r="K17" s="75" t="s">
         <v>271</v>
@@ -8017,23 +8017,23 @@
       </c>
       <c r="V17" s="76" t="n">
         <f aca="false">J17+O17+R17+T17+U17</f>
-        <v>13.2565027777778</v>
+        <v>14.4213027777778</v>
       </c>
       <c r="W17" s="76" t="n">
         <f aca="false">V17*Assumptions!$B$39</f>
-        <v>1.06052022222222</v>
+        <v>1.15370422222222</v>
       </c>
       <c r="X17" s="76" t="n">
         <f aca="false">(V17+W17)*Assumptions!$B$40</f>
-        <v>1.4317023</v>
+        <v>1.5575007</v>
       </c>
       <c r="Y17" s="78" t="n">
         <f aca="false">V17+W17+X17</f>
-        <v>15.7487253</v>
+        <v>17.1325077</v>
       </c>
       <c r="Z17" s="78" t="n">
         <f aca="false">Y17*E17</f>
-        <v>15.7487253</v>
+        <v>17.1325077</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8060,7 +8060,7 @@
       </c>
       <c r="H18" s="67" t="n">
         <f aca="false">Assumptions!$B$10</f>
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I18" s="67" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -8068,7 +8068,7 @@
       </c>
       <c r="J18" s="67" t="n">
         <f aca="false">F18*(1+G18)*H18-F18*G18*I18</f>
-        <v>5.016</v>
+        <v>5.744</v>
       </c>
       <c r="K18" s="64" t="s">
         <v>271</v>
@@ -8111,23 +8111,23 @@
       </c>
       <c r="V18" s="67" t="n">
         <f aca="false">J18+O18+R18+T18+U18</f>
-        <v>9.43030555555555</v>
+        <v>10.1583055555556</v>
       </c>
       <c r="W18" s="67" t="n">
         <f aca="false">V18*Assumptions!$B$39</f>
-        <v>0.754424444444444</v>
+        <v>0.812664444444445</v>
       </c>
       <c r="X18" s="67" t="n">
         <f aca="false">(V18+W18)*Assumptions!$B$40</f>
-        <v>1.018473</v>
+        <v>1.097097</v>
       </c>
       <c r="Y18" s="72" t="n">
         <f aca="false">V18+W18+X18</f>
-        <v>11.203203</v>
+        <v>12.068067</v>
       </c>
       <c r="Z18" s="72" t="n">
         <f aca="false">Y18*E18</f>
-        <v>11.203203</v>
+        <v>12.068067</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8154,7 +8154,7 @@
       </c>
       <c r="H19" s="76" t="n">
         <f aca="false">Assumptions!$B$10</f>
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I19" s="76" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -8162,7 +8162,7 @@
       </c>
       <c r="J19" s="76" t="n">
         <f aca="false">F19*(1+G19)*H19-F19*G19*I19</f>
-        <v>35.315</v>
+        <v>40.46</v>
       </c>
       <c r="K19" s="75" t="s">
         <v>267</v>
@@ -8205,23 +8205,23 @@
       </c>
       <c r="V19" s="76" t="n">
         <f aca="false">J19+O19+R19+T19+U19</f>
-        <v>53.4363166666667</v>
+        <v>58.5813166666667</v>
       </c>
       <c r="W19" s="76" t="n">
         <f aca="false">V19*Assumptions!$B$39</f>
-        <v>4.27490533333333</v>
+        <v>4.68650533333333</v>
       </c>
       <c r="X19" s="76" t="n">
         <f aca="false">(V19+W19)*Assumptions!$B$40</f>
-        <v>5.7711222</v>
+        <v>6.3267822</v>
       </c>
       <c r="Y19" s="78" t="n">
         <f aca="false">V19+W19+X19</f>
-        <v>63.4823442</v>
+        <v>69.5946042</v>
       </c>
       <c r="Z19" s="78" t="n">
         <f aca="false">Y19*E19</f>
-        <v>63.4823442</v>
+        <v>69.5946042</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8248,7 +8248,7 @@
       </c>
       <c r="H20" s="67" t="n">
         <f aca="false">Assumptions!$B$10</f>
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I20" s="67" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="J20" s="67" t="n">
         <f aca="false">F20*(1+G20)*H20-F20*G20*I20</f>
-        <v>15.048</v>
+        <v>17.232</v>
       </c>
       <c r="K20" s="64" t="s">
         <v>275</v>
@@ -8299,23 +8299,23 @@
       </c>
       <c r="V20" s="67" t="n">
         <f aca="false">J20+O20+R20+T20+U20</f>
-        <v>20.6693055555556</v>
+        <v>22.8533055555556</v>
       </c>
       <c r="W20" s="67" t="n">
         <f aca="false">V20*Assumptions!$B$39</f>
-        <v>1.65354444444444</v>
+        <v>1.82826444444444</v>
       </c>
       <c r="X20" s="67" t="n">
         <f aca="false">(V20+W20)*Assumptions!$B$40</f>
-        <v>2.232285</v>
+        <v>2.468157</v>
       </c>
       <c r="Y20" s="72" t="n">
         <f aca="false">V20+W20+X20</f>
-        <v>24.555135</v>
+        <v>27.149727</v>
       </c>
       <c r="Z20" s="72" t="n">
         <f aca="false">Y20*E20</f>
-        <v>49.11027</v>
+        <v>54.299454</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8342,7 +8342,7 @@
       </c>
       <c r="H21" s="76" t="n">
         <f aca="false">Assumptions!$B$10</f>
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I21" s="76" t="n">
         <f aca="false">Assumptions!$B$17</f>
@@ -8350,7 +8350,7 @@
       </c>
       <c r="J21" s="76" t="n">
         <f aca="false">F21*(1+G21)*H21-F21*G21*I21</f>
-        <v>15.048</v>
+        <v>17.232</v>
       </c>
       <c r="K21" s="75" t="s">
         <v>275</v>
@@ -8393,23 +8393,23 @@
       </c>
       <c r="V21" s="76" t="n">
         <f aca="false">J21+O21+R21+T21+U21</f>
-        <v>20.6693055555556</v>
+        <v>22.8533055555556</v>
       </c>
       <c r="W21" s="76" t="n">
         <f aca="false">V21*Assumptions!$B$39</f>
-        <v>1.65354444444444</v>
+        <v>1.82826444444444</v>
       </c>
       <c r="X21" s="76" t="n">
         <f aca="false">(V21+W21)*Assumptions!$B$40</f>
-        <v>2.232285</v>
+        <v>2.468157</v>
       </c>
       <c r="Y21" s="78" t="n">
         <f aca="false">V21+W21+X21</f>
-        <v>24.555135</v>
+        <v>27.149727</v>
       </c>
       <c r="Z21" s="78" t="n">
         <f aca="false">Y21*E21</f>
-        <v>49.11027</v>
+        <v>54.299454</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8445,7 +8445,7 @@
       <c r="Y22" s="36"/>
       <c r="Z22" s="81" t="n">
         <f aca="false">SUM(Z4:Z21)</f>
-        <v>2276.1288891</v>
+        <v>2495.4976035</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bumper should-cost: paint & tooling deep-dive sections in Methodology
Two new Methodology sections between the 8-step method and the Q&A, all
values live: PAINT (P1-P6: material basis 0.40 l/bumper, booth-hour logic,
robotic manning, jig amortisation, overhead/markups, 280-380 benchmark
sanity check and the moulded-in-colour lever) and TOOLING (T1-T6: 7.28 Cr
investment scope, fascia mould 1.8 Cr vs 1.5-2.5 Cr India benchmark,
amortisation formula, family-tool per-piece logic, 360k-shot life check
vs 500k-1M capability, 174/vehicle total and the OEM-paid alternative).
Tool costs double-checked line by line; totals unchanged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142L4rKS2AV8rxQTDWMs7dy
</commit_message>
<xml_diff>
--- a/Altroz-Front-Bumper-Should-Cost-India.xlsx
+++ b/Altroz-Front-Bumper-Should-Cost-India.xlsx
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="398">
   <si>
     <t xml:space="preserve">TATA ALTROZ — FRONT BUMPER ASSEMBLY  ·  SHOULD-COST SUMMARY (INDIA)</t>
   </si>
@@ -395,6 +395,150 @@
     <t xml:space="preserve">TOTAL should cost ₹</t>
   </si>
   <si>
+    <t xml:space="preserve">DEEP-DIVE: PAINT COST — how the body-colour paint line item is built (all values LIVE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paint material — ₹160/bumper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primer + basecoat + clearcoat + thinners, materials only. Basis: ~0.40 litre of mixed paint per bumper at OEM robotic transfer efficiency, ~₹400/litre blended across the three coats. This is an input (Assumptions B18) — put in our paint shop's actual chemical cost per unit if we have it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paint material ₹</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paint line time — the biggest piece</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A conveyorised robotic bumper paint line costs ₹2,400/hr all-in: booth depreciation, ventilation and booth energy (the big consumers), robots, sludge/filter handling. At ~110 s effective takt per bumper: 110 ÷ 3600 × 2,400. Painting is a PROCESS cost — the booth hour, not the paint, is what you pay for.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line cost ₹/bumper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labour — small by design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Robotic line: 0.5 manning (loader/unloader shared) × skilled rate ₹260/hr × 110 s. Manual painting would triple this and hurt quality consistency.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paint labour ₹</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paint jigs &amp; masks — ₹60 L amortised</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bumper-specific carriers, masking jigs and skids, spread over volume × years like any tool: ₹60 L ÷ 360,000 bumpers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jig amortisation ₹</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overhead + markups</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factory overhead 40% on the conversion (line + labour, NOT on paint material), then SG&amp;A 8% and profit 10% like every other line.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paint line item ₹</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sanity checks &amp; the lever</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checks: India tier-1 bumper paint jobs benchmark at ₹280–₹380 all-in — we sit mid-range. First-run yield ~92–95% is assumed inside the line rate. The lever: if the fascia can be moulded-in-colour (masterbatch), this entire line item disappears — savings idea #1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEEP-DIVE: TOOLING — what is in the investment and how it reaches the piece price (all values LIVE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What the investment covers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Injection moulds for every plastic part, the EPP shape mould, rollform tooling for the beam, the progressive die for crash-box brackets, weld fixtures, paint jigs, assembly fixtures and end-of-line equipment. Parts tooling ₹6.28 Cr + assembly fixtures ₹0.40 Cr + EOL equipment ₹0.60 Cr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total investment ₹</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The biggest tool — fascia mould ₹1.8 Cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A single-cavity hot-runner mould for a 1500-tonne press, ~3.6 kg part with texture and complex shut-offs. India toolroom benchmark: ₹1.5–2.5 Cr (the same tool imported from Japan/Korea would be 2–3×). Next: paint jigs ₹60 L, grille moulds ₹50 L each, beam rollform set ₹50 L, EPP mould ₹35 L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fascia mould ₹</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The amortisation formula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool ÷ (annual volume × years × parts per vehicle). Fascia: ₹1.8 Cr ÷ (72,000 × 5 × 1) = ₹50.00 per part. Every tool row uses the same formula — column T on Parts Costing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fascia amort ₹/pc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Family tools cost less per piece</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LH+RH parts share one mould and come out in the same shot, so the tool spreads over twice the pieces: side brackets ₹18 L ÷ (72,000 × 5 × 2) = ₹2.50/pc. The sensor holder runs 4 cavities for the same reason.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Side-bracket amort ₹/pc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool life check — why 5 years is safe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 years × 72,000 = 360,000 shots on the fascia mould. A hardened hot-runner bumper mould is good for 500k–1M shots, so life does not limit the amortisation period; small tools are specified hardened (H13/P20) for the same duty.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What tooling adds to each vehicle — and who pays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summing column T × qty across all parts: the tooling inside the piece prices. If the OEM pays tooling up-front instead (common for dedicated moulds), zero column S — piece prices drop by this amount and the ₹7.28 Cr becomes a separate one-time negotiation with tool-ownership rights.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tooling ₹/vehicle</t>
+  </si>
+  <si>
     <t xml:space="preserve">MANAGER Q&amp;A — the questions you will get, and the answers (live numbers in the right column)</t>
   </si>
   <si>
@@ -489,9 +633,6 @@
   </si>
   <si>
     <t xml:space="preserve">Body-colour painting is a process cost, not a material cost: a robotic paint line at ₹2,400/hr with booth energy and ventilation, ~110 s per bumper, plus overhead and margin on that conversion. If the fascia is supplied moulded-in-colour, delete the paint row — the model drops it cleanly.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paint line item ₹</t>
   </si>
   <si>
     <t xml:space="preserve">“4 parking sensors or 8?”</t>
@@ -1462,7 +1603,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="104">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1640,6 +1781,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="30" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="30" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5577,7 +5722,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -5772,38 +5917,34 @@
       <c r="C20" s="39"/>
       <c r="D20" s="39"/>
     </row>
-    <row r="21" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="45" t="s">
+    <row r="21" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="40" t="s">
         <v>114</v>
       </c>
-      <c r="B21" s="46" t="s">
+      <c r="B21" s="41" t="s">
         <v>115</v>
       </c>
-      <c r="C21" s="47" t="s">
+      <c r="C21" s="42" t="s">
         <v>116</v>
       </c>
-      <c r="D21" s="31"/>
-    </row>
-    <row r="22" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="48" t="s">
-        <v>114</v>
-      </c>
-      <c r="B22" s="49" t="s">
+      <c r="D21" s="43" t="s">
         <v>117</v>
       </c>
-      <c r="C22" s="50" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D22" s="44" t="n">
+        <f aca="false">Assumptions!$B$18</f>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="40" t="s">
         <v>118</v>
       </c>
-      <c r="D22" s="51"/>
-    </row>
-    <row r="23" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="B23" s="46" t="s">
+      <c r="B23" s="41" t="s">
         <v>119</v>
       </c>
-      <c r="C23" s="47" t="s">
+      <c r="C23" s="42" t="s">
         <v>120</v>
       </c>
       <c r="D23" s="43" t="s">
@@ -5812,200 +5953,446 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D24" s="44" t="n">
+        <f aca="false">'Parts Costing'!O5</f>
+        <v>73.3333333333333</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="B25" s="41" t="s">
+        <v>123</v>
+      </c>
+      <c r="C25" s="42" t="s">
+        <v>124</v>
+      </c>
+      <c r="D25" s="43" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D26" s="44" t="n">
+        <f aca="false">'Parts Costing'!R5</f>
+        <v>3.97222222222222</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="40" t="s">
+        <v>126</v>
+      </c>
+      <c r="B27" s="41" t="s">
+        <v>127</v>
+      </c>
+      <c r="C27" s="42" t="s">
+        <v>128</v>
+      </c>
+      <c r="D27" s="43" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D28" s="44" t="n">
+        <f aca="false">'Parts Costing'!T5</f>
+        <v>16.6666666666667</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="B29" s="41" t="s">
+        <v>131</v>
+      </c>
+      <c r="C29" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D29" s="43" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D30" s="44" t="n">
+        <f aca="false">'Parts Costing'!Y5</f>
+        <v>338.4546</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="B31" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="C31" s="42" t="s">
+        <v>136</v>
+      </c>
+      <c r="D31" s="31"/>
+    </row>
+    <row r="33" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="39" t="s">
+        <v>137</v>
+      </c>
+      <c r="B33" s="39"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="39"/>
+    </row>
+    <row r="34" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="40" t="s">
+        <v>138</v>
+      </c>
+      <c r="B34" s="41" t="s">
+        <v>139</v>
+      </c>
+      <c r="C34" s="42" t="s">
+        <v>140</v>
+      </c>
+      <c r="D34" s="43" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D35" s="45" t="n">
+        <f aca="false">Tooling!B7</f>
+        <v>72800000</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="40" t="s">
+        <v>142</v>
+      </c>
+      <c r="B36" s="41" t="s">
+        <v>143</v>
+      </c>
+      <c r="C36" s="42" t="s">
+        <v>144</v>
+      </c>
+      <c r="D36" s="43" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D37" s="45" t="n">
+        <f aca="false">'Parts Costing'!S4</f>
+        <v>18000000</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="40" t="s">
+        <v>146</v>
+      </c>
+      <c r="B38" s="41" t="s">
+        <v>147</v>
+      </c>
+      <c r="C38" s="42" t="s">
+        <v>148</v>
+      </c>
+      <c r="D38" s="43" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D39" s="44" t="n">
+        <f aca="false">'Parts Costing'!T4</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="40" t="s">
+        <v>150</v>
+      </c>
+      <c r="B40" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="C40" s="42" t="s">
+        <v>152</v>
+      </c>
+      <c r="D40" s="43" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D41" s="44" t="n">
+        <f aca="false">'Parts Costing'!T8</f>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="40" t="s">
+        <v>154</v>
+      </c>
+      <c r="B42" s="41" t="s">
+        <v>155</v>
+      </c>
+      <c r="C42" s="42" t="s">
+        <v>156</v>
+      </c>
+      <c r="D42" s="31"/>
+    </row>
+    <row r="43" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="40" t="s">
+        <v>157</v>
+      </c>
+      <c r="B43" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="C43" s="42" t="s">
+        <v>159</v>
+      </c>
+      <c r="D43" s="43" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D44" s="44" t="n">
+        <f aca="false">Summary!B105</f>
+        <v>174.444444444444</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="39" t="s">
+        <v>161</v>
+      </c>
+      <c r="B46" s="39"/>
+      <c r="C46" s="39"/>
+      <c r="D46" s="39"/>
+    </row>
+    <row r="47" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="B47" s="47" t="s">
+        <v>163</v>
+      </c>
+      <c r="C47" s="48" t="s">
+        <v>164</v>
+      </c>
+      <c r="D47" s="31"/>
+    </row>
+    <row r="48" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="B48" s="50" t="s">
+        <v>165</v>
+      </c>
+      <c r="C48" s="51" t="s">
+        <v>166</v>
+      </c>
+      <c r="D48" s="52"/>
+    </row>
+    <row r="49" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="B49" s="47" t="s">
+        <v>167</v>
+      </c>
+      <c r="C49" s="48" t="s">
+        <v>168</v>
+      </c>
+      <c r="D49" s="43" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D50" s="44" t="n">
         <f aca="false">Summary!D10</f>
         <v>2786.48413127778</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="B25" s="46" t="s">
-        <v>122</v>
-      </c>
-      <c r="C25" s="47" t="s">
-        <v>123</v>
-      </c>
-      <c r="D25" s="43" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D26" s="52" t="n">
+    <row r="51" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="B51" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="C51" s="48" t="s">
+        <v>171</v>
+      </c>
+      <c r="D51" s="43" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D52" s="53" t="n">
         <f aca="false">Assumptions!$B$4</f>
         <v>72000</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="B27" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="C27" s="47" t="s">
-        <v>126</v>
-      </c>
-      <c r="D27" s="43" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D28" s="44" t="n">
+    <row r="53" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="B53" s="47" t="s">
+        <v>173</v>
+      </c>
+      <c r="C53" s="48" t="s">
+        <v>174</v>
+      </c>
+      <c r="D53" s="43" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D54" s="44" t="n">
         <f aca="false">Tooling!B7</f>
         <v>72800000</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="B29" s="46" t="s">
-        <v>128</v>
-      </c>
-      <c r="C29" s="47" t="s">
-        <v>129</v>
-      </c>
-      <c r="D29" s="31"/>
-    </row>
-    <row r="30" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="48" t="s">
-        <v>114</v>
-      </c>
-      <c r="B30" s="49" t="s">
-        <v>130</v>
-      </c>
-      <c r="C30" s="50" t="s">
-        <v>131</v>
-      </c>
-      <c r="D30" s="51"/>
-    </row>
-    <row r="31" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="B31" s="46" t="s">
-        <v>132</v>
-      </c>
-      <c r="C31" s="47" t="s">
-        <v>133</v>
-      </c>
-      <c r="D31" s="31"/>
-    </row>
-    <row r="32" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="48" t="s">
-        <v>114</v>
-      </c>
-      <c r="B32" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="C32" s="50" t="s">
-        <v>135</v>
-      </c>
-      <c r="D32" s="51"/>
-    </row>
-    <row r="33" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="B33" s="46" t="s">
-        <v>136</v>
-      </c>
-      <c r="C33" s="47" t="s">
-        <v>137</v>
-      </c>
-      <c r="D33" s="31"/>
-    </row>
-    <row r="34" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="48" t="s">
-        <v>114</v>
-      </c>
-      <c r="B34" s="49" t="s">
-        <v>138</v>
-      </c>
-      <c r="C34" s="50" t="s">
-        <v>139</v>
-      </c>
-      <c r="D34" s="53" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D35" s="44" t="n">
+    <row r="55" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="B55" s="47" t="s">
+        <v>176</v>
+      </c>
+      <c r="C55" s="48" t="s">
+        <v>177</v>
+      </c>
+      <c r="D55" s="31"/>
+    </row>
+    <row r="56" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="B56" s="50" t="s">
+        <v>178</v>
+      </c>
+      <c r="C56" s="51" t="s">
+        <v>179</v>
+      </c>
+      <c r="D56" s="52"/>
+    </row>
+    <row r="57" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="B57" s="47" t="s">
+        <v>180</v>
+      </c>
+      <c r="C57" s="48" t="s">
+        <v>181</v>
+      </c>
+      <c r="D57" s="31"/>
+    </row>
+    <row r="58" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="B58" s="50" t="s">
+        <v>182</v>
+      </c>
+      <c r="C58" s="51" t="s">
+        <v>183</v>
+      </c>
+      <c r="D58" s="52"/>
+    </row>
+    <row r="59" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="B59" s="47" t="s">
+        <v>184</v>
+      </c>
+      <c r="C59" s="48" t="s">
+        <v>185</v>
+      </c>
+      <c r="D59" s="31"/>
+    </row>
+    <row r="60" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="B60" s="50" t="s">
+        <v>186</v>
+      </c>
+      <c r="C60" s="51" t="s">
+        <v>187</v>
+      </c>
+      <c r="D60" s="54" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D61" s="44" t="n">
         <f aca="false">'Parts Costing'!Y4+'Parts Costing'!Y5</f>
         <v>1136.20683</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="48" t="s">
-        <v>114</v>
-      </c>
-      <c r="B36" s="49" t="s">
-        <v>141</v>
-      </c>
-      <c r="C36" s="50" t="s">
-        <v>142</v>
-      </c>
-      <c r="D36" s="51"/>
-    </row>
-    <row r="37" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="B37" s="46" t="s">
-        <v>143</v>
-      </c>
-      <c r="C37" s="47" t="s">
-        <v>144</v>
-      </c>
-      <c r="D37" s="43" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D38" s="44" t="n">
+    <row r="62" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="B62" s="50" t="s">
+        <v>189</v>
+      </c>
+      <c r="C62" s="51" t="s">
+        <v>190</v>
+      </c>
+      <c r="D62" s="52"/>
+    </row>
+    <row r="63" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="B63" s="47" t="s">
+        <v>191</v>
+      </c>
+      <c r="C63" s="48" t="s">
+        <v>192</v>
+      </c>
+      <c r="D63" s="43" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D64" s="44" t="n">
         <f aca="false">'Parts Costing'!Y5</f>
         <v>338.4546</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="B39" s="46" t="s">
-        <v>146</v>
-      </c>
-      <c r="C39" s="47" t="s">
-        <v>147</v>
-      </c>
-      <c r="D39" s="31"/>
-    </row>
-    <row r="40" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="48" t="s">
-        <v>114</v>
-      </c>
-      <c r="B40" s="49" t="s">
-        <v>148</v>
-      </c>
-      <c r="C40" s="50" t="s">
-        <v>149</v>
-      </c>
-      <c r="D40" s="53" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D41" s="44" t="n">
+    <row r="65" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="B65" s="47" t="s">
+        <v>193</v>
+      </c>
+      <c r="C65" s="48" t="s">
+        <v>194</v>
+      </c>
+      <c r="D65" s="31"/>
+    </row>
+    <row r="66" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="B66" s="50" t="s">
+        <v>195</v>
+      </c>
+      <c r="C66" s="51" t="s">
+        <v>196</v>
+      </c>
+      <c r="D66" s="54" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D67" s="44" t="n">
         <f aca="false">Summary!D69</f>
         <v>875.5276952</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A46:D46"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -6033,7 +6420,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>151</v>
+        <v>198</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6041,508 +6428,508 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>152</v>
+        <v>199</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="54" t="s">
-        <v>153</v>
-      </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
+      <c r="A3" s="55" t="s">
+        <v>200</v>
+      </c>
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="55" t="s">
-        <v>154</v>
-      </c>
-      <c r="B4" s="56" t="n">
+      <c r="A4" s="56" t="s">
+        <v>201</v>
+      </c>
+      <c r="B4" s="57" t="n">
         <v>72000</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>155</v>
+        <v>202</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>156</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="55" t="s">
-        <v>157</v>
-      </c>
-      <c r="B5" s="57" t="n">
+      <c r="A5" s="56" t="s">
+        <v>204</v>
+      </c>
+      <c r="B5" s="58" t="n">
         <v>5</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>158</v>
+        <v>205</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="55" t="s">
-        <v>160</v>
-      </c>
-      <c r="B6" s="57" t="s">
-        <v>161</v>
+      <c r="A6" s="56" t="s">
+        <v>207</v>
+      </c>
+      <c r="B6" s="58" t="s">
+        <v>208</v>
       </c>
       <c r="C6" s="23"/>
       <c r="D6" s="23" t="s">
-        <v>162</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="55" t="s">
-        <v>163</v>
-      </c>
-      <c r="B7" s="56" t="n">
+      <c r="A7" s="56" t="s">
+        <v>210</v>
+      </c>
+      <c r="B7" s="57" t="n">
         <v>106</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>164</v>
+        <v>211</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>165</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="54" t="s">
-        <v>166</v>
-      </c>
-      <c r="B9" s="54"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
+      <c r="A9" s="55" t="s">
+        <v>213</v>
+      </c>
+      <c r="B9" s="55"/>
+      <c r="C9" s="55"/>
+      <c r="D9" s="55"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="55" t="s">
-        <v>167</v>
-      </c>
-      <c r="B10" s="58" t="n">
+      <c r="A10" s="56" t="s">
+        <v>214</v>
+      </c>
+      <c r="B10" s="59" t="n">
         <v>112</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>169</v>
+        <v>216</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="55" t="s">
-        <v>170</v>
-      </c>
-      <c r="B11" s="58" t="n">
+      <c r="A11" s="56" t="s">
+        <v>217</v>
+      </c>
+      <c r="B11" s="59" t="n">
         <v>155</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="55" t="s">
-        <v>172</v>
-      </c>
-      <c r="B12" s="58" t="n">
+      <c r="A12" s="56" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12" s="59" t="n">
         <v>158</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>173</v>
+        <v>220</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="55" t="s">
-        <v>174</v>
-      </c>
-      <c r="B13" s="58" t="n">
+      <c r="A13" s="56" t="s">
+        <v>221</v>
+      </c>
+      <c r="B13" s="59" t="n">
         <v>700</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>175</v>
+        <v>222</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="55" t="s">
-        <v>176</v>
-      </c>
-      <c r="B14" s="58" t="n">
+      <c r="A14" s="56" t="s">
+        <v>223</v>
+      </c>
+      <c r="B14" s="59" t="n">
         <v>210</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>177</v>
+        <v>224</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="55" t="s">
-        <v>178</v>
-      </c>
-      <c r="B15" s="58" t="n">
+      <c r="A15" s="56" t="s">
+        <v>225</v>
+      </c>
+      <c r="B15" s="59" t="n">
         <v>68</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>179</v>
+        <v>226</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="55" t="s">
-        <v>180</v>
-      </c>
-      <c r="B16" s="58" t="n">
+      <c r="A16" s="56" t="s">
+        <v>227</v>
+      </c>
+      <c r="B16" s="59" t="n">
         <v>32</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>181</v>
+        <v>228</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="55" t="s">
-        <v>182</v>
-      </c>
-      <c r="B17" s="58" t="n">
+      <c r="A17" s="56" t="s">
+        <v>229</v>
+      </c>
+      <c r="B17" s="59" t="n">
         <v>40</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>183</v>
+        <v>230</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="55" t="s">
-        <v>184</v>
-      </c>
-      <c r="B18" s="58" t="n">
+      <c r="A18" s="56" t="s">
+        <v>231</v>
+      </c>
+      <c r="B18" s="59" t="n">
         <v>160</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>185</v>
+        <v>232</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>186</v>
+        <v>233</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="54" t="s">
-        <v>187</v>
-      </c>
-      <c r="B20" s="54"/>
-      <c r="C20" s="54"/>
-      <c r="D20" s="54"/>
+      <c r="A20" s="55" t="s">
+        <v>234</v>
+      </c>
+      <c r="B20" s="55"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="55" t="s">
-        <v>188</v>
-      </c>
-      <c r="B21" s="59" t="n">
+      <c r="A21" s="56" t="s">
+        <v>235</v>
+      </c>
+      <c r="B21" s="60" t="n">
         <v>2100</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>189</v>
+        <v>236</v>
       </c>
       <c r="D21" s="23" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="56" t="s">
+        <v>238</v>
+      </c>
+      <c r="B22" s="60" t="n">
+        <v>1150</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="56" t="s">
+        <v>240</v>
+      </c>
+      <c r="B23" s="60" t="n">
+        <v>700</v>
+      </c>
+      <c r="C23" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="56" t="s">
+        <v>242</v>
+      </c>
+      <c r="B24" s="60" t="n">
+        <v>520</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="56" t="s">
+        <v>244</v>
+      </c>
+      <c r="B25" s="60" t="n">
+        <v>400</v>
+      </c>
+      <c r="C25" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="56" t="s">
+        <v>246</v>
+      </c>
+      <c r="B26" s="60" t="n">
+        <v>650</v>
+      </c>
+      <c r="C26" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="56" t="s">
+        <v>248</v>
+      </c>
+      <c r="B27" s="60" t="n">
+        <v>900</v>
+      </c>
+      <c r="C27" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="56" t="s">
+        <v>250</v>
+      </c>
+      <c r="B28" s="60" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C28" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="56" t="s">
+        <v>252</v>
+      </c>
+      <c r="B29" s="60" t="n">
+        <v>800</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="56" t="s">
+        <v>254</v>
+      </c>
+      <c r="B30" s="60" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C30" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="D30" s="23" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="55" t="s">
+        <v>256</v>
+      </c>
+      <c r="B32" s="55"/>
+      <c r="C32" s="55"/>
+      <c r="D32" s="55"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="56" t="s">
+        <v>257</v>
+      </c>
+      <c r="B33" s="60" t="n">
         <v>190</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="55" t="s">
-        <v>191</v>
-      </c>
-      <c r="B22" s="59" t="n">
-        <v>1150</v>
-      </c>
-      <c r="C22" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="D22" s="23" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="55" t="s">
-        <v>193</v>
-      </c>
-      <c r="B23" s="59" t="n">
-        <v>700</v>
-      </c>
-      <c r="C23" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="D23" s="23" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="55" t="s">
-        <v>195</v>
-      </c>
-      <c r="B24" s="59" t="n">
-        <v>520</v>
-      </c>
-      <c r="C24" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="D24" s="23" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="55" t="s">
-        <v>197</v>
-      </c>
-      <c r="B25" s="59" t="n">
-        <v>400</v>
-      </c>
-      <c r="C25" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="D25" s="23" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="55" t="s">
-        <v>199</v>
-      </c>
-      <c r="B26" s="59" t="n">
-        <v>650</v>
-      </c>
-      <c r="C26" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="D26" s="23" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="55" t="s">
-        <v>201</v>
-      </c>
-      <c r="B27" s="59" t="n">
-        <v>900</v>
-      </c>
-      <c r="C27" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="D27" s="23" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="55" t="s">
-        <v>203</v>
-      </c>
-      <c r="B28" s="59" t="n">
-        <v>1600</v>
-      </c>
-      <c r="C28" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="D28" s="23" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="55" t="s">
-        <v>205</v>
-      </c>
-      <c r="B29" s="59" t="n">
-        <v>800</v>
-      </c>
-      <c r="C29" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="D29" s="23" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="55" t="s">
-        <v>207</v>
-      </c>
-      <c r="B30" s="59" t="n">
-        <v>2400</v>
-      </c>
-      <c r="C30" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="D30" s="23" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="54" t="s">
-        <v>209</v>
-      </c>
-      <c r="B32" s="54"/>
-      <c r="C32" s="54"/>
-      <c r="D32" s="54"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="55" t="s">
-        <v>210</v>
-      </c>
-      <c r="B33" s="59" t="n">
-        <v>190</v>
-      </c>
       <c r="C33" s="23" t="s">
-        <v>189</v>
+        <v>236</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>211</v>
+        <v>258</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="55" t="s">
-        <v>212</v>
-      </c>
-      <c r="B34" s="59" t="n">
+      <c r="A34" s="56" t="s">
+        <v>259</v>
+      </c>
+      <c r="B34" s="60" t="n">
         <v>260</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>189</v>
+        <v>236</v>
       </c>
       <c r="D34" s="23"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="55" t="s">
-        <v>213</v>
-      </c>
-      <c r="B35" s="59" t="n">
+      <c r="A35" s="56" t="s">
+        <v>260</v>
+      </c>
+      <c r="B35" s="60" t="n">
         <v>230</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>189</v>
+        <v>236</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>214</v>
+        <v>261</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="54" t="s">
-        <v>215</v>
-      </c>
-      <c r="B37" s="54"/>
-      <c r="C37" s="54"/>
-      <c r="D37" s="54"/>
+      <c r="A37" s="55" t="s">
+        <v>262</v>
+      </c>
+      <c r="B37" s="55"/>
+      <c r="C37" s="55"/>
+      <c r="D37" s="55"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="55" t="s">
-        <v>216</v>
-      </c>
-      <c r="B38" s="60" t="n">
+      <c r="A38" s="56" t="s">
+        <v>263</v>
+      </c>
+      <c r="B38" s="61" t="n">
         <v>0.4</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>217</v>
+        <v>264</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>218</v>
+        <v>265</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="55" t="s">
+      <c r="A39" s="56" t="s">
         <v>79</v>
       </c>
-      <c r="B39" s="60" t="n">
+      <c r="B39" s="61" t="n">
         <v>0.08</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>217</v>
+        <v>264</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>219</v>
+        <v>266</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="55" t="s">
+      <c r="A40" s="56" t="s">
         <v>80</v>
       </c>
-      <c r="B40" s="60" t="n">
+      <c r="B40" s="61" t="n">
         <v>0.1</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>217</v>
+        <v>264</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>220</v>
+        <v>267</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="55" t="s">
-        <v>221</v>
-      </c>
-      <c r="B41" s="60" t="n">
+      <c r="A41" s="56" t="s">
+        <v>268</v>
+      </c>
+      <c r="B41" s="61" t="n">
         <v>0.03</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>217</v>
+        <v>264</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>222</v>
+        <v>269</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="55" t="s">
-        <v>223</v>
-      </c>
-      <c r="B42" s="60" t="n">
+      <c r="A42" s="56" t="s">
+        <v>270</v>
+      </c>
+      <c r="B42" s="61" t="n">
         <v>0.45</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>217</v>
+        <v>264</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>224</v>
+        <v>271</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="55" t="s">
-        <v>225</v>
-      </c>
-      <c r="B43" s="58" t="n">
+      <c r="A43" s="56" t="s">
+        <v>272</v>
+      </c>
+      <c r="B43" s="59" t="n">
         <v>55</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>185</v>
+        <v>232</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>226</v>
+        <v>273</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="55" t="s">
-        <v>227</v>
-      </c>
-      <c r="B44" s="61" t="n">
+      <c r="A44" s="56" t="s">
+        <v>274</v>
+      </c>
+      <c r="B44" s="62" t="n">
         <v>4</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>228</v>
+        <v>275</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>229</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -6599,7 +6986,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>230</v>
+        <v>277</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6629,7 +7016,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>231</v>
+        <v>278</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6659,10 +7046,10 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>232</v>
+        <v>279</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>233</v>
+        <v>280</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>53</v>
@@ -6671,1743 +7058,1743 @@
         <v>50</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>234</v>
+        <v>281</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>235</v>
+        <v>282</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>236</v>
+        <v>283</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>237</v>
+        <v>284</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>238</v>
+        <v>285</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>239</v>
+        <v>286</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>240</v>
+        <v>287</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>241</v>
+        <v>288</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>242</v>
+        <v>289</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>243</v>
+        <v>290</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>244</v>
+        <v>291</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>245</v>
+        <v>292</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>246</v>
+        <v>293</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>247</v>
+        <v>294</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>248</v>
+        <v>295</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>249</v>
+        <v>296</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>250</v>
+        <v>297</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>251</v>
+        <v>298</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>252</v>
+        <v>299</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>253</v>
+        <v>300</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>254</v>
+        <v>301</v>
       </c>
       <c r="Z3" s="3" t="s">
-        <v>255</v>
+        <v>302</v>
       </c>
       <c r="AA3" s="3" t="s">
-        <v>256</v>
+        <v>303</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="62" t="n">
+      <c r="A4" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="63" t="s">
-        <v>257</v>
-      </c>
-      <c r="C4" s="64" t="s">
-        <v>258</v>
-      </c>
-      <c r="D4" s="64" t="s">
-        <v>259</v>
-      </c>
-      <c r="E4" s="62" t="n">
+      <c r="B4" s="64" t="s">
+        <v>304</v>
+      </c>
+      <c r="C4" s="65" t="s">
+        <v>305</v>
+      </c>
+      <c r="D4" s="65" t="s">
+        <v>306</v>
+      </c>
+      <c r="E4" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="65" t="n">
+      <c r="F4" s="66" t="n">
         <v>3.6</v>
       </c>
-      <c r="G4" s="66" t="n">
+      <c r="G4" s="67" t="n">
         <v>0.04</v>
       </c>
-      <c r="H4" s="67" t="n">
+      <c r="H4" s="68" t="n">
         <f aca="false">Assumptions!$B$11</f>
         <v>155</v>
       </c>
-      <c r="I4" s="67" t="n">
+      <c r="I4" s="68" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J4" s="67" t="n">
+      <c r="J4" s="68" t="n">
         <f aca="false">F4*(1+G4)*H4-F4*G4*I4</f>
         <v>574.56</v>
       </c>
-      <c r="K4" s="64" t="s">
-        <v>260</v>
-      </c>
-      <c r="L4" s="68" t="n">
+      <c r="K4" s="65" t="s">
+        <v>307</v>
+      </c>
+      <c r="L4" s="69" t="n">
         <f aca="false">Assumptions!$B$21</f>
         <v>2100</v>
       </c>
-      <c r="M4" s="69" t="n">
+      <c r="M4" s="70" t="n">
         <v>55</v>
       </c>
-      <c r="N4" s="70" t="n">
+      <c r="N4" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="O4" s="67" t="n">
+      <c r="O4" s="68" t="n">
         <f aca="false">M4*L4/3600/N4</f>
         <v>32.0833333333333</v>
       </c>
-      <c r="P4" s="70" t="n">
+      <c r="P4" s="71" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q4" s="68" t="n">
+      <c r="Q4" s="69" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R4" s="67" t="n">
+      <c r="R4" s="68" t="n">
         <f aca="false">M4*P4*Q4/3600/N4</f>
         <v>1.45138888888889</v>
       </c>
-      <c r="S4" s="71" t="n">
+      <c r="S4" s="72" t="n">
         <v>18000000</v>
       </c>
-      <c r="T4" s="67" t="n">
+      <c r="T4" s="68" t="n">
         <f aca="false">S4/(Assumptions!$B$4*Assumptions!$B$5*E4)</f>
         <v>50</v>
       </c>
-      <c r="U4" s="67" t="n">
+      <c r="U4" s="68" t="n">
         <f aca="false">(O4+R4)*Assumptions!$B$38</f>
         <v>13.4138888888889</v>
       </c>
-      <c r="V4" s="67" t="n">
+      <c r="V4" s="68" t="n">
         <f aca="false">J4+O4+R4+T4+U4</f>
         <v>671.508611111111</v>
       </c>
-      <c r="W4" s="67" t="n">
+      <c r="W4" s="68" t="n">
         <f aca="false">V4*Assumptions!$B$39</f>
         <v>53.7206888888889</v>
       </c>
-      <c r="X4" s="67" t="n">
+      <c r="X4" s="68" t="n">
         <f aca="false">(V4+W4)*Assumptions!$B$40</f>
         <v>72.52293</v>
       </c>
-      <c r="Y4" s="72" t="n">
+      <c r="Y4" s="73" t="n">
         <f aca="false">V4+W4+X4</f>
         <v>797.75223</v>
       </c>
-      <c r="Z4" s="72" t="n">
+      <c r="Z4" s="73" t="n">
         <f aca="false">Y4*E4</f>
         <v>797.75223</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="73" t="n">
+      <c r="A5" s="74" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="74" t="s">
-        <v>261</v>
-      </c>
-      <c r="C5" s="75" t="s">
-        <v>262</v>
-      </c>
-      <c r="D5" s="75" t="s">
-        <v>263</v>
-      </c>
-      <c r="E5" s="73" t="n">
+      <c r="B5" s="75" t="s">
+        <v>308</v>
+      </c>
+      <c r="C5" s="76" t="s">
+        <v>309</v>
+      </c>
+      <c r="D5" s="76" t="s">
+        <v>310</v>
+      </c>
+      <c r="E5" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="73"/>
-      <c r="G5" s="73"/>
-      <c r="H5" s="73"/>
-      <c r="I5" s="73"/>
-      <c r="J5" s="76" t="n">
+      <c r="F5" s="74"/>
+      <c r="G5" s="74"/>
+      <c r="H5" s="74"/>
+      <c r="I5" s="74"/>
+      <c r="J5" s="77" t="n">
         <f aca="false">Assumptions!$B$18</f>
         <v>160</v>
       </c>
-      <c r="K5" s="75" t="s">
-        <v>264</v>
-      </c>
-      <c r="L5" s="77" t="n">
+      <c r="K5" s="76" t="s">
+        <v>311</v>
+      </c>
+      <c r="L5" s="78" t="n">
         <f aca="false">Assumptions!$B$30</f>
         <v>2400</v>
       </c>
-      <c r="M5" s="69" t="n">
+      <c r="M5" s="70" t="n">
         <v>110</v>
       </c>
-      <c r="N5" s="70" t="n">
+      <c r="N5" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="O5" s="76" t="n">
+      <c r="O5" s="77" t="n">
         <f aca="false">M5*L5/3600/N5</f>
         <v>73.3333333333333</v>
       </c>
-      <c r="P5" s="70" t="n">
+      <c r="P5" s="71" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q5" s="77" t="n">
+      <c r="Q5" s="78" t="n">
         <f aca="false">Assumptions!$B$34</f>
         <v>260</v>
       </c>
-      <c r="R5" s="76" t="n">
+      <c r="R5" s="77" t="n">
         <f aca="false">M5*P5*Q5/3600/N5</f>
         <v>3.97222222222222</v>
       </c>
-      <c r="S5" s="71" t="n">
+      <c r="S5" s="72" t="n">
         <v>6000000</v>
       </c>
-      <c r="T5" s="76" t="n">
+      <c r="T5" s="77" t="n">
         <f aca="false">S5/(Assumptions!$B$4*Assumptions!$B$5*E5)</f>
         <v>16.6666666666667</v>
       </c>
-      <c r="U5" s="76" t="n">
+      <c r="U5" s="77" t="n">
         <f aca="false">(O5+R5)*Assumptions!$B$38</f>
         <v>30.9222222222222</v>
       </c>
-      <c r="V5" s="76" t="n">
+      <c r="V5" s="77" t="n">
         <f aca="false">J5+O5+R5+T5+U5</f>
         <v>284.894444444444</v>
       </c>
-      <c r="W5" s="76" t="n">
+      <c r="W5" s="77" t="n">
         <f aca="false">V5*Assumptions!$B$39</f>
         <v>22.7915555555556</v>
       </c>
-      <c r="X5" s="76" t="n">
+      <c r="X5" s="77" t="n">
         <f aca="false">(V5+W5)*Assumptions!$B$40</f>
         <v>30.7686</v>
       </c>
-      <c r="Y5" s="78" t="n">
+      <c r="Y5" s="79" t="n">
         <f aca="false">V5+W5+X5</f>
         <v>338.4546</v>
       </c>
-      <c r="Z5" s="78" t="n">
+      <c r="Z5" s="79" t="n">
         <f aca="false">Y5*E5</f>
         <v>338.4546</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="62" t="n">
+      <c r="A6" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="63" t="s">
-        <v>265</v>
-      </c>
-      <c r="C6" s="64" t="s">
-        <v>258</v>
-      </c>
-      <c r="D6" s="64" t="s">
-        <v>266</v>
-      </c>
-      <c r="E6" s="62" t="n">
+      <c r="B6" s="64" t="s">
+        <v>312</v>
+      </c>
+      <c r="C6" s="65" t="s">
+        <v>305</v>
+      </c>
+      <c r="D6" s="65" t="s">
+        <v>313</v>
+      </c>
+      <c r="E6" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="65" t="n">
+      <c r="F6" s="66" t="n">
         <v>0.45</v>
       </c>
-      <c r="G6" s="66" t="n">
+      <c r="G6" s="67" t="n">
         <v>0.05</v>
       </c>
-      <c r="H6" s="67" t="n">
+      <c r="H6" s="68" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>112</v>
       </c>
-      <c r="I6" s="67" t="n">
+      <c r="I6" s="68" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J6" s="67" t="n">
+      <c r="J6" s="68" t="n">
         <f aca="false">F6*(1+G6)*H6-F6*G6*I6</f>
         <v>52.02</v>
       </c>
-      <c r="K6" s="64" t="s">
-        <v>267</v>
-      </c>
-      <c r="L6" s="68" t="n">
+      <c r="K6" s="65" t="s">
+        <v>314</v>
+      </c>
+      <c r="L6" s="69" t="n">
         <f aca="false">Assumptions!$B$23</f>
         <v>700</v>
       </c>
-      <c r="M6" s="69" t="n">
+      <c r="M6" s="70" t="n">
         <v>32</v>
       </c>
-      <c r="N6" s="70" t="n">
+      <c r="N6" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="O6" s="67" t="n">
+      <c r="O6" s="68" t="n">
         <f aca="false">M6*L6/3600/N6</f>
         <v>6.22222222222222</v>
       </c>
-      <c r="P6" s="70" t="n">
+      <c r="P6" s="71" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q6" s="68" t="n">
+      <c r="Q6" s="69" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R6" s="67" t="n">
+      <c r="R6" s="68" t="n">
         <f aca="false">M6*P6*Q6/3600/N6</f>
         <v>0.557333333333333</v>
       </c>
-      <c r="S6" s="71" t="n">
+      <c r="S6" s="72" t="n">
         <v>5000000</v>
       </c>
-      <c r="T6" s="67" t="n">
+      <c r="T6" s="68" t="n">
         <f aca="false">S6/(Assumptions!$B$4*Assumptions!$B$5*E6)</f>
         <v>13.8888888888889</v>
       </c>
-      <c r="U6" s="67" t="n">
+      <c r="U6" s="68" t="n">
         <f aca="false">(O6+R6)*Assumptions!$B$38</f>
         <v>2.71182222222222</v>
       </c>
-      <c r="V6" s="67" t="n">
+      <c r="V6" s="68" t="n">
         <f aca="false">J6+O6+R6+T6+U6</f>
         <v>75.4002666666667</v>
       </c>
-      <c r="W6" s="67" t="n">
+      <c r="W6" s="68" t="n">
         <f aca="false">V6*Assumptions!$B$39</f>
         <v>6.03202133333333</v>
       </c>
-      <c r="X6" s="67" t="n">
+      <c r="X6" s="68" t="n">
         <f aca="false">(V6+W6)*Assumptions!$B$40</f>
         <v>8.1432288</v>
       </c>
-      <c r="Y6" s="72" t="n">
+      <c r="Y6" s="73" t="n">
         <f aca="false">V6+W6+X6</f>
         <v>89.5755168</v>
       </c>
-      <c r="Z6" s="72" t="n">
+      <c r="Z6" s="73" t="n">
         <f aca="false">Y6*E6</f>
         <v>89.5755168</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="73" t="n">
+      <c r="A7" s="74" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="74" t="s">
-        <v>268</v>
-      </c>
-      <c r="C7" s="75" t="s">
-        <v>258</v>
-      </c>
-      <c r="D7" s="75" t="s">
-        <v>266</v>
-      </c>
-      <c r="E7" s="73" t="n">
+      <c r="B7" s="75" t="s">
+        <v>315</v>
+      </c>
+      <c r="C7" s="76" t="s">
+        <v>305</v>
+      </c>
+      <c r="D7" s="76" t="s">
+        <v>313</v>
+      </c>
+      <c r="E7" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="65" t="n">
+      <c r="F7" s="66" t="n">
         <v>0.55</v>
       </c>
-      <c r="G7" s="66" t="n">
+      <c r="G7" s="67" t="n">
         <v>0.05</v>
       </c>
-      <c r="H7" s="76" t="n">
+      <c r="H7" s="77" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>112</v>
       </c>
-      <c r="I7" s="76" t="n">
+      <c r="I7" s="77" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J7" s="76" t="n">
+      <c r="J7" s="77" t="n">
         <f aca="false">F7*(1+G7)*H7-F7*G7*I7</f>
         <v>63.58</v>
       </c>
-      <c r="K7" s="75" t="s">
-        <v>267</v>
-      </c>
-      <c r="L7" s="77" t="n">
+      <c r="K7" s="76" t="s">
+        <v>314</v>
+      </c>
+      <c r="L7" s="78" t="n">
         <f aca="false">Assumptions!$B$23</f>
         <v>700</v>
       </c>
-      <c r="M7" s="69" t="n">
+      <c r="M7" s="70" t="n">
         <v>38</v>
       </c>
-      <c r="N7" s="70" t="n">
+      <c r="N7" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="O7" s="76" t="n">
+      <c r="O7" s="77" t="n">
         <f aca="false">M7*L7/3600/N7</f>
         <v>7.38888888888889</v>
       </c>
-      <c r="P7" s="70" t="n">
+      <c r="P7" s="71" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q7" s="77" t="n">
+      <c r="Q7" s="78" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R7" s="76" t="n">
+      <c r="R7" s="77" t="n">
         <f aca="false">M7*P7*Q7/3600/N7</f>
         <v>0.661833333333333</v>
       </c>
-      <c r="S7" s="71" t="n">
+      <c r="S7" s="72" t="n">
         <v>5000000</v>
       </c>
-      <c r="T7" s="76" t="n">
+      <c r="T7" s="77" t="n">
         <f aca="false">S7/(Assumptions!$B$4*Assumptions!$B$5*E7)</f>
         <v>13.8888888888889</v>
       </c>
-      <c r="U7" s="76" t="n">
+      <c r="U7" s="77" t="n">
         <f aca="false">(O7+R7)*Assumptions!$B$38</f>
         <v>3.22028888888889</v>
       </c>
-      <c r="V7" s="76" t="n">
+      <c r="V7" s="77" t="n">
         <f aca="false">J7+O7+R7+T7+U7</f>
         <v>88.7399</v>
       </c>
-      <c r="W7" s="76" t="n">
+      <c r="W7" s="77" t="n">
         <f aca="false">V7*Assumptions!$B$39</f>
         <v>7.099192</v>
       </c>
-      <c r="X7" s="76" t="n">
+      <c r="X7" s="77" t="n">
         <f aca="false">(V7+W7)*Assumptions!$B$40</f>
         <v>9.5839092</v>
       </c>
-      <c r="Y7" s="78" t="n">
+      <c r="Y7" s="79" t="n">
         <f aca="false">V7+W7+X7</f>
         <v>105.4230012</v>
       </c>
-      <c r="Z7" s="78" t="n">
+      <c r="Z7" s="79" t="n">
         <f aca="false">Y7*E7</f>
         <v>105.4230012</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="62" t="n">
+      <c r="A8" s="63" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="63" t="s">
-        <v>269</v>
-      </c>
-      <c r="C8" s="64" t="s">
-        <v>258</v>
-      </c>
-      <c r="D8" s="64" t="s">
-        <v>270</v>
-      </c>
-      <c r="E8" s="62" t="n">
+      <c r="B8" s="64" t="s">
+        <v>316</v>
+      </c>
+      <c r="C8" s="65" t="s">
+        <v>305</v>
+      </c>
+      <c r="D8" s="65" t="s">
+        <v>317</v>
+      </c>
+      <c r="E8" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="65" t="n">
+      <c r="F8" s="66" t="n">
         <v>0.12</v>
       </c>
-      <c r="G8" s="66" t="n">
+      <c r="G8" s="67" t="n">
         <v>0.04</v>
       </c>
-      <c r="H8" s="67" t="n">
+      <c r="H8" s="68" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>112</v>
       </c>
-      <c r="I8" s="67" t="n">
+      <c r="I8" s="68" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J8" s="67" t="n">
+      <c r="J8" s="68" t="n">
         <f aca="false">F8*(1+G8)*H8-F8*G8*I8</f>
         <v>13.7856</v>
       </c>
-      <c r="K8" s="64" t="s">
-        <v>271</v>
-      </c>
-      <c r="L8" s="68" t="n">
+      <c r="K8" s="65" t="s">
+        <v>318</v>
+      </c>
+      <c r="L8" s="69" t="n">
         <f aca="false">Assumptions!$B$25</f>
         <v>400</v>
       </c>
-      <c r="M8" s="69" t="n">
+      <c r="M8" s="70" t="n">
         <v>26</v>
       </c>
-      <c r="N8" s="70" t="n">
+      <c r="N8" s="71" t="n">
         <v>2</v>
       </c>
-      <c r="O8" s="67" t="n">
+      <c r="O8" s="68" t="n">
         <f aca="false">M8*L8/3600/N8</f>
         <v>1.44444444444444</v>
       </c>
-      <c r="P8" s="70" t="n">
+      <c r="P8" s="71" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q8" s="68" t="n">
+      <c r="Q8" s="69" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R8" s="67" t="n">
+      <c r="R8" s="68" t="n">
         <f aca="false">M8*P8*Q8/3600/N8</f>
         <v>0.171527777777778</v>
       </c>
-      <c r="S8" s="71" t="n">
+      <c r="S8" s="72" t="n">
         <v>1800000</v>
       </c>
-      <c r="T8" s="67" t="n">
+      <c r="T8" s="68" t="n">
         <f aca="false">S8/(Assumptions!$B$4*Assumptions!$B$5*E8)</f>
         <v>2.5</v>
       </c>
-      <c r="U8" s="67" t="n">
+      <c r="U8" s="68" t="n">
         <f aca="false">(O8+R8)*Assumptions!$B$38</f>
         <v>0.646388888888889</v>
       </c>
-      <c r="V8" s="67" t="n">
+      <c r="V8" s="68" t="n">
         <f aca="false">J8+O8+R8+T8+U8</f>
         <v>18.5479611111111</v>
       </c>
-      <c r="W8" s="67" t="n">
+      <c r="W8" s="68" t="n">
         <f aca="false">V8*Assumptions!$B$39</f>
         <v>1.48383688888889</v>
       </c>
-      <c r="X8" s="67" t="n">
+      <c r="X8" s="68" t="n">
         <f aca="false">(V8+W8)*Assumptions!$B$40</f>
         <v>2.0031798</v>
       </c>
-      <c r="Y8" s="72" t="n">
+      <c r="Y8" s="73" t="n">
         <f aca="false">V8+W8+X8</f>
         <v>22.0349778</v>
       </c>
-      <c r="Z8" s="72" t="n">
+      <c r="Z8" s="73" t="n">
         <f aca="false">Y8*E8</f>
         <v>44.0699556</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="73" t="n">
+      <c r="A9" s="74" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="74" t="s">
-        <v>272</v>
-      </c>
-      <c r="C9" s="75" t="s">
-        <v>258</v>
-      </c>
-      <c r="D9" s="75" t="s">
-        <v>270</v>
-      </c>
-      <c r="E9" s="73" t="n">
+      <c r="B9" s="75" t="s">
+        <v>319</v>
+      </c>
+      <c r="C9" s="76" t="s">
+        <v>305</v>
+      </c>
+      <c r="D9" s="76" t="s">
+        <v>317</v>
+      </c>
+      <c r="E9" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="65" t="n">
+      <c r="F9" s="66" t="n">
         <v>0.18</v>
       </c>
-      <c r="G9" s="66" t="n">
+      <c r="G9" s="67" t="n">
         <v>0.04</v>
       </c>
-      <c r="H9" s="76" t="n">
+      <c r="H9" s="77" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>112</v>
       </c>
-      <c r="I9" s="76" t="n">
+      <c r="I9" s="77" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J9" s="76" t="n">
+      <c r="J9" s="77" t="n">
         <f aca="false">F9*(1+G9)*H9-F9*G9*I9</f>
         <v>20.6784</v>
       </c>
-      <c r="K9" s="75" t="s">
-        <v>271</v>
-      </c>
-      <c r="L9" s="77" t="n">
+      <c r="K9" s="76" t="s">
+        <v>318</v>
+      </c>
+      <c r="L9" s="78" t="n">
         <f aca="false">Assumptions!$B$25</f>
         <v>400</v>
       </c>
-      <c r="M9" s="69" t="n">
+      <c r="M9" s="70" t="n">
         <v>28</v>
       </c>
-      <c r="N9" s="70" t="n">
+      <c r="N9" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="O9" s="76" t="n">
+      <c r="O9" s="77" t="n">
         <f aca="false">M9*L9/3600/N9</f>
         <v>3.11111111111111</v>
       </c>
-      <c r="P9" s="70" t="n">
+      <c r="P9" s="71" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q9" s="77" t="n">
+      <c r="Q9" s="78" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R9" s="76" t="n">
+      <c r="R9" s="77" t="n">
         <f aca="false">M9*P9*Q9/3600/N9</f>
         <v>0.369444444444444</v>
       </c>
-      <c r="S9" s="71" t="n">
+      <c r="S9" s="72" t="n">
         <v>1200000</v>
       </c>
-      <c r="T9" s="76" t="n">
+      <c r="T9" s="77" t="n">
         <f aca="false">S9/(Assumptions!$B$4*Assumptions!$B$5*E9)</f>
         <v>3.33333333333333</v>
       </c>
-      <c r="U9" s="76" t="n">
+      <c r="U9" s="77" t="n">
         <f aca="false">(O9+R9)*Assumptions!$B$38</f>
         <v>1.39222222222222</v>
       </c>
-      <c r="V9" s="76" t="n">
+      <c r="V9" s="77" t="n">
         <f aca="false">J9+O9+R9+T9+U9</f>
         <v>28.8845111111111</v>
       </c>
-      <c r="W9" s="76" t="n">
+      <c r="W9" s="77" t="n">
         <f aca="false">V9*Assumptions!$B$39</f>
         <v>2.31076088888889</v>
       </c>
-      <c r="X9" s="76" t="n">
+      <c r="X9" s="77" t="n">
         <f aca="false">(V9+W9)*Assumptions!$B$40</f>
         <v>3.1195272</v>
       </c>
-      <c r="Y9" s="78" t="n">
+      <c r="Y9" s="79" t="n">
         <f aca="false">V9+W9+X9</f>
         <v>34.3147992</v>
       </c>
-      <c r="Z9" s="78" t="n">
+      <c r="Z9" s="79" t="n">
         <f aca="false">Y9*E9</f>
         <v>34.3147992</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="62" t="n">
+      <c r="A10" s="63" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="63" t="s">
-        <v>273</v>
-      </c>
-      <c r="C10" s="64" t="s">
-        <v>258</v>
-      </c>
-      <c r="D10" s="64" t="s">
-        <v>274</v>
-      </c>
-      <c r="E10" s="62" t="n">
+      <c r="B10" s="64" t="s">
+        <v>320</v>
+      </c>
+      <c r="C10" s="65" t="s">
+        <v>305</v>
+      </c>
+      <c r="D10" s="65" t="s">
+        <v>321</v>
+      </c>
+      <c r="E10" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="65" t="n">
+      <c r="F10" s="66" t="n">
         <v>0.15</v>
       </c>
-      <c r="G10" s="66" t="n">
+      <c r="G10" s="67" t="n">
         <v>0.05</v>
       </c>
-      <c r="H10" s="67" t="n">
+      <c r="H10" s="68" t="n">
         <f aca="false">Assumptions!$B$12</f>
         <v>158</v>
       </c>
-      <c r="I10" s="67" t="n">
+      <c r="I10" s="68" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J10" s="67" t="n">
+      <c r="J10" s="68" t="n">
         <f aca="false">F10*(1+G10)*H10-F10*G10*I10</f>
         <v>24.585</v>
       </c>
-      <c r="K10" s="64" t="s">
-        <v>275</v>
-      </c>
-      <c r="L10" s="68" t="n">
+      <c r="K10" s="65" t="s">
+        <v>322</v>
+      </c>
+      <c r="L10" s="69" t="n">
         <f aca="false">Assumptions!$B$24</f>
         <v>520</v>
       </c>
-      <c r="M10" s="69" t="n">
+      <c r="M10" s="70" t="n">
         <v>34</v>
       </c>
-      <c r="N10" s="70" t="n">
+      <c r="N10" s="71" t="n">
         <v>2</v>
       </c>
-      <c r="O10" s="67" t="n">
+      <c r="O10" s="68" t="n">
         <f aca="false">M10*L10/3600/N10</f>
         <v>2.45555555555556</v>
       </c>
-      <c r="P10" s="70" t="n">
+      <c r="P10" s="71" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q10" s="68" t="n">
+      <c r="Q10" s="69" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R10" s="67" t="n">
+      <c r="R10" s="68" t="n">
         <f aca="false">M10*P10*Q10/3600/N10</f>
         <v>0.296083333333333</v>
       </c>
-      <c r="S10" s="71" t="n">
+      <c r="S10" s="72" t="n">
         <v>2800000</v>
       </c>
-      <c r="T10" s="67" t="n">
+      <c r="T10" s="68" t="n">
         <f aca="false">S10/(Assumptions!$B$4*Assumptions!$B$5*E10)</f>
         <v>3.88888888888889</v>
       </c>
-      <c r="U10" s="67" t="n">
+      <c r="U10" s="68" t="n">
         <f aca="false">(O10+R10)*Assumptions!$B$38</f>
         <v>1.10065555555556</v>
       </c>
-      <c r="V10" s="67" t="n">
+      <c r="V10" s="68" t="n">
         <f aca="false">J10+O10+R10+T10+U10</f>
         <v>32.3261833333333</v>
       </c>
-      <c r="W10" s="67" t="n">
+      <c r="W10" s="68" t="n">
         <f aca="false">V10*Assumptions!$B$39</f>
         <v>2.58609466666667</v>
       </c>
-      <c r="X10" s="67" t="n">
+      <c r="X10" s="68" t="n">
         <f aca="false">(V10+W10)*Assumptions!$B$40</f>
         <v>3.4912278</v>
       </c>
-      <c r="Y10" s="72" t="n">
+      <c r="Y10" s="73" t="n">
         <f aca="false">V10+W10+X10</f>
         <v>38.4035058</v>
       </c>
-      <c r="Z10" s="72" t="n">
+      <c r="Z10" s="73" t="n">
         <f aca="false">Y10*E10</f>
         <v>76.8070116</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="73" t="n">
+      <c r="A11" s="74" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="74" t="s">
+      <c r="B11" s="75" t="s">
         <v>58</v>
       </c>
-      <c r="C11" s="75" t="s">
-        <v>276</v>
-      </c>
-      <c r="D11" s="75" t="s">
-        <v>277</v>
-      </c>
-      <c r="E11" s="73" t="n">
+      <c r="C11" s="76" t="s">
+        <v>323</v>
+      </c>
+      <c r="D11" s="76" t="s">
+        <v>324</v>
+      </c>
+      <c r="E11" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="65" t="n">
+      <c r="F11" s="66" t="n">
         <v>0.25</v>
       </c>
-      <c r="G11" s="66" t="n">
+      <c r="G11" s="67" t="n">
         <v>0.02</v>
       </c>
-      <c r="H11" s="76" t="n">
+      <c r="H11" s="77" t="n">
         <f aca="false">Assumptions!$B$13</f>
         <v>700</v>
       </c>
-      <c r="I11" s="76" t="n">
+      <c r="I11" s="77" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J11" s="76" t="n">
+      <c r="J11" s="77" t="n">
         <f aca="false">F11*(1+G11)*H11-F11*G11*I11</f>
         <v>178.3</v>
       </c>
-      <c r="K11" s="75" t="s">
-        <v>278</v>
-      </c>
-      <c r="L11" s="77" t="n">
+      <c r="K11" s="76" t="s">
+        <v>325</v>
+      </c>
+      <c r="L11" s="78" t="n">
         <f aca="false">Assumptions!$B$26</f>
         <v>650</v>
       </c>
-      <c r="M11" s="69" t="n">
+      <c r="M11" s="70" t="n">
         <v>90</v>
       </c>
-      <c r="N11" s="70" t="n">
+      <c r="N11" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="O11" s="76" t="n">
+      <c r="O11" s="77" t="n">
         <f aca="false">M11*L11/3600/N11</f>
         <v>16.25</v>
       </c>
-      <c r="P11" s="70" t="n">
+      <c r="P11" s="71" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q11" s="77" t="n">
+      <c r="Q11" s="78" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R11" s="76" t="n">
+      <c r="R11" s="77" t="n">
         <f aca="false">M11*P11*Q11/3600/N11</f>
         <v>2.375</v>
       </c>
-      <c r="S11" s="71" t="n">
+      <c r="S11" s="72" t="n">
         <v>3500000</v>
       </c>
-      <c r="T11" s="76" t="n">
+      <c r="T11" s="77" t="n">
         <f aca="false">S11/(Assumptions!$B$4*Assumptions!$B$5*E11)</f>
         <v>9.72222222222222</v>
       </c>
-      <c r="U11" s="76" t="n">
+      <c r="U11" s="77" t="n">
         <f aca="false">(O11+R11)*Assumptions!$B$38</f>
         <v>7.45</v>
       </c>
-      <c r="V11" s="76" t="n">
+      <c r="V11" s="77" t="n">
         <f aca="false">J11+O11+R11+T11+U11</f>
         <v>214.097222222222</v>
       </c>
-      <c r="W11" s="76" t="n">
+      <c r="W11" s="77" t="n">
         <f aca="false">V11*Assumptions!$B$39</f>
         <v>17.1277777777778</v>
       </c>
-      <c r="X11" s="76" t="n">
+      <c r="X11" s="77" t="n">
         <f aca="false">(V11+W11)*Assumptions!$B$40</f>
         <v>23.1225</v>
       </c>
-      <c r="Y11" s="78" t="n">
+      <c r="Y11" s="79" t="n">
         <f aca="false">V11+W11+X11</f>
         <v>254.3475</v>
       </c>
-      <c r="Z11" s="78" t="n">
+      <c r="Z11" s="79" t="n">
         <f aca="false">Y11*E11</f>
         <v>254.3475</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="62" t="n">
+      <c r="A12" s="63" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="63" t="s">
-        <v>279</v>
-      </c>
-      <c r="C12" s="64" t="s">
-        <v>280</v>
-      </c>
-      <c r="D12" s="64" t="s">
-        <v>281</v>
-      </c>
-      <c r="E12" s="62" t="n">
+      <c r="B12" s="64" t="s">
+        <v>326</v>
+      </c>
+      <c r="C12" s="65" t="s">
+        <v>327</v>
+      </c>
+      <c r="D12" s="65" t="s">
+        <v>328</v>
+      </c>
+      <c r="E12" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="65" t="n">
+      <c r="F12" s="66" t="n">
         <v>4.2</v>
       </c>
-      <c r="G12" s="66" t="n">
+      <c r="G12" s="67" t="n">
         <v>0.08</v>
       </c>
-      <c r="H12" s="67" t="n">
+      <c r="H12" s="68" t="n">
         <f aca="false">Assumptions!$B$15</f>
         <v>68</v>
       </c>
-      <c r="I12" s="67" t="n">
+      <c r="I12" s="68" t="n">
         <f aca="false">Assumptions!$B$16</f>
         <v>32</v>
       </c>
-      <c r="J12" s="67" t="n">
+      <c r="J12" s="68" t="n">
         <f aca="false">F12*(1+G12)*H12-F12*G12*I12</f>
         <v>297.696</v>
       </c>
-      <c r="K12" s="64" t="s">
-        <v>282</v>
-      </c>
-      <c r="L12" s="68" t="n">
+      <c r="K12" s="65" t="s">
+        <v>329</v>
+      </c>
+      <c r="L12" s="69" t="n">
         <f aca="false">Assumptions!$B$28</f>
         <v>1600</v>
       </c>
-      <c r="M12" s="69" t="n">
+      <c r="M12" s="70" t="n">
         <v>45</v>
       </c>
-      <c r="N12" s="70" t="n">
+      <c r="N12" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="O12" s="67" t="n">
+      <c r="O12" s="68" t="n">
         <f aca="false">M12*L12/3600/N12</f>
         <v>20</v>
       </c>
-      <c r="P12" s="70" t="n">
+      <c r="P12" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="Q12" s="68" t="n">
+      <c r="Q12" s="69" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R12" s="67" t="n">
+      <c r="R12" s="68" t="n">
         <f aca="false">M12*P12*Q12/3600/N12</f>
         <v>2.375</v>
       </c>
-      <c r="S12" s="71" t="n">
+      <c r="S12" s="72" t="n">
         <v>5000000</v>
       </c>
-      <c r="T12" s="67" t="n">
+      <c r="T12" s="68" t="n">
         <f aca="false">S12/(Assumptions!$B$4*Assumptions!$B$5*E12)</f>
         <v>13.8888888888889</v>
       </c>
-      <c r="U12" s="67" t="n">
+      <c r="U12" s="68" t="n">
         <f aca="false">(O12+R12)*Assumptions!$B$38</f>
         <v>8.95</v>
       </c>
-      <c r="V12" s="67" t="n">
+      <c r="V12" s="68" t="n">
         <f aca="false">J12+O12+R12+T12+U12</f>
         <v>342.909888888889</v>
       </c>
-      <c r="W12" s="67" t="n">
+      <c r="W12" s="68" t="n">
         <f aca="false">V12*Assumptions!$B$39</f>
         <v>27.4327911111111</v>
       </c>
-      <c r="X12" s="67" t="n">
+      <c r="X12" s="68" t="n">
         <f aca="false">(V12+W12)*Assumptions!$B$40</f>
         <v>37.034268</v>
       </c>
-      <c r="Y12" s="72" t="n">
+      <c r="Y12" s="73" t="n">
         <f aca="false">V12+W12+X12</f>
         <v>407.376948</v>
       </c>
-      <c r="Z12" s="72" t="n">
+      <c r="Z12" s="73" t="n">
         <f aca="false">Y12*E12</f>
         <v>407.376948</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="73" t="n">
+      <c r="A13" s="74" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="74" t="s">
-        <v>283</v>
-      </c>
-      <c r="C13" s="75" t="s">
-        <v>284</v>
-      </c>
-      <c r="D13" s="75" t="s">
-        <v>285</v>
-      </c>
-      <c r="E13" s="73" t="n">
+      <c r="B13" s="75" t="s">
+        <v>330</v>
+      </c>
+      <c r="C13" s="76" t="s">
+        <v>331</v>
+      </c>
+      <c r="D13" s="76" t="s">
+        <v>332</v>
+      </c>
+      <c r="E13" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="73"/>
-      <c r="G13" s="73"/>
-      <c r="H13" s="73"/>
-      <c r="I13" s="73"/>
-      <c r="J13" s="76" t="n">
+      <c r="F13" s="74"/>
+      <c r="G13" s="74"/>
+      <c r="H13" s="74"/>
+      <c r="I13" s="74"/>
+      <c r="J13" s="77" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="75" t="s">
-        <v>286</v>
-      </c>
-      <c r="L13" s="77" t="n">
+      <c r="K13" s="76" t="s">
+        <v>333</v>
+      </c>
+      <c r="L13" s="78" t="n">
         <f aca="false">Assumptions!$B$29</f>
         <v>800</v>
       </c>
-      <c r="M13" s="69" t="n">
+      <c r="M13" s="70" t="n">
         <v>60</v>
       </c>
-      <c r="N13" s="70" t="n">
+      <c r="N13" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="O13" s="76" t="n">
+      <c r="O13" s="77" t="n">
         <f aca="false">M13*L13/3600/N13</f>
         <v>13.3333333333333</v>
       </c>
-      <c r="P13" s="70" t="n">
+      <c r="P13" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="Q13" s="77" t="n">
+      <c r="Q13" s="78" t="n">
         <f aca="false">Assumptions!$B$34</f>
         <v>260</v>
       </c>
-      <c r="R13" s="76" t="n">
+      <c r="R13" s="77" t="n">
         <f aca="false">M13*P13*Q13/3600/N13</f>
         <v>4.33333333333333</v>
       </c>
-      <c r="S13" s="71" t="n">
+      <c r="S13" s="72" t="n">
         <v>1500000</v>
       </c>
-      <c r="T13" s="76" t="n">
+      <c r="T13" s="77" t="n">
         <f aca="false">S13/(Assumptions!$B$4*Assumptions!$B$5*E13)</f>
         <v>4.16666666666667</v>
       </c>
-      <c r="U13" s="76" t="n">
+      <c r="U13" s="77" t="n">
         <f aca="false">(O13+R13)*Assumptions!$B$38</f>
         <v>7.06666666666667</v>
       </c>
-      <c r="V13" s="76" t="n">
+      <c r="V13" s="77" t="n">
         <f aca="false">J13+O13+R13+T13+U13</f>
         <v>28.9</v>
       </c>
-      <c r="W13" s="76" t="n">
+      <c r="W13" s="77" t="n">
         <f aca="false">V13*Assumptions!$B$39</f>
         <v>2.312</v>
       </c>
-      <c r="X13" s="76" t="n">
+      <c r="X13" s="77" t="n">
         <f aca="false">(V13+W13)*Assumptions!$B$40</f>
         <v>3.1212</v>
       </c>
-      <c r="Y13" s="78" t="n">
+      <c r="Y13" s="79" t="n">
         <f aca="false">V13+W13+X13</f>
         <v>34.3332</v>
       </c>
-      <c r="Z13" s="78" t="n">
+      <c r="Z13" s="79" t="n">
         <f aca="false">Y13*E13</f>
         <v>34.3332</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="62" t="n">
+      <c r="A14" s="63" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="63" t="s">
-        <v>287</v>
-      </c>
-      <c r="C14" s="64" t="s">
-        <v>288</v>
-      </c>
-      <c r="D14" s="64" t="s">
-        <v>281</v>
-      </c>
-      <c r="E14" s="62" t="n">
+      <c r="B14" s="64" t="s">
+        <v>334</v>
+      </c>
+      <c r="C14" s="65" t="s">
+        <v>335</v>
+      </c>
+      <c r="D14" s="65" t="s">
+        <v>328</v>
+      </c>
+      <c r="E14" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="65" t="n">
+      <c r="F14" s="66" t="n">
         <v>0.35</v>
       </c>
-      <c r="G14" s="66" t="n">
+      <c r="G14" s="67" t="n">
         <v>0.12</v>
       </c>
-      <c r="H14" s="67" t="n">
+      <c r="H14" s="68" t="n">
         <f aca="false">Assumptions!$B$15</f>
         <v>68</v>
       </c>
-      <c r="I14" s="67" t="n">
+      <c r="I14" s="68" t="n">
         <f aca="false">Assumptions!$B$16</f>
         <v>32</v>
       </c>
-      <c r="J14" s="67" t="n">
+      <c r="J14" s="68" t="n">
         <f aca="false">F14*(1+G14)*H14-F14*G14*I14</f>
         <v>25.312</v>
       </c>
-      <c r="K14" s="64" t="s">
-        <v>289</v>
-      </c>
-      <c r="L14" s="68" t="n">
+      <c r="K14" s="65" t="s">
+        <v>336</v>
+      </c>
+      <c r="L14" s="69" t="n">
         <f aca="false">Assumptions!$B$27</f>
         <v>900</v>
       </c>
-      <c r="M14" s="69" t="n">
+      <c r="M14" s="70" t="n">
         <v>12</v>
       </c>
-      <c r="N14" s="70" t="n">
+      <c r="N14" s="71" t="n">
         <v>2</v>
       </c>
-      <c r="O14" s="67" t="n">
+      <c r="O14" s="68" t="n">
         <f aca="false">M14*L14/3600/N14</f>
         <v>1.5</v>
       </c>
-      <c r="P14" s="70" t="n">
+      <c r="P14" s="71" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q14" s="68" t="n">
+      <c r="Q14" s="69" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R14" s="67" t="n">
+      <c r="R14" s="68" t="n">
         <f aca="false">M14*P14*Q14/3600/N14</f>
         <v>0.158333333333333</v>
       </c>
-      <c r="S14" s="71" t="n">
+      <c r="S14" s="72" t="n">
         <v>2500000</v>
       </c>
-      <c r="T14" s="67" t="n">
+      <c r="T14" s="68" t="n">
         <f aca="false">S14/(Assumptions!$B$4*Assumptions!$B$5*E14)</f>
         <v>3.47222222222222</v>
       </c>
-      <c r="U14" s="67" t="n">
+      <c r="U14" s="68" t="n">
         <f aca="false">(O14+R14)*Assumptions!$B$38</f>
         <v>0.663333333333333</v>
       </c>
-      <c r="V14" s="67" t="n">
+      <c r="V14" s="68" t="n">
         <f aca="false">J14+O14+R14+T14+U14</f>
         <v>31.1058888888889</v>
       </c>
-      <c r="W14" s="67" t="n">
+      <c r="W14" s="68" t="n">
         <f aca="false">V14*Assumptions!$B$39</f>
         <v>2.48847111111111</v>
       </c>
-      <c r="X14" s="67" t="n">
+      <c r="X14" s="68" t="n">
         <f aca="false">(V14+W14)*Assumptions!$B$40</f>
         <v>3.359436</v>
       </c>
-      <c r="Y14" s="72" t="n">
+      <c r="Y14" s="73" t="n">
         <f aca="false">V14+W14+X14</f>
         <v>36.953796</v>
       </c>
-      <c r="Z14" s="72" t="n">
+      <c r="Z14" s="73" t="n">
         <f aca="false">Y14*E14</f>
         <v>73.907592</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="73" t="n">
+      <c r="A15" s="74" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="74" t="s">
-        <v>290</v>
-      </c>
-      <c r="C15" s="75" t="s">
-        <v>258</v>
-      </c>
-      <c r="D15" s="75" t="s">
-        <v>270</v>
-      </c>
-      <c r="E15" s="73" t="n">
+      <c r="B15" s="75" t="s">
+        <v>337</v>
+      </c>
+      <c r="C15" s="76" t="s">
+        <v>305</v>
+      </c>
+      <c r="D15" s="76" t="s">
+        <v>317</v>
+      </c>
+      <c r="E15" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="65" t="n">
+      <c r="F15" s="66" t="n">
         <v>0.05</v>
       </c>
-      <c r="G15" s="66" t="n">
+      <c r="G15" s="67" t="n">
         <v>0.04</v>
       </c>
-      <c r="H15" s="76" t="n">
+      <c r="H15" s="77" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>112</v>
       </c>
-      <c r="I15" s="76" t="n">
+      <c r="I15" s="77" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J15" s="76" t="n">
+      <c r="J15" s="77" t="n">
         <f aca="false">F15*(1+G15)*H15-F15*G15*I15</f>
         <v>5.744</v>
       </c>
-      <c r="K15" s="75" t="s">
-        <v>271</v>
-      </c>
-      <c r="L15" s="77" t="n">
+      <c r="K15" s="76" t="s">
+        <v>318</v>
+      </c>
+      <c r="L15" s="78" t="n">
         <f aca="false">Assumptions!$B$25</f>
         <v>400</v>
       </c>
-      <c r="M15" s="69" t="n">
+      <c r="M15" s="70" t="n">
         <v>22</v>
       </c>
-      <c r="N15" s="70" t="n">
+      <c r="N15" s="71" t="n">
         <v>2</v>
       </c>
-      <c r="O15" s="76" t="n">
+      <c r="O15" s="77" t="n">
         <f aca="false">M15*L15/3600/N15</f>
         <v>1.22222222222222</v>
       </c>
-      <c r="P15" s="70" t="n">
+      <c r="P15" s="71" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q15" s="77" t="n">
+      <c r="Q15" s="78" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R15" s="76" t="n">
+      <c r="R15" s="77" t="n">
         <f aca="false">M15*P15*Q15/3600/N15</f>
         <v>0.145138888888889</v>
       </c>
-      <c r="S15" s="71" t="n">
+      <c r="S15" s="72" t="n">
         <v>900000</v>
       </c>
-      <c r="T15" s="76" t="n">
+      <c r="T15" s="77" t="n">
         <f aca="false">S15/(Assumptions!$B$4*Assumptions!$B$5*E15)</f>
         <v>2.5</v>
       </c>
-      <c r="U15" s="76" t="n">
+      <c r="U15" s="77" t="n">
         <f aca="false">(O15+R15)*Assumptions!$B$38</f>
         <v>0.546944444444445</v>
       </c>
-      <c r="V15" s="76" t="n">
+      <c r="V15" s="77" t="n">
         <f aca="false">J15+O15+R15+T15+U15</f>
         <v>10.1583055555556</v>
       </c>
-      <c r="W15" s="76" t="n">
+      <c r="W15" s="77" t="n">
         <f aca="false">V15*Assumptions!$B$39</f>
         <v>0.812664444444445</v>
       </c>
-      <c r="X15" s="76" t="n">
+      <c r="X15" s="77" t="n">
         <f aca="false">(V15+W15)*Assumptions!$B$40</f>
         <v>1.097097</v>
       </c>
-      <c r="Y15" s="78" t="n">
+      <c r="Y15" s="79" t="n">
         <f aca="false">V15+W15+X15</f>
         <v>12.068067</v>
       </c>
-      <c r="Z15" s="78" t="n">
+      <c r="Z15" s="79" t="n">
         <f aca="false">Y15*E15</f>
         <v>12.068067</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="62" t="n">
+      <c r="A16" s="63" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="63" t="s">
-        <v>291</v>
-      </c>
-      <c r="C16" s="64" t="s">
-        <v>258</v>
-      </c>
-      <c r="D16" s="64" t="s">
-        <v>270</v>
-      </c>
-      <c r="E16" s="79" t="n">
+      <c r="B16" s="64" t="s">
+        <v>338</v>
+      </c>
+      <c r="C16" s="65" t="s">
+        <v>305</v>
+      </c>
+      <c r="D16" s="65" t="s">
+        <v>317</v>
+      </c>
+      <c r="E16" s="80" t="n">
         <f aca="false">Assumptions!$B$44</f>
         <v>4</v>
       </c>
-      <c r="F16" s="65" t="n">
+      <c r="F16" s="66" t="n">
         <v>0.02</v>
       </c>
-      <c r="G16" s="66" t="n">
+      <c r="G16" s="67" t="n">
         <v>0.04</v>
       </c>
-      <c r="H16" s="67" t="n">
+      <c r="H16" s="68" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>112</v>
       </c>
-      <c r="I16" s="67" t="n">
+      <c r="I16" s="68" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J16" s="67" t="n">
+      <c r="J16" s="68" t="n">
         <f aca="false">F16*(1+G16)*H16-F16*G16*I16</f>
         <v>2.2976</v>
       </c>
-      <c r="K16" s="64" t="s">
-        <v>271</v>
-      </c>
-      <c r="L16" s="68" t="n">
+      <c r="K16" s="65" t="s">
+        <v>318</v>
+      </c>
+      <c r="L16" s="69" t="n">
         <f aca="false">Assumptions!$B$25</f>
         <v>400</v>
       </c>
-      <c r="M16" s="69" t="n">
+      <c r="M16" s="70" t="n">
         <v>20</v>
       </c>
-      <c r="N16" s="70" t="n">
+      <c r="N16" s="71" t="n">
         <v>4</v>
       </c>
-      <c r="O16" s="67" t="n">
+      <c r="O16" s="68" t="n">
         <f aca="false">M16*L16/3600/N16</f>
         <v>0.555555555555556</v>
       </c>
-      <c r="P16" s="70" t="n">
+      <c r="P16" s="71" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q16" s="68" t="n">
+      <c r="Q16" s="69" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R16" s="67" t="n">
+      <c r="R16" s="68" t="n">
         <f aca="false">M16*P16*Q16/3600/N16</f>
         <v>0.0659722222222222</v>
       </c>
-      <c r="S16" s="71" t="n">
+      <c r="S16" s="72" t="n">
         <v>1400000</v>
       </c>
-      <c r="T16" s="67" t="n">
+      <c r="T16" s="68" t="n">
         <f aca="false">S16/(Assumptions!$B$4*Assumptions!$B$5*E16)</f>
         <v>0.972222222222222</v>
       </c>
-      <c r="U16" s="67" t="n">
+      <c r="U16" s="68" t="n">
         <f aca="false">(O16+R16)*Assumptions!$B$38</f>
         <v>0.248611111111111</v>
       </c>
-      <c r="V16" s="67" t="n">
+      <c r="V16" s="68" t="n">
         <f aca="false">J16+O16+R16+T16+U16</f>
         <v>4.13996111111111</v>
       </c>
-      <c r="W16" s="67" t="n">
+      <c r="W16" s="68" t="n">
         <f aca="false">V16*Assumptions!$B$39</f>
         <v>0.331196888888889</v>
       </c>
-      <c r="X16" s="67" t="n">
+      <c r="X16" s="68" t="n">
         <f aca="false">(V16+W16)*Assumptions!$B$40</f>
         <v>0.4471158</v>
       </c>
-      <c r="Y16" s="72" t="n">
+      <c r="Y16" s="73" t="n">
         <f aca="false">V16+W16+X16</f>
         <v>4.9182738</v>
       </c>
-      <c r="Z16" s="72" t="n">
+      <c r="Z16" s="73" t="n">
         <f aca="false">Y16*E16</f>
         <v>19.6730952</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="73" t="n">
+      <c r="A17" s="74" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="74" t="s">
-        <v>292</v>
-      </c>
-      <c r="C17" s="75" t="s">
-        <v>258</v>
-      </c>
-      <c r="D17" s="75" t="s">
-        <v>270</v>
-      </c>
-      <c r="E17" s="73" t="n">
+      <c r="B17" s="75" t="s">
+        <v>339</v>
+      </c>
+      <c r="C17" s="76" t="s">
+        <v>305</v>
+      </c>
+      <c r="D17" s="76" t="s">
+        <v>317</v>
+      </c>
+      <c r="E17" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="65" t="n">
+      <c r="F17" s="66" t="n">
         <v>0.08</v>
       </c>
-      <c r="G17" s="66" t="n">
+      <c r="G17" s="67" t="n">
         <v>0.04</v>
       </c>
-      <c r="H17" s="76" t="n">
+      <c r="H17" s="77" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>112</v>
       </c>
-      <c r="I17" s="76" t="n">
+      <c r="I17" s="77" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J17" s="76" t="n">
+      <c r="J17" s="77" t="n">
         <f aca="false">F17*(1+G17)*H17-F17*G17*I17</f>
         <v>9.1904</v>
       </c>
-      <c r="K17" s="75" t="s">
-        <v>271</v>
-      </c>
-      <c r="L17" s="77" t="n">
+      <c r="K17" s="76" t="s">
+        <v>318</v>
+      </c>
+      <c r="L17" s="78" t="n">
         <f aca="false">Assumptions!$B$25</f>
         <v>400</v>
       </c>
-      <c r="M17" s="69" t="n">
+      <c r="M17" s="70" t="n">
         <v>25</v>
       </c>
-      <c r="N17" s="70" t="n">
+      <c r="N17" s="71" t="n">
         <v>2</v>
       </c>
-      <c r="O17" s="76" t="n">
+      <c r="O17" s="77" t="n">
         <f aca="false">M17*L17/3600/N17</f>
         <v>1.38888888888889</v>
       </c>
-      <c r="P17" s="70" t="n">
+      <c r="P17" s="71" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q17" s="77" t="n">
+      <c r="Q17" s="78" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R17" s="76" t="n">
+      <c r="R17" s="77" t="n">
         <f aca="false">M17*P17*Q17/3600/N17</f>
         <v>0.164930555555556</v>
       </c>
-      <c r="S17" s="71" t="n">
+      <c r="S17" s="72" t="n">
         <v>1100000</v>
       </c>
-      <c r="T17" s="76" t="n">
+      <c r="T17" s="77" t="n">
         <f aca="false">S17/(Assumptions!$B$4*Assumptions!$B$5*E17)</f>
         <v>3.05555555555556</v>
       </c>
-      <c r="U17" s="76" t="n">
+      <c r="U17" s="77" t="n">
         <f aca="false">(O17+R17)*Assumptions!$B$38</f>
         <v>0.621527777777778</v>
       </c>
-      <c r="V17" s="76" t="n">
+      <c r="V17" s="77" t="n">
         <f aca="false">J17+O17+R17+T17+U17</f>
         <v>14.4213027777778</v>
       </c>
-      <c r="W17" s="76" t="n">
+      <c r="W17" s="77" t="n">
         <f aca="false">V17*Assumptions!$B$39</f>
         <v>1.15370422222222</v>
       </c>
-      <c r="X17" s="76" t="n">
+      <c r="X17" s="77" t="n">
         <f aca="false">(V17+W17)*Assumptions!$B$40</f>
         <v>1.5575007</v>
       </c>
-      <c r="Y17" s="78" t="n">
+      <c r="Y17" s="79" t="n">
         <f aca="false">V17+W17+X17</f>
         <v>17.1325077</v>
       </c>
-      <c r="Z17" s="78" t="n">
+      <c r="Z17" s="79" t="n">
         <f aca="false">Y17*E17</f>
         <v>17.1325077</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="62" t="n">
+      <c r="A18" s="63" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="63" t="s">
-        <v>293</v>
-      </c>
-      <c r="C18" s="64" t="s">
-        <v>258</v>
-      </c>
-      <c r="D18" s="64" t="s">
-        <v>270</v>
-      </c>
-      <c r="E18" s="62" t="n">
+      <c r="B18" s="64" t="s">
+        <v>340</v>
+      </c>
+      <c r="C18" s="65" t="s">
+        <v>305</v>
+      </c>
+      <c r="D18" s="65" t="s">
+        <v>317</v>
+      </c>
+      <c r="E18" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="F18" s="65" t="n">
+      <c r="F18" s="66" t="n">
         <v>0.05</v>
       </c>
-      <c r="G18" s="66" t="n">
+      <c r="G18" s="67" t="n">
         <v>0.04</v>
       </c>
-      <c r="H18" s="67" t="n">
+      <c r="H18" s="68" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>112</v>
       </c>
-      <c r="I18" s="67" t="n">
+      <c r="I18" s="68" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J18" s="67" t="n">
+      <c r="J18" s="68" t="n">
         <f aca="false">F18*(1+G18)*H18-F18*G18*I18</f>
         <v>5.744</v>
       </c>
-      <c r="K18" s="64" t="s">
-        <v>271</v>
-      </c>
-      <c r="L18" s="68" t="n">
+      <c r="K18" s="65" t="s">
+        <v>318</v>
+      </c>
+      <c r="L18" s="69" t="n">
         <f aca="false">Assumptions!$B$25</f>
         <v>400</v>
       </c>
-      <c r="M18" s="69" t="n">
+      <c r="M18" s="70" t="n">
         <v>22</v>
       </c>
-      <c r="N18" s="70" t="n">
+      <c r="N18" s="71" t="n">
         <v>2</v>
       </c>
-      <c r="O18" s="67" t="n">
+      <c r="O18" s="68" t="n">
         <f aca="false">M18*L18/3600/N18</f>
         <v>1.22222222222222</v>
       </c>
-      <c r="P18" s="70" t="n">
+      <c r="P18" s="71" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q18" s="68" t="n">
+      <c r="Q18" s="69" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R18" s="67" t="n">
+      <c r="R18" s="68" t="n">
         <f aca="false">M18*P18*Q18/3600/N18</f>
         <v>0.145138888888889</v>
       </c>
-      <c r="S18" s="71" t="n">
+      <c r="S18" s="72" t="n">
         <v>900000</v>
       </c>
-      <c r="T18" s="67" t="n">
+      <c r="T18" s="68" t="n">
         <f aca="false">S18/(Assumptions!$B$4*Assumptions!$B$5*E18)</f>
         <v>2.5</v>
       </c>
-      <c r="U18" s="67" t="n">
+      <c r="U18" s="68" t="n">
         <f aca="false">(O18+R18)*Assumptions!$B$38</f>
         <v>0.546944444444445</v>
       </c>
-      <c r="V18" s="67" t="n">
+      <c r="V18" s="68" t="n">
         <f aca="false">J18+O18+R18+T18+U18</f>
         <v>10.1583055555556</v>
       </c>
-      <c r="W18" s="67" t="n">
+      <c r="W18" s="68" t="n">
         <f aca="false">V18*Assumptions!$B$39</f>
         <v>0.812664444444445</v>
       </c>
-      <c r="X18" s="67" t="n">
+      <c r="X18" s="68" t="n">
         <f aca="false">(V18+W18)*Assumptions!$B$40</f>
         <v>1.097097</v>
       </c>
-      <c r="Y18" s="72" t="n">
+      <c r="Y18" s="73" t="n">
         <f aca="false">V18+W18+X18</f>
         <v>12.068067</v>
       </c>
-      <c r="Z18" s="72" t="n">
+      <c r="Z18" s="73" t="n">
         <f aca="false">Y18*E18</f>
         <v>12.068067</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="73" t="n">
+      <c r="A19" s="74" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="74" t="s">
-        <v>294</v>
-      </c>
-      <c r="C19" s="75" t="s">
-        <v>258</v>
-      </c>
-      <c r="D19" s="75" t="s">
-        <v>270</v>
-      </c>
-      <c r="E19" s="73" t="n">
+      <c r="B19" s="75" t="s">
+        <v>341</v>
+      </c>
+      <c r="C19" s="76" t="s">
+        <v>305</v>
+      </c>
+      <c r="D19" s="76" t="s">
+        <v>317</v>
+      </c>
+      <c r="E19" s="74" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="65" t="n">
+      <c r="F19" s="66" t="n">
         <v>0.35</v>
       </c>
-      <c r="G19" s="66" t="n">
+      <c r="G19" s="67" t="n">
         <v>0.05</v>
       </c>
-      <c r="H19" s="76" t="n">
+      <c r="H19" s="77" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>112</v>
       </c>
-      <c r="I19" s="76" t="n">
+      <c r="I19" s="77" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J19" s="76" t="n">
+      <c r="J19" s="77" t="n">
         <f aca="false">F19*(1+G19)*H19-F19*G19*I19</f>
         <v>40.46</v>
       </c>
-      <c r="K19" s="75" t="s">
-        <v>267</v>
-      </c>
-      <c r="L19" s="77" t="n">
+      <c r="K19" s="76" t="s">
+        <v>314</v>
+      </c>
+      <c r="L19" s="78" t="n">
         <f aca="false">Assumptions!$B$23</f>
         <v>700</v>
       </c>
-      <c r="M19" s="69" t="n">
+      <c r="M19" s="70" t="n">
         <v>33</v>
       </c>
-      <c r="N19" s="70" t="n">
+      <c r="N19" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="O19" s="76" t="n">
+      <c r="O19" s="77" t="n">
         <f aca="false">M19*L19/3600/N19</f>
         <v>6.41666666666667</v>
       </c>
-      <c r="P19" s="70" t="n">
+      <c r="P19" s="71" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q19" s="77" t="n">
+      <c r="Q19" s="78" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R19" s="76" t="n">
+      <c r="R19" s="77" t="n">
         <f aca="false">M19*P19*Q19/3600/N19</f>
         <v>0.57475</v>
       </c>
-      <c r="S19" s="71" t="n">
+      <c r="S19" s="72" t="n">
         <v>3000000</v>
       </c>
-      <c r="T19" s="76" t="n">
+      <c r="T19" s="77" t="n">
         <f aca="false">S19/(Assumptions!$B$4*Assumptions!$B$5*E19)</f>
         <v>8.33333333333333</v>
       </c>
-      <c r="U19" s="76" t="n">
+      <c r="U19" s="77" t="n">
         <f aca="false">(O19+R19)*Assumptions!$B$38</f>
         <v>2.79656666666667</v>
       </c>
-      <c r="V19" s="76" t="n">
+      <c r="V19" s="77" t="n">
         <f aca="false">J19+O19+R19+T19+U19</f>
         <v>58.5813166666667</v>
       </c>
-      <c r="W19" s="76" t="n">
+      <c r="W19" s="77" t="n">
         <f aca="false">V19*Assumptions!$B$39</f>
         <v>4.68650533333333</v>
       </c>
-      <c r="X19" s="76" t="n">
+      <c r="X19" s="77" t="n">
         <f aca="false">(V19+W19)*Assumptions!$B$40</f>
         <v>6.3267822</v>
       </c>
-      <c r="Y19" s="78" t="n">
+      <c r="Y19" s="79" t="n">
         <f aca="false">V19+W19+X19</f>
         <v>69.5946042</v>
       </c>
-      <c r="Z19" s="78" t="n">
+      <c r="Z19" s="79" t="n">
         <f aca="false">Y19*E19</f>
         <v>69.5946042</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="62" t="n">
+      <c r="A20" s="63" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="63" t="s">
-        <v>295</v>
-      </c>
-      <c r="C20" s="64" t="s">
-        <v>258</v>
-      </c>
-      <c r="D20" s="64" t="s">
-        <v>270</v>
-      </c>
-      <c r="E20" s="62" t="n">
+      <c r="B20" s="64" t="s">
+        <v>342</v>
+      </c>
+      <c r="C20" s="65" t="s">
+        <v>305</v>
+      </c>
+      <c r="D20" s="65" t="s">
+        <v>317</v>
+      </c>
+      <c r="E20" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="F20" s="65" t="n">
+      <c r="F20" s="66" t="n">
         <v>0.15</v>
       </c>
-      <c r="G20" s="66" t="n">
+      <c r="G20" s="67" t="n">
         <v>0.04</v>
       </c>
-      <c r="H20" s="67" t="n">
+      <c r="H20" s="68" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>112</v>
       </c>
-      <c r="I20" s="67" t="n">
+      <c r="I20" s="68" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J20" s="67" t="n">
+      <c r="J20" s="68" t="n">
         <f aca="false">F20*(1+G20)*H20-F20*G20*I20</f>
         <v>17.232</v>
       </c>
-      <c r="K20" s="64" t="s">
-        <v>275</v>
-      </c>
-      <c r="L20" s="68" t="n">
+      <c r="K20" s="65" t="s">
+        <v>322</v>
+      </c>
+      <c r="L20" s="69" t="n">
         <f aca="false">Assumptions!$B$24</f>
         <v>520</v>
       </c>
-      <c r="M20" s="69" t="n">
+      <c r="M20" s="70" t="n">
         <v>30</v>
       </c>
-      <c r="N20" s="70" t="n">
+      <c r="N20" s="71" t="n">
         <v>2</v>
       </c>
-      <c r="O20" s="67" t="n">
+      <c r="O20" s="68" t="n">
         <f aca="false">M20*L20/3600/N20</f>
         <v>2.16666666666667</v>
       </c>
-      <c r="P20" s="70" t="n">
+      <c r="P20" s="71" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q20" s="68" t="n">
+      <c r="Q20" s="69" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R20" s="67" t="n">
+      <c r="R20" s="68" t="n">
         <f aca="false">M20*P20*Q20/3600/N20</f>
         <v>0.26125</v>
       </c>
-      <c r="S20" s="71" t="n">
+      <c r="S20" s="72" t="n">
         <v>1600000</v>
       </c>
-      <c r="T20" s="67" t="n">
+      <c r="T20" s="68" t="n">
         <f aca="false">S20/(Assumptions!$B$4*Assumptions!$B$5*E20)</f>
         <v>2.22222222222222</v>
       </c>
-      <c r="U20" s="67" t="n">
+      <c r="U20" s="68" t="n">
         <f aca="false">(O20+R20)*Assumptions!$B$38</f>
         <v>0.971166666666667</v>
       </c>
-      <c r="V20" s="67" t="n">
+      <c r="V20" s="68" t="n">
         <f aca="false">J20+O20+R20+T20+U20</f>
         <v>22.8533055555556</v>
       </c>
-      <c r="W20" s="67" t="n">
+      <c r="W20" s="68" t="n">
         <f aca="false">V20*Assumptions!$B$39</f>
         <v>1.82826444444444</v>
       </c>
-      <c r="X20" s="67" t="n">
+      <c r="X20" s="68" t="n">
         <f aca="false">(V20+W20)*Assumptions!$B$40</f>
         <v>2.468157</v>
       </c>
-      <c r="Y20" s="72" t="n">
+      <c r="Y20" s="73" t="n">
         <f aca="false">V20+W20+X20</f>
         <v>27.149727</v>
       </c>
-      <c r="Z20" s="72" t="n">
+      <c r="Z20" s="73" t="n">
         <f aca="false">Y20*E20</f>
         <v>54.299454</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="73" t="n">
+      <c r="A21" s="74" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="74" t="s">
-        <v>296</v>
-      </c>
-      <c r="C21" s="75" t="s">
-        <v>258</v>
-      </c>
-      <c r="D21" s="75" t="s">
-        <v>270</v>
-      </c>
-      <c r="E21" s="73" t="n">
+      <c r="B21" s="75" t="s">
+        <v>343</v>
+      </c>
+      <c r="C21" s="76" t="s">
+        <v>305</v>
+      </c>
+      <c r="D21" s="76" t="s">
+        <v>317</v>
+      </c>
+      <c r="E21" s="74" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="65" t="n">
+      <c r="F21" s="66" t="n">
         <v>0.15</v>
       </c>
-      <c r="G21" s="66" t="n">
+      <c r="G21" s="67" t="n">
         <v>0.04</v>
       </c>
-      <c r="H21" s="76" t="n">
+      <c r="H21" s="77" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>112</v>
       </c>
-      <c r="I21" s="76" t="n">
+      <c r="I21" s="77" t="n">
         <f aca="false">Assumptions!$B$17</f>
         <v>40</v>
       </c>
-      <c r="J21" s="76" t="n">
+      <c r="J21" s="77" t="n">
         <f aca="false">F21*(1+G21)*H21-F21*G21*I21</f>
         <v>17.232</v>
       </c>
-      <c r="K21" s="75" t="s">
-        <v>275</v>
-      </c>
-      <c r="L21" s="77" t="n">
+      <c r="K21" s="76" t="s">
+        <v>322</v>
+      </c>
+      <c r="L21" s="78" t="n">
         <f aca="false">Assumptions!$B$24</f>
         <v>520</v>
       </c>
-      <c r="M21" s="69" t="n">
+      <c r="M21" s="70" t="n">
         <v>30</v>
       </c>
-      <c r="N21" s="70" t="n">
+      <c r="N21" s="71" t="n">
         <v>2</v>
       </c>
-      <c r="O21" s="76" t="n">
+      <c r="O21" s="77" t="n">
         <f aca="false">M21*L21/3600/N21</f>
         <v>2.16666666666667</v>
       </c>
-      <c r="P21" s="70" t="n">
+      <c r="P21" s="71" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q21" s="77" t="n">
+      <c r="Q21" s="78" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="R21" s="76" t="n">
+      <c r="R21" s="77" t="n">
         <f aca="false">M21*P21*Q21/3600/N21</f>
         <v>0.26125</v>
       </c>
-      <c r="S21" s="71" t="n">
+      <c r="S21" s="72" t="n">
         <v>1600000</v>
       </c>
-      <c r="T21" s="76" t="n">
+      <c r="T21" s="77" t="n">
         <f aca="false">S21/(Assumptions!$B$4*Assumptions!$B$5*E21)</f>
         <v>2.22222222222222</v>
       </c>
-      <c r="U21" s="76" t="n">
+      <c r="U21" s="77" t="n">
         <f aca="false">(O21+R21)*Assumptions!$B$38</f>
         <v>0.971166666666667</v>
       </c>
-      <c r="V21" s="76" t="n">
+      <c r="V21" s="77" t="n">
         <f aca="false">J21+O21+R21+T21+U21</f>
         <v>22.8533055555556</v>
       </c>
-      <c r="W21" s="76" t="n">
+      <c r="W21" s="77" t="n">
         <f aca="false">V21*Assumptions!$B$39</f>
         <v>1.82826444444444</v>
       </c>
-      <c r="X21" s="76" t="n">
+      <c r="X21" s="77" t="n">
         <f aca="false">(V21+W21)*Assumptions!$B$40</f>
         <v>2.468157</v>
       </c>
-      <c r="Y21" s="78" t="n">
+      <c r="Y21" s="79" t="n">
         <f aca="false">V21+W21+X21</f>
         <v>27.149727</v>
       </c>
-      <c r="Z21" s="78" t="n">
+      <c r="Z21" s="79" t="n">
         <f aca="false">Y21*E21</f>
         <v>54.299454</v>
       </c>
@@ -8415,7 +8802,7 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="36"/>
       <c r="B22" s="36" t="s">
-        <v>297</v>
+        <v>344</v>
       </c>
       <c r="C22" s="36"/>
       <c r="D22" s="36"/>
@@ -8433,7 +8820,7 @@
       <c r="P22" s="36"/>
       <c r="Q22" s="36"/>
       <c r="R22" s="36"/>
-      <c r="S22" s="80" t="n">
+      <c r="S22" s="81" t="n">
         <f aca="false">SUM(S4:S21)</f>
         <v>62800000</v>
       </c>
@@ -8443,7 +8830,7 @@
       <c r="W22" s="36"/>
       <c r="X22" s="36"/>
       <c r="Y22" s="36"/>
-      <c r="Z22" s="81" t="n">
+      <c r="Z22" s="82" t="n">
         <f aca="false">SUM(Z4:Z21)</f>
         <v>2495.4976035</v>
       </c>
@@ -8483,7 +8870,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>298</v>
+        <v>345</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8494,7 +8881,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>299</v>
+        <v>346</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -8505,199 +8892,199 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>232</v>
+        <v>279</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>300</v>
+        <v>347</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>254</v>
-      </c>
       <c r="F3" s="3" t="s">
-        <v>302</v>
+        <v>349</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>303</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="82" t="n">
+      <c r="A4" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="83" t="s">
-        <v>304</v>
-      </c>
-      <c r="C4" s="83" t="s">
+      <c r="B4" s="84" t="s">
+        <v>351</v>
+      </c>
+      <c r="C4" s="84" t="s">
         <v>68</v>
       </c>
-      <c r="D4" s="84" t="n">
+      <c r="D4" s="85" t="n">
         <f aca="false">Assumptions!$B$44</f>
         <v>4</v>
       </c>
-      <c r="E4" s="85" t="n">
+      <c r="E4" s="86" t="n">
         <v>220</v>
       </c>
-      <c r="F4" s="86" t="n">
+      <c r="F4" s="87" t="n">
         <f aca="false">E4*Assumptions!$B$41</f>
         <v>6.6</v>
       </c>
-      <c r="G4" s="86" t="n">
+      <c r="G4" s="87" t="n">
         <f aca="false">(E4+F4)*D4</f>
         <v>906.4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="82" t="n">
+      <c r="A5" s="83" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="83" t="s">
-        <v>305</v>
-      </c>
-      <c r="C5" s="83" t="s">
+      <c r="B5" s="84" t="s">
+        <v>352</v>
+      </c>
+      <c r="C5" s="84" t="s">
         <v>68</v>
       </c>
-      <c r="D5" s="82" t="n">
+      <c r="D5" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="85" t="n">
+      <c r="E5" s="86" t="n">
         <v>3200</v>
       </c>
-      <c r="F5" s="86" t="n">
+      <c r="F5" s="87" t="n">
         <f aca="false">E5*Assumptions!$B$41</f>
         <v>96</v>
       </c>
-      <c r="G5" s="86" t="n">
+      <c r="G5" s="87" t="n">
         <f aca="false">(E5+F5)*D5</f>
         <v>3296</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="82" t="n">
+      <c r="A6" s="83" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="83" t="s">
-        <v>306</v>
-      </c>
-      <c r="C6" s="83" t="s">
+      <c r="B6" s="84" t="s">
+        <v>353</v>
+      </c>
+      <c r="C6" s="84" t="s">
         <v>68</v>
       </c>
-      <c r="D6" s="82" t="n">
+      <c r="D6" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="85" t="n">
+      <c r="E6" s="86" t="n">
         <v>1500</v>
       </c>
-      <c r="F6" s="86" t="n">
+      <c r="F6" s="87" t="n">
         <f aca="false">E6*Assumptions!$B$41</f>
         <v>45</v>
       </c>
-      <c r="G6" s="86" t="n">
+      <c r="G6" s="87" t="n">
         <f aca="false">(E6+F6)*D6</f>
         <v>1545</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="82" t="n">
+      <c r="A7" s="83" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="83" t="s">
-        <v>307</v>
-      </c>
-      <c r="C7" s="83" t="s">
-        <v>308</v>
-      </c>
-      <c r="D7" s="82" t="n">
+      <c r="B7" s="84" t="s">
+        <v>354</v>
+      </c>
+      <c r="C7" s="84" t="s">
+        <v>355</v>
+      </c>
+      <c r="D7" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="85" t="n">
+      <c r="E7" s="86" t="n">
         <v>420</v>
       </c>
-      <c r="F7" s="86" t="n">
+      <c r="F7" s="87" t="n">
         <f aca="false">E7*Assumptions!$B$41</f>
         <v>12.6</v>
       </c>
-      <c r="G7" s="86" t="n">
+      <c r="G7" s="87" t="n">
         <f aca="false">(E7+F7)*D7</f>
         <v>432.6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="82" t="n">
+      <c r="A8" s="83" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="83" t="s">
-        <v>309</v>
-      </c>
-      <c r="C8" s="83" t="s">
-        <v>310</v>
-      </c>
-      <c r="D8" s="82" t="n">
+      <c r="B8" s="84" t="s">
+        <v>356</v>
+      </c>
+      <c r="C8" s="84" t="s">
+        <v>357</v>
+      </c>
+      <c r="D8" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="85" t="n">
+      <c r="E8" s="86" t="n">
         <v>95</v>
       </c>
-      <c r="F8" s="86" t="n">
+      <c r="F8" s="87" t="n">
         <f aca="false">E8*Assumptions!$B$41</f>
         <v>2.85</v>
       </c>
-      <c r="G8" s="86" t="n">
+      <c r="G8" s="87" t="n">
         <f aca="false">(E8+F8)*D8</f>
         <v>97.85</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="82" t="n">
+      <c r="A9" s="83" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="83" t="s">
-        <v>311</v>
-      </c>
-      <c r="C9" s="83" t="s">
-        <v>310</v>
-      </c>
-      <c r="D9" s="82" t="n">
+      <c r="B9" s="84" t="s">
+        <v>358</v>
+      </c>
+      <c r="C9" s="84" t="s">
+        <v>357</v>
+      </c>
+      <c r="D9" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="85" t="n">
+      <c r="E9" s="86" t="n">
         <v>28</v>
       </c>
-      <c r="F9" s="86" t="n">
+      <c r="F9" s="87" t="n">
         <f aca="false">E9*Assumptions!$B$41</f>
         <v>0.84</v>
       </c>
-      <c r="G9" s="86" t="n">
+      <c r="G9" s="87" t="n">
         <f aca="false">(E9+F9)*D9</f>
         <v>28.84</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="82" t="n">
+      <c r="A10" s="83" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="83" t="s">
-        <v>312</v>
-      </c>
-      <c r="C10" s="83" t="s">
-        <v>310</v>
-      </c>
-      <c r="D10" s="82" t="n">
+      <c r="B10" s="84" t="s">
+        <v>359</v>
+      </c>
+      <c r="C10" s="84" t="s">
+        <v>357</v>
+      </c>
+      <c r="D10" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="85" t="n">
+      <c r="E10" s="86" t="n">
         <v>20</v>
       </c>
-      <c r="F10" s="86" t="n">
+      <c r="F10" s="87" t="n">
         <f aca="false">E10*Assumptions!$B$41</f>
         <v>0.6</v>
       </c>
-      <c r="G10" s="86" t="n">
+      <c r="G10" s="87" t="n">
         <f aca="false">(E10+F10)*D10</f>
         <v>20.6</v>
       </c>
@@ -8705,20 +9092,20 @@
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="36"/>
       <c r="B11" s="36" t="s">
-        <v>313</v>
+        <v>360</v>
       </c>
       <c r="C11" s="36"/>
       <c r="D11" s="36"/>
       <c r="E11" s="36"/>
       <c r="F11" s="36"/>
-      <c r="G11" s="81" t="n">
+      <c r="G11" s="82" t="n">
         <f aca="false">SUM(G4:G10)</f>
         <v>6327.29</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="87" t="s">
-        <v>314</v>
+      <c r="B12" s="88" t="s">
+        <v>361</v>
       </c>
       <c r="G12" s="18" t="n">
         <f aca="false">SUM(G4:G7)</f>
@@ -8758,7 +9145,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>315</v>
+        <v>362</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8769,7 +9156,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>316</v>
+        <v>363</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -8780,268 +9167,268 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>317</v>
+        <v>364</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>318</v>
+        <v>365</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>319</v>
+        <v>366</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>320</v>
+        <v>367</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>246</v>
+        <v>293</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>321</v>
+        <v>368</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>322</v>
+        <v>369</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="82" t="n">
+      <c r="A4" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="88" t="s">
-        <v>323</v>
-      </c>
-      <c r="C4" s="89" t="n">
+      <c r="B4" s="89" t="s">
+        <v>370</v>
+      </c>
+      <c r="C4" s="90" t="n">
         <v>60</v>
       </c>
-      <c r="D4" s="90" t="n">
+      <c r="D4" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="91" t="n">
+      <c r="E4" s="92" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="F4" s="86" t="n">
+      <c r="F4" s="87" t="n">
         <f aca="false">C4*D4*E4/3600</f>
         <v>3.16666666666667</v>
       </c>
-      <c r="G4" s="88" t="s">
-        <v>324</v>
+      <c r="G4" s="89" t="s">
+        <v>371</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="82" t="n">
+      <c r="A5" s="83" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="88" t="s">
-        <v>325</v>
-      </c>
-      <c r="C5" s="89" t="n">
+      <c r="B5" s="89" t="s">
+        <v>372</v>
+      </c>
+      <c r="C5" s="90" t="n">
         <v>120</v>
       </c>
-      <c r="D5" s="90" t="n">
+      <c r="D5" s="91" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="91" t="n">
+      <c r="E5" s="92" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="F5" s="86" t="n">
+      <c r="F5" s="87" t="n">
         <f aca="false">C5*D5*E5/3600</f>
         <v>12.6666666666667</v>
       </c>
-      <c r="G5" s="88" t="s">
-        <v>326</v>
+      <c r="G5" s="89" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="82" t="n">
+      <c r="A6" s="83" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="88" t="s">
-        <v>327</v>
-      </c>
-      <c r="C6" s="89" t="n">
+      <c r="B6" s="89" t="s">
+        <v>374</v>
+      </c>
+      <c r="C6" s="90" t="n">
         <v>150</v>
       </c>
-      <c r="D6" s="90" t="n">
+      <c r="D6" s="91" t="n">
         <v>1.5</v>
       </c>
-      <c r="E6" s="91" t="n">
+      <c r="E6" s="92" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="F6" s="86" t="n">
+      <c r="F6" s="87" t="n">
         <f aca="false">C6*D6*E6/3600</f>
         <v>11.875</v>
       </c>
-      <c r="G6" s="88" t="s">
-        <v>328</v>
+      <c r="G6" s="89" t="s">
+        <v>375</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="82" t="n">
+      <c r="A7" s="83" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="88" t="s">
-        <v>329</v>
-      </c>
-      <c r="C7" s="89" t="n">
+      <c r="B7" s="89" t="s">
+        <v>376</v>
+      </c>
+      <c r="C7" s="90" t="n">
         <v>75</v>
       </c>
-      <c r="D7" s="90" t="n">
+      <c r="D7" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="91" t="n">
+      <c r="E7" s="92" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="F7" s="86" t="n">
+      <c r="F7" s="87" t="n">
         <f aca="false">C7*D7*E7/3600</f>
         <v>3.95833333333333</v>
       </c>
-      <c r="G7" s="88"/>
+      <c r="G7" s="89"/>
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="82" t="n">
+      <c r="A8" s="83" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="88" t="s">
-        <v>330</v>
-      </c>
-      <c r="C8" s="89" t="n">
+      <c r="B8" s="89" t="s">
+        <v>377</v>
+      </c>
+      <c r="C8" s="90" t="n">
         <v>60</v>
       </c>
-      <c r="D8" s="90" t="n">
+      <c r="D8" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="91" t="n">
+      <c r="E8" s="92" t="n">
         <f aca="false">Assumptions!$B$35</f>
         <v>230</v>
       </c>
-      <c r="F8" s="86" t="n">
+      <c r="F8" s="87" t="n">
         <f aca="false">C8*D8*E8/3600</f>
         <v>3.83333333333333</v>
       </c>
-      <c r="G8" s="88" t="s">
-        <v>331</v>
+      <c r="G8" s="89" t="s">
+        <v>378</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="82" t="n">
+      <c r="A9" s="83" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="88" t="s">
-        <v>332</v>
-      </c>
-      <c r="C9" s="89" t="n">
+      <c r="B9" s="89" t="s">
+        <v>379</v>
+      </c>
+      <c r="C9" s="90" t="n">
         <v>45</v>
       </c>
-      <c r="D9" s="90" t="n">
+      <c r="D9" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="91" t="n">
+      <c r="E9" s="92" t="n">
         <f aca="false">Assumptions!$B$33</f>
         <v>190</v>
       </c>
-      <c r="F9" s="86" t="n">
+      <c r="F9" s="87" t="n">
         <f aca="false">C9*D9*E9/3600</f>
         <v>2.375</v>
       </c>
-      <c r="G9" s="88"/>
+      <c r="G9" s="89"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="92" t="s">
-        <v>333</v>
+      <c r="B11" s="93" t="s">
+        <v>380</v>
       </c>
       <c r="C11" s="31"/>
       <c r="D11" s="31"/>
       <c r="E11" s="31"/>
-      <c r="F11" s="93" t="n">
+      <c r="F11" s="94" t="n">
         <f aca="false">SUM(F4:F9)</f>
         <v>37.875</v>
       </c>
-      <c r="G11" s="94"/>
+      <c r="G11" s="95"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="92" t="s">
-        <v>334</v>
+      <c r="B12" s="93" t="s">
+        <v>381</v>
       </c>
       <c r="C12" s="31"/>
       <c r="D12" s="31"/>
       <c r="E12" s="31"/>
-      <c r="F12" s="93" t="n">
+      <c r="F12" s="94" t="n">
         <f aca="false">4000000/(Assumptions!$B$4*Assumptions!$B$5)</f>
         <v>11.1111111111111</v>
       </c>
-      <c r="G12" s="94" t="s">
-        <v>335</v>
+      <c r="G12" s="95" t="s">
+        <v>382</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="92" t="s">
-        <v>336</v>
+      <c r="B13" s="93" t="s">
+        <v>383</v>
       </c>
       <c r="C13" s="31"/>
       <c r="D13" s="31"/>
       <c r="E13" s="31"/>
-      <c r="F13" s="93" t="n">
+      <c r="F13" s="94" t="n">
         <f aca="false">6000000/(Assumptions!$B$4*Assumptions!$B$5)</f>
         <v>16.6666666666667</v>
       </c>
-      <c r="G13" s="94"/>
+      <c r="G13" s="95"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="92" t="s">
-        <v>337</v>
+      <c r="B14" s="93" t="s">
+        <v>384</v>
       </c>
       <c r="C14" s="31"/>
       <c r="D14" s="31"/>
       <c r="E14" s="31"/>
-      <c r="F14" s="95" t="n">
+      <c r="F14" s="96" t="n">
         <v>6</v>
       </c>
-      <c r="G14" s="94" t="s">
-        <v>338</v>
+      <c r="G14" s="95" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="92" t="s">
-        <v>339</v>
+      <c r="B15" s="93" t="s">
+        <v>386</v>
       </c>
       <c r="C15" s="31"/>
       <c r="D15" s="31"/>
       <c r="E15" s="31"/>
-      <c r="F15" s="93" t="n">
+      <c r="F15" s="94" t="n">
         <f aca="false">F11*Assumptions!$B$42</f>
         <v>17.04375</v>
       </c>
-      <c r="G15" s="94" t="s">
-        <v>340</v>
+      <c r="G15" s="95" t="s">
+        <v>387</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="92" t="s">
-        <v>341</v>
+      <c r="B16" s="93" t="s">
+        <v>388</v>
       </c>
       <c r="C16" s="31"/>
       <c r="D16" s="31"/>
       <c r="E16" s="31"/>
-      <c r="F16" s="93" t="n">
+      <c r="F16" s="94" t="n">
         <f aca="false">Assumptions!$B$43</f>
         <v>55</v>
       </c>
-      <c r="G16" s="94"/>
+      <c r="G16" s="95"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="96" t="s">
-        <v>342</v>
-      </c>
-      <c r="C17" s="96"/>
-      <c r="D17" s="96"/>
-      <c r="E17" s="96"/>
-      <c r="F17" s="97" t="n">
+      <c r="B17" s="97" t="s">
+        <v>389</v>
+      </c>
+      <c r="C17" s="97"/>
+      <c r="D17" s="97"/>
+      <c r="E17" s="97"/>
+      <c r="F17" s="98" t="n">
         <f aca="false">SUM(F11:F16)</f>
         <v>143.696527777778</v>
       </c>
-      <c r="G17" s="96"/>
+      <c r="G17" s="97"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -9072,7 +9459,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>343</v>
+        <v>390</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9080,7 +9467,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>344</v>
+        <v>391</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -9088,51 +9475,51 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>300</v>
+        <v>347</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>345</v>
+        <v>392</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>346</v>
-      </c>
-      <c r="B4" s="98" t="n">
+        <v>393</v>
+      </c>
+      <c r="B4" s="99" t="n">
         <f aca="false">'Parts Costing'!S22</f>
         <v>62800000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>347</v>
-      </c>
-      <c r="B5" s="98" t="n">
+        <v>394</v>
+      </c>
+      <c r="B5" s="99" t="n">
         <v>4000000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="31" t="s">
-        <v>348</v>
-      </c>
-      <c r="B6" s="98" t="n">
+        <v>395</v>
+      </c>
+      <c r="B6" s="99" t="n">
         <v>6000000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="99" t="s">
-        <v>349</v>
-      </c>
-      <c r="B7" s="100" t="n">
+      <c r="A7" s="100" t="s">
+        <v>396</v>
+      </c>
+      <c r="B7" s="101" t="n">
         <f aca="false">SUM(B4:B6)</f>
         <v>72800000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="101" t="s">
-        <v>350</v>
-      </c>
-      <c r="B9" s="102" t="n">
+      <c r="A9" s="102" t="s">
+        <v>397</v>
+      </c>
+      <c r="B9" s="103" t="n">
         <f aca="false">B7/10000000</f>
         <v>7.28</v>
       </c>

</xml_diff>